<commit_message>
Add live Google Flights availability snapshot (2026-10-09)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MqDR8ErShU29xSVraYyKeW
</commit_message>
<xml_diff>
--- a/japan-ginzan-plan.xlsx
+++ b/japan-ginzan-plan.xlsx
@@ -9,12 +9,13 @@
   </bookViews>
   <sheets>
     <sheet name="總覽" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="每日行程" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="機票價格" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="方案比較" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="行程預算" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="待辦清單" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="資料來源" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="即時查價 10-9" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="每日行程" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="機票價格" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="方案比較" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="行程預算" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="待辦清單" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="資料來源" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="428">
   <si>
     <r>
       <rPr>
@@ -403,43 +404,463 @@
         <b val="true"/>
         <sz val="13"/>
         <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">定案行程：早去晚回 </t>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Google Flights </t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="13"/>
         <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6 </t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">即時查價（</t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="13"/>
         <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">天 </t>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026/10/9 </t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="13"/>
         <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5 </t>
-    </r>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">查詢，每人單程經濟艙，含稅，新台幣）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">有列出價格＝當下還有位子可以買。價格會變動，而且廉航不含托運行李。「商務艙」代表經濟艙已經查不到，只剩商務艙。</t>
+  </si>
+  <si>
+    <t xml:space="preserve">航線</t>
+  </si>
+  <si>
+    <t xml:space="preserve">航空</t>
+  </si>
+  <si>
+    <t xml:space="preserve">起飛 → 抵達</t>
+  </si>
+  <si>
+    <t xml:space="preserve">價格</t>
+  </si>
+  <si>
+    <t xml:space="preserve">艙等</t>
+  </si>
+  <si>
+    <t xml:space="preserve">狀態／備註</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/26 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">二</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">桃園→仙台</t>
+  </si>
+  <si>
+    <t xml:space="preserve">長榮航空</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10:15 → 14:25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">經濟</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">有位；比原本查到的 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">08:45 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">晚</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">星宇航空</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:50 → 16:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有位</t>
+  </si>
+  <si>
+    <t xml:space="preserve">台灣虎航</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14:35 → 18:45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有位；不含托運行李</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/27 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">三</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">有位，比 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/26 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">便宜很多</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/28 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">四</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">松山→羽田</t>
+  </si>
+  <si>
+    <t xml:space="preserve">日航／華航</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09:10 → 13:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有位，早班又便宜</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07:15 → 11:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有位，最早的一班</t>
+  </si>
+  <si>
+    <t xml:space="preserve">華航／日航</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09:00 → 12:50</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/31 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">仙台→桃園</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:15 → 19:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">商務</t>
+  </si>
+  <si>
+    <t xml:space="preserve">經濟艙查不到，只剩商務艙</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:25 → 20:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">沒有班次（或已售完）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">六</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">直飛</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">沒有直飛，只有轉機（約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NT$12,900 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">起，飛行 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">19 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">小時以上）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">一</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">經濟艙查不到</t>
+  </si>
+  <si>
+    <t xml:space="preserve">成田→桃園</t>
+  </si>
+  <si>
+    <t xml:space="preserve">泰國獅航</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:25 → 20:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有位；晚回又能搭捷運回家</t>
+  </si>
+  <si>
+    <t xml:space="preserve">酷航</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:45 → 22:55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:25 → 23:25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有位；落地太晚，可能趕不上末班捷運</t>
+  </si>
+  <si>
+    <t xml:space="preserve">樂桃航空</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:35 → 20:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15:40 → 18:45</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">有位；另有 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20:10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">的班次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">20:20 → 23:25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">羽田→松山</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07:55 → 10:55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有位，但太早</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:05 → 21:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有位，但很貴</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -448,7 +869,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">夜（</t>
+      <t xml:space="preserve">定案行程：早去晚回 </t>
     </r>
     <r>
       <rPr>
@@ -459,7 +880,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2027/1/26 </t>
+      <t xml:space="preserve">6 </t>
     </r>
     <r>
       <rPr>
@@ -469,7 +890,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">二 – </t>
+      <t xml:space="preserve">天 </t>
     </r>
     <r>
       <rPr>
@@ -480,7 +901,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1/31 </t>
+      <t xml:space="preserve">5 </t>
     </r>
     <r>
       <rPr>
@@ -490,7 +911,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">日，請假 </t>
+      <t xml:space="preserve">夜（</t>
     </r>
     <r>
       <rPr>
@@ -501,7 +922,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">4 </t>
+      <t xml:space="preserve">2027/1/26 </t>
     </r>
     <r>
       <rPr>
@@ -511,6 +932,48 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">二 – </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/31 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日，請假 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">天）</t>
     </r>
   </si>
@@ -2311,12 +2774,6 @@
     <t xml:space="preserve">編號</t>
   </si>
   <si>
-    <t xml:space="preserve">航線</t>
-  </si>
-  <si>
-    <t xml:space="preserve">航空</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -2392,9 +2849,6 @@
     <t xml:space="preserve">桃園⇄仙台</t>
   </si>
   <si>
-    <t xml:space="preserve">台灣虎航</t>
-  </si>
-  <si>
     <t xml:space="preserve">IT254 / IT255</t>
   </si>
   <si>
@@ -2538,9 +2992,6 @@
     <t xml:space="preserve">F2</t>
   </si>
   <si>
-    <t xml:space="preserve">長榮航空</t>
-  </si>
-  <si>
     <t xml:space="preserve">BR118 / BR117</t>
   </si>
   <si>
@@ -2626,9 +3077,6 @@
     <t xml:space="preserve">F3</t>
   </si>
   <si>
-    <t xml:space="preserve">星宇航空</t>
-  </si>
-  <si>
     <t xml:space="preserve">JX862 / JX863</t>
   </si>
   <si>
@@ -3163,9 +3611,6 @@
     <t xml:space="preserve">桃園⇄羽田</t>
   </si>
   <si>
-    <t xml:space="preserve">樂桃航空</t>
-  </si>
-  <si>
     <t xml:space="preserve">MM</t>
   </si>
   <si>
@@ -4136,27 +4581,6 @@
     <t xml:space="preserve">小計（新台幣）</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1/26 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">二</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">桃園 → 仙台；下午仙台城跡、瑞鳳殿，晚餐吃牛舌</t>
   </si>
   <si>
@@ -4281,27 +4705,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1/27 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">三</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">山寺（立石寺）→ 藏王溫泉，看樹冰夜景</t>
   </si>
   <si>
@@ -4388,27 +4791,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1/28 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">四</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">藏王樹冰（白天）→ 山形市區</t>
   </si>
   <si>
@@ -4573,27 +4955,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1/30 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">六</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">銀山溫泉清晨拍照 → 仙台</t>
   </si>
   <si>
@@ -4656,27 +5017,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1/31 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">日</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">松島（遊覽船、瑞巖寺、烤牡蠣）→ 仙台機場 → 桃園</t>
   </si>
   <si>
@@ -4728,9 +5068,6 @@
       </rPr>
       <t xml:space="preserve">¥680</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
   </si>
   <si>
     <r>
@@ -5780,16 +6117,16 @@
       <b val="true"/>
       <sz val="13"/>
       <color rgb="FF000000"/>
-      <name val="WenQuanYi Zen Hei"/>
-      <family val="2"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="13"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -5814,7 +6151,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5837,6 +6174,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFE3F3E7"/>
         <bgColor rgb="FFE1EEFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDEAE3"/>
+        <bgColor rgb="FFE3F3E7"/>
       </patternFill>
     </fill>
     <fill>
@@ -5895,7 +6238,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="51">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -5976,7 +6319,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5988,15 +6335,27 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6113,7 +6472,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFFDEAE3"/>
       <rgbColor rgb="FFE1EEFB"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -6722,14 +7081,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6758,582 +7119,536 @@
       <c r="E4" s="8" t="s">
         <v>32</v>
       </c>
+      <c r="F4" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="B5" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="22" t="s">
+      <c r="C5" s="16" t="s">
         <v>37</v>
       </c>
+      <c r="D5" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>25165</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16"/>
-      <c r="B6" s="23" t="s">
+      <c r="A6" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>22778</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>15599</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>15727</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="E9" s="21" t="n">
+        <v>17775</v>
+      </c>
+      <c r="F9" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="E6" s="16" t="s">
+      <c r="G9" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>14099</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="16" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16"/>
-      <c r="B7" s="23" t="s">
+      <c r="D11" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="E11" s="21" t="n">
+        <v>22778</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G11" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>14137</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G12" s="16" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>17309</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="16" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="21" t="n">
+        <v>17246</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E15" s="24" t="n">
+        <v>33008</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G15" s="23" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" s="24" t="n">
+        <v>34279</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G16" s="23" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="23" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16"/>
-      <c r="B8" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16"/>
-      <c r="B9" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16"/>
-      <c r="B10" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16"/>
-      <c r="B11" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16" t="s">
+      <c r="D17" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" s="24"/>
+      <c r="F17" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="G17" s="23" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="D18" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" s="24"/>
+      <c r="F18" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="G18" s="23" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="E19" s="24" t="n">
+        <v>34279</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G19" s="23" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="20" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="C12" s="22" t="s">
-        <v>61</v>
-      </c>
-      <c r="D12" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="E12" s="22" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16"/>
-      <c r="B13" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16"/>
-      <c r="B14" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16"/>
-      <c r="B15" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="C15" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="D15" s="23" t="s">
+      <c r="B20" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="E15" s="16"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="16"/>
-      <c r="B16" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="C16" s="16" t="s">
+      <c r="C20" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="D20" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="E16" s="16" t="s">
+      <c r="E20" s="21" t="n">
+        <v>14542</v>
+      </c>
+      <c r="F20" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G20" s="16" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="16"/>
-      <c r="B17" s="23" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C21" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="D21" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16" t="s">
+      <c r="E21" s="21" t="n">
+        <v>13212</v>
+      </c>
+      <c r="F21" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G21" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" s="20" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="16"/>
-      <c r="B18" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="C18" s="16" t="s">
+      <c r="E22" s="21" t="n">
+        <v>13149</v>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G22" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="D18" s="16" t="s">
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="E18" s="16" t="s">
+      <c r="D23" s="20" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="B19" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="C19" s="22" t="s">
-        <v>82</v>
-      </c>
-      <c r="D19" s="22" t="s">
-        <v>83</v>
-      </c>
-      <c r="E19" s="22" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="16"/>
-      <c r="B20" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="16"/>
-      <c r="B21" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="D21" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="E21" s="16"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="16"/>
-      <c r="B22" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="16"/>
-      <c r="B23" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="C23" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16" t="s">
-        <v>92</v>
+      <c r="E23" s="21" t="n">
+        <v>18549</v>
+      </c>
+      <c r="F23" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G23" s="16" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>93</v>
-      </c>
-      <c r="B24" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="C24" s="22" t="s">
-        <v>95</v>
-      </c>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="16"/>
-      <c r="B25" s="23" t="s">
-        <v>97</v>
+        <v>58</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="E24" s="21" t="n">
+        <v>21166</v>
+      </c>
+      <c r="F24" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G24" s="16" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>71</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="D25" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="E25" s="16"/>
+        <v>37</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="E25" s="21" t="n">
+        <v>27583</v>
+      </c>
+      <c r="F25" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G25" s="16" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="16"/>
-      <c r="B26" s="23" t="s">
+      <c r="A26" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="E26" s="21" t="n">
+        <v>15742</v>
+      </c>
+      <c r="F26" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G26" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="C26" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="D26" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="E26" s="16" t="s">
-        <v>102</v>
-      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12"/>
-      <c r="B27" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="16"/>
-      <c r="B28" s="23" t="s">
-        <v>105</v>
-      </c>
-      <c r="C28" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="16"/>
-      <c r="B29" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="C29" s="16" t="s">
-        <v>109</v>
-      </c>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="16"/>
-      <c r="B30" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="C30" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="B31" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="C31" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="16"/>
-      <c r="B32" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="C32" s="16" t="s">
-        <v>118</v>
-      </c>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="16"/>
-      <c r="B33" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="C33" s="16" t="s">
-        <v>120</v>
-      </c>
-      <c r="D33" s="16" t="s">
-        <v>121</v>
-      </c>
-      <c r="E33" s="16"/>
-    </row>
-    <row r="34" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="16"/>
-      <c r="B34" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="C34" s="16" t="s">
-        <v>123</v>
-      </c>
-      <c r="D34" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="E34" s="16" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="16"/>
-      <c r="B35" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="C35" s="16" t="s">
-        <v>126</v>
-      </c>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="16"/>
-      <c r="B36" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="C36" s="16" t="s">
-        <v>127</v>
-      </c>
-      <c r="D36" s="16"/>
-      <c r="E36" s="16" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="16"/>
-      <c r="B37" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="C37" s="16" t="s">
-        <v>129</v>
-      </c>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="20" t="s">
-        <v>131</v>
-      </c>
-      <c r="B38" s="21" t="s">
-        <v>117</v>
-      </c>
-      <c r="C38" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="D38" s="22"/>
-      <c r="E38" s="22"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="16"/>
-      <c r="B39" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="C39" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="D39" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="E39" s="16"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="16"/>
-      <c r="B40" s="23" t="s">
-        <v>135</v>
-      </c>
-      <c r="C40" s="16" t="s">
-        <v>136</v>
-      </c>
-      <c r="D40" s="16" t="s">
-        <v>137</v>
-      </c>
-      <c r="E40" s="16"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="16"/>
-      <c r="B41" s="23" t="s">
-        <v>138</v>
-      </c>
-      <c r="C41" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="D41" s="16" t="s">
-        <v>140</v>
-      </c>
-      <c r="E41" s="16"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="16"/>
-      <c r="B42" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="C42" s="16" t="s">
-        <v>141</v>
-      </c>
-      <c r="D42" s="16"/>
-      <c r="E42" s="16" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="16"/>
-      <c r="B43" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="C43" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="D43" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="E43" s="16"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="16"/>
-      <c r="B44" s="23" t="s">
-        <v>144</v>
-      </c>
-      <c r="C44" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="D44" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="E44" s="16" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="16"/>
-      <c r="B45" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="C45" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="D45" s="16"/>
-      <c r="E45" s="16" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="16"/>
-      <c r="B46" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>151</v>
-      </c>
-      <c r="D46" s="16" t="s">
-        <v>152</v>
-      </c>
-      <c r="E46" s="16" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="2" t="s">
-        <v>154</v>
+      <c r="A27" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B27" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="E27" s="21" t="n">
+        <v>37120</v>
+      </c>
+      <c r="F27" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G27" s="16" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -7348,6 +7663,636 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E48"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="26" t="s">
+        <v>95</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="C5" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="D5" s="28" t="s">
+        <v>98</v>
+      </c>
+      <c r="E5" s="28" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16"/>
+      <c r="B6" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16"/>
+      <c r="B7" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16"/>
+      <c r="B8" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16"/>
+      <c r="B9" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="16"/>
+      <c r="B10" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="16"/>
+      <c r="B11" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="B12" s="27" t="s">
+        <v>122</v>
+      </c>
+      <c r="C12" s="28" t="s">
+        <v>123</v>
+      </c>
+      <c r="D12" s="27" t="s">
+        <v>124</v>
+      </c>
+      <c r="E12" s="28" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="16"/>
+      <c r="B13" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="16"/>
+      <c r="B14" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16"/>
+      <c r="B15" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="E15" s="16"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16"/>
+      <c r="B16" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16"/>
+      <c r="B17" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="16"/>
+      <c r="B18" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="D18" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="E18" s="16" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="26" t="s">
+        <v>143</v>
+      </c>
+      <c r="B19" s="27" t="s">
+        <v>122</v>
+      </c>
+      <c r="C19" s="28" t="s">
+        <v>144</v>
+      </c>
+      <c r="D19" s="28" t="s">
+        <v>145</v>
+      </c>
+      <c r="E19" s="28" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="16"/>
+      <c r="B20" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="16"/>
+      <c r="B21" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="D21" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="E21" s="16"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="16"/>
+      <c r="B22" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="D22" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="E22" s="16" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="16"/>
+      <c r="B23" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="B24" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="C24" s="28" t="s">
+        <v>157</v>
+      </c>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="16"/>
+      <c r="B25" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>160</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="E25" s="16"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="16"/>
+      <c r="B26" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>162</v>
+      </c>
+      <c r="D26" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="E26" s="16" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="12"/>
+      <c r="B27" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="16"/>
+      <c r="B28" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="16"/>
+      <c r="B29" s="20" t="s">
+        <v>170</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>171</v>
+      </c>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="16"/>
+      <c r="B30" s="20" t="s">
+        <v>172</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>173</v>
+      </c>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="26" t="s">
+        <v>175</v>
+      </c>
+      <c r="B31" s="27" t="s">
+        <v>176</v>
+      </c>
+      <c r="C31" s="28" t="s">
+        <v>177</v>
+      </c>
+      <c r="D31" s="28"/>
+      <c r="E31" s="28" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="16"/>
+      <c r="B32" s="20" t="s">
+        <v>179</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>180</v>
+      </c>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="16"/>
+      <c r="B33" s="20" t="s">
+        <v>181</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>182</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="E33" s="16"/>
+    </row>
+    <row r="34" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="16"/>
+      <c r="B34" s="20" t="s">
+        <v>184</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="D34" s="20" t="s">
+        <v>186</v>
+      </c>
+      <c r="E34" s="16" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="16"/>
+      <c r="B35" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="16"/>
+      <c r="B36" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="16"/>
+      <c r="B37" s="20" t="s">
+        <v>170</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="26" t="s">
+        <v>193</v>
+      </c>
+      <c r="B38" s="27" t="s">
+        <v>179</v>
+      </c>
+      <c r="C38" s="28" t="s">
+        <v>194</v>
+      </c>
+      <c r="D38" s="28"/>
+      <c r="E38" s="28"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="16"/>
+      <c r="B39" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="D39" s="20" t="s">
+        <v>196</v>
+      </c>
+      <c r="E39" s="16"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="16"/>
+      <c r="B40" s="20" t="s">
+        <v>197</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>198</v>
+      </c>
+      <c r="D40" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="E40" s="16"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="16"/>
+      <c r="B41" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="D41" s="16" t="s">
+        <v>202</v>
+      </c>
+      <c r="E41" s="16"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="16"/>
+      <c r="B42" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="C42" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="D42" s="16"/>
+      <c r="E42" s="16" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="16"/>
+      <c r="B43" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="C43" s="16" t="s">
+        <v>205</v>
+      </c>
+      <c r="D43" s="20" t="s">
+        <v>196</v>
+      </c>
+      <c r="E43" s="16"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="16"/>
+      <c r="B44" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="C44" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="D44" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="E44" s="16" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="16"/>
+      <c r="B45" s="20" t="s">
+        <v>209</v>
+      </c>
+      <c r="C45" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="D45" s="16"/>
+      <c r="E45" s="16" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="16"/>
+      <c r="B46" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="C46" s="16" t="s">
+        <v>213</v>
+      </c>
+      <c r="D46" s="16" t="s">
+        <v>214</v>
+      </c>
+      <c r="E46" s="16" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -7370,551 +8315,551 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
-        <v>155</v>
+      <c r="A1" s="25" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>156</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>157</v>
+        <v>219</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>158</v>
+        <v>29</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>159</v>
+        <v>30</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>160</v>
+        <v>220</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>161</v>
+        <v>221</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>162</v>
+        <v>222</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>163</v>
+        <v>223</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>164</v>
+        <v>224</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>165</v>
+        <v>225</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>166</v>
+        <v>226</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>167</v>
+        <v>227</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>168</v>
+        <v>228</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>169</v>
+        <v>229</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>170</v>
+        <v>230</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>171</v>
+        <v>231</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>172</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
-        <v>173</v>
+      <c r="A5" s="20" t="s">
+        <v>233</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>174</v>
+        <v>234</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>175</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>177</v>
-      </c>
-      <c r="F5" s="23" t="s">
-        <v>178</v>
+        <v>44</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="E5" s="20" t="s">
+        <v>236</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>237</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>179</v>
-      </c>
-      <c r="H5" s="25" t="n">
+        <v>238</v>
+      </c>
+      <c r="H5" s="21" t="n">
         <v>4743</v>
       </c>
-      <c r="I5" s="25" t="n">
+      <c r="I5" s="21" t="n">
         <v>9676</v>
       </c>
-      <c r="J5" s="26"/>
-      <c r="K5" s="26"/>
-      <c r="L5" s="27" t="n">
+      <c r="J5" s="30"/>
+      <c r="K5" s="30"/>
+      <c r="L5" s="31" t="n">
         <f aca="false">IF(J5&gt;0,J5,H5)</f>
         <v>4743</v>
       </c>
-      <c r="M5" s="27" t="n">
+      <c r="M5" s="31" t="n">
         <f aca="false">IF(K5&gt;0,K5,I5)</f>
         <v>9676</v>
       </c>
       <c r="N5" s="16" t="s">
-        <v>180</v>
-      </c>
-      <c r="O5" s="25" t="n">
+        <v>239</v>
+      </c>
+      <c r="O5" s="21" t="n">
         <v>950</v>
       </c>
       <c r="P5" s="16" t="s">
-        <v>181</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
-        <v>182</v>
+      <c r="A6" s="20" t="s">
+        <v>241</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>174</v>
+        <v>234</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>183</v>
-      </c>
-      <c r="D6" s="23" t="s">
-        <v>184</v>
-      </c>
-      <c r="E6" s="23" t="s">
-        <v>185</v>
-      </c>
-      <c r="F6" s="23" t="s">
-        <v>186</v>
+        <v>37</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>243</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>244</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>187</v>
-      </c>
-      <c r="H6" s="25" t="n">
+        <v>245</v>
+      </c>
+      <c r="H6" s="21" t="n">
         <v>9845</v>
       </c>
-      <c r="I6" s="25" t="n">
+      <c r="I6" s="21" t="n">
         <v>17878</v>
       </c>
-      <c r="J6" s="26"/>
-      <c r="K6" s="26"/>
-      <c r="L6" s="27" t="n">
+      <c r="J6" s="30"/>
+      <c r="K6" s="30"/>
+      <c r="L6" s="31" t="n">
         <f aca="false">IF(J6&gt;0,J6,H6)</f>
         <v>9845</v>
       </c>
-      <c r="M6" s="27" t="n">
+      <c r="M6" s="31" t="n">
         <f aca="false">IF(K6&gt;0,K6,I6)</f>
         <v>17878</v>
       </c>
       <c r="N6" s="16" t="s">
-        <v>188</v>
-      </c>
-      <c r="O6" s="25" t="n">
+        <v>246</v>
+      </c>
+      <c r="O6" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P6" s="16" t="s">
-        <v>189</v>
+        <v>247</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="s">
-        <v>190</v>
+      <c r="A7" s="20" t="s">
+        <v>248</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>174</v>
+        <v>234</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>192</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>193</v>
-      </c>
-      <c r="F7" s="23" t="s">
-        <v>194</v>
+        <v>41</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>249</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>250</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>251</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="H7" s="25" t="n">
+        <v>252</v>
+      </c>
+      <c r="H7" s="21" t="n">
         <v>9720</v>
       </c>
-      <c r="I7" s="25" t="n">
+      <c r="I7" s="21" t="n">
         <v>19586</v>
       </c>
-      <c r="J7" s="26"/>
-      <c r="K7" s="26"/>
-      <c r="L7" s="27" t="n">
+      <c r="J7" s="30"/>
+      <c r="K7" s="30"/>
+      <c r="L7" s="31" t="n">
         <f aca="false">IF(J7&gt;0,J7,H7)</f>
         <v>9720</v>
       </c>
-      <c r="M7" s="27" t="n">
+      <c r="M7" s="31" t="n">
         <f aca="false">IF(K7&gt;0,K7,I7)</f>
         <v>19586</v>
       </c>
       <c r="N7" s="16" t="s">
-        <v>188</v>
-      </c>
-      <c r="O7" s="25" t="n">
+        <v>246</v>
+      </c>
+      <c r="O7" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P7" s="16" t="s">
-        <v>196</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23" t="s">
-        <v>197</v>
+      <c r="A8" s="20" t="s">
+        <v>254</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>198</v>
+        <v>255</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>183</v>
-      </c>
-      <c r="D8" s="23" t="s">
-        <v>199</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>200</v>
+        <v>37</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>256</v>
+      </c>
+      <c r="E8" s="20" t="s">
+        <v>257</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>201</v>
+        <v>258</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="H8" s="25" t="n">
+        <v>252</v>
+      </c>
+      <c r="H8" s="21" t="n">
         <v>10361</v>
       </c>
-      <c r="I8" s="25" t="n">
+      <c r="I8" s="21" t="n">
         <v>16526</v>
       </c>
-      <c r="J8" s="26"/>
-      <c r="K8" s="26"/>
-      <c r="L8" s="27" t="n">
+      <c r="J8" s="30"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="31" t="n">
         <f aca="false">IF(J8&gt;0,J8,H8)</f>
         <v>10361</v>
       </c>
-      <c r="M8" s="27" t="n">
+      <c r="M8" s="31" t="n">
         <f aca="false">IF(K8&gt;0,K8,I8)</f>
         <v>16526</v>
       </c>
       <c r="N8" s="16" t="s">
-        <v>188</v>
-      </c>
-      <c r="O8" s="25" t="n">
+        <v>246</v>
+      </c>
+      <c r="O8" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P8" s="16" t="s">
-        <v>202</v>
+        <v>259</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="s">
-        <v>203</v>
+      <c r="A9" s="20" t="s">
+        <v>260</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>198</v>
+        <v>255</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>204</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>205</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>206</v>
+        <v>261</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>263</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>201</v>
+        <v>258</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="H9" s="25" t="n">
+        <v>252</v>
+      </c>
+      <c r="H9" s="21" t="n">
         <v>10361</v>
       </c>
-      <c r="I9" s="25" t="n">
+      <c r="I9" s="21" t="n">
         <v>16526</v>
       </c>
-      <c r="J9" s="26"/>
-      <c r="K9" s="26"/>
-      <c r="L9" s="27" t="n">
+      <c r="J9" s="30"/>
+      <c r="K9" s="30"/>
+      <c r="L9" s="31" t="n">
         <f aca="false">IF(J9&gt;0,J9,H9)</f>
         <v>10361</v>
       </c>
-      <c r="M9" s="27" t="n">
+      <c r="M9" s="31" t="n">
         <f aca="false">IF(K9&gt;0,K9,I9)</f>
         <v>16526</v>
       </c>
       <c r="N9" s="16" t="s">
-        <v>188</v>
-      </c>
-      <c r="O9" s="25" t="n">
+        <v>246</v>
+      </c>
+      <c r="O9" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P9" s="16" t="s">
-        <v>207</v>
+        <v>264</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
-        <v>208</v>
+      <c r="A10" s="20" t="s">
+        <v>265</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>198</v>
+        <v>255</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>209</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>210</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>211</v>
+        <v>266</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>267</v>
+      </c>
+      <c r="E10" s="20" t="s">
+        <v>268</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>201</v>
+        <v>258</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="H10" s="25" t="n">
+        <v>252</v>
+      </c>
+      <c r="H10" s="21" t="n">
         <v>10361</v>
       </c>
-      <c r="I10" s="25" t="n">
+      <c r="I10" s="21" t="n">
         <v>16526</v>
       </c>
-      <c r="J10" s="26"/>
-      <c r="K10" s="26"/>
-      <c r="L10" s="27" t="n">
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="31" t="n">
         <f aca="false">IF(J10&gt;0,J10,H10)</f>
         <v>10361</v>
       </c>
-      <c r="M10" s="27" t="n">
+      <c r="M10" s="31" t="n">
         <f aca="false">IF(K10&gt;0,K10,I10)</f>
         <v>16526</v>
       </c>
       <c r="N10" s="16" t="s">
-        <v>188</v>
-      </c>
-      <c r="O10" s="25" t="n">
+        <v>246</v>
+      </c>
+      <c r="O10" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P10" s="16" t="s">
-        <v>207</v>
+        <v>264</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="s">
-        <v>212</v>
+      <c r="A11" s="20" t="s">
+        <v>269</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>198</v>
+        <v>255</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>213</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>214</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>215</v>
+        <v>270</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>271</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>272</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>201</v>
+        <v>258</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="H11" s="25" t="n">
+        <v>252</v>
+      </c>
+      <c r="H11" s="21" t="n">
         <v>10361</v>
       </c>
-      <c r="I11" s="25" t="n">
+      <c r="I11" s="21" t="n">
         <v>16526</v>
       </c>
-      <c r="J11" s="26"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="27" t="n">
+      <c r="J11" s="30"/>
+      <c r="K11" s="30"/>
+      <c r="L11" s="31" t="n">
         <f aca="false">IF(J11&gt;0,J11,H11)</f>
         <v>10361</v>
       </c>
-      <c r="M11" s="27" t="n">
+      <c r="M11" s="31" t="n">
         <f aca="false">IF(K11&gt;0,K11,I11)</f>
         <v>16526</v>
       </c>
       <c r="N11" s="16" t="s">
-        <v>188</v>
-      </c>
-      <c r="O11" s="25" t="n">
+        <v>246</v>
+      </c>
+      <c r="O11" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P11" s="16" t="s">
-        <v>207</v>
+        <v>264</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23" t="s">
-        <v>216</v>
+      <c r="A12" s="20" t="s">
+        <v>273</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>217</v>
+        <v>274</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>218</v>
-      </c>
-      <c r="D12" s="23" t="s">
-        <v>219</v>
+        <v>79</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>275</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>220</v>
+        <v>276</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>220</v>
+        <v>276</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="H12" s="25" t="n">
+        <v>252</v>
+      </c>
+      <c r="H12" s="21" t="n">
         <v>5386</v>
       </c>
-      <c r="I12" s="27" t="n">
+      <c r="I12" s="31" t="n">
         <f aca="false">H12*2</f>
         <v>10772</v>
       </c>
-      <c r="J12" s="26"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="27" t="n">
+      <c r="J12" s="30"/>
+      <c r="K12" s="30"/>
+      <c r="L12" s="31" t="n">
         <f aca="false">IF(J12&gt;0,J12,H12)</f>
         <v>5386</v>
       </c>
-      <c r="M12" s="27" t="n">
+      <c r="M12" s="31" t="n">
         <f aca="false">IF(K12&gt;0,K12,I12)</f>
         <v>10772</v>
       </c>
       <c r="N12" s="16" t="s">
-        <v>180</v>
-      </c>
-      <c r="O12" s="25" t="n">
+        <v>239</v>
+      </c>
+      <c r="O12" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="P12" s="16" t="s">
-        <v>221</v>
+        <v>277</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="23" t="s">
-        <v>222</v>
+      <c r="A13" s="20" t="s">
+        <v>278</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>223</v>
+        <v>279</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>224</v>
-      </c>
-      <c r="D13" s="23" t="s">
-        <v>225</v>
+        <v>280</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>281</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>220</v>
+        <v>276</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>220</v>
+        <v>276</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="H13" s="25" t="n">
+        <v>252</v>
+      </c>
+      <c r="H13" s="21" t="n">
         <v>3748</v>
       </c>
-      <c r="I13" s="27" t="n">
+      <c r="I13" s="31" t="n">
         <f aca="false">H13*2</f>
         <v>7496</v>
       </c>
-      <c r="J13" s="26"/>
-      <c r="K13" s="26"/>
-      <c r="L13" s="27" t="n">
+      <c r="J13" s="30"/>
+      <c r="K13" s="30"/>
+      <c r="L13" s="31" t="n">
         <f aca="false">IF(J13&gt;0,J13,H13)</f>
         <v>3748</v>
       </c>
-      <c r="M13" s="27" t="n">
+      <c r="M13" s="31" t="n">
         <f aca="false">IF(K13&gt;0,K13,I13)</f>
         <v>7496</v>
       </c>
       <c r="N13" s="16" t="s">
-        <v>180</v>
-      </c>
-      <c r="O13" s="25" t="n">
+        <v>239</v>
+      </c>
+      <c r="O13" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="P13" s="16" t="s">
-        <v>226</v>
+        <v>282</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="23" t="s">
-        <v>227</v>
+      <c r="A14" s="20" t="s">
+        <v>283</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>217</v>
+        <v>274</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>175</v>
-      </c>
-      <c r="D14" s="23" t="s">
-        <v>228</v>
+        <v>44</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>284</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>220</v>
+        <v>276</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>220</v>
+        <v>276</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="H14" s="25" t="n">
+        <v>252</v>
+      </c>
+      <c r="H14" s="21" t="n">
         <v>6702</v>
       </c>
-      <c r="I14" s="27" t="n">
+      <c r="I14" s="31" t="n">
         <f aca="false">H14*2</f>
         <v>13404</v>
       </c>
-      <c r="J14" s="26"/>
-      <c r="K14" s="26"/>
-      <c r="L14" s="27" t="n">
+      <c r="J14" s="30"/>
+      <c r="K14" s="30"/>
+      <c r="L14" s="31" t="n">
         <f aca="false">IF(J14&gt;0,J14,H14)</f>
         <v>6702</v>
       </c>
-      <c r="M14" s="27" t="n">
+      <c r="M14" s="31" t="n">
         <f aca="false">IF(K14&gt;0,K14,I14)</f>
         <v>13404</v>
       </c>
       <c r="N14" s="16" t="s">
-        <v>180</v>
-      </c>
-      <c r="O14" s="25" t="n">
+        <v>239</v>
+      </c>
+      <c r="O14" s="21" t="n">
         <v>950</v>
       </c>
       <c r="P14" s="16" t="s">
-        <v>229</v>
+        <v>285</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>230</v>
+        <v>286</v>
       </c>
     </row>
   </sheetData>
@@ -7928,7 +8873,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -7950,18 +8895,18 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
-        <v>231</v>
+      <c r="A1" s="25" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>232</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>233</v>
+        <v>289</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>10</v>
@@ -7973,51 +8918,51 @@
         <v>12</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>234</v>
+        <v>290</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>235</v>
+        <v>291</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>236</v>
+        <v>292</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>237</v>
+        <v>293</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>238</v>
+        <v>294</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>239</v>
+        <v>295</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>240</v>
+        <v>296</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>241</v>
+        <v>297</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>242</v>
+        <v>298</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
-        <v>243</v>
-      </c>
-      <c r="B5" s="28" t="s">
-        <v>244</v>
-      </c>
-      <c r="C5" s="24" t="s">
-        <v>245</v>
-      </c>
-      <c r="D5" s="29" t="n">
+      <c r="A5" s="29" t="s">
+        <v>299</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>300</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>301</v>
+      </c>
+      <c r="D5" s="33" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="24" t="s">
-        <v>246</v>
-      </c>
-      <c r="F5" s="24" t="s">
-        <v>247</v>
+      <c r="E5" s="29" t="s">
+        <v>302</v>
+      </c>
+      <c r="F5" s="29" t="s">
+        <v>303</v>
       </c>
       <c r="G5" s="11" t="n">
         <f aca="false">機票價格!L6+機票價格!L5</f>
@@ -8027,42 +8972,42 @@
         <f aca="false">機票價格!O5</f>
         <v>950</v>
       </c>
-      <c r="I5" s="30" t="n">
+      <c r="I5" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="31" t="n">
+      <c r="J5" s="35" t="n">
         <f aca="false">I5*總覽!$B$5</f>
         <v>0</v>
       </c>
-      <c r="K5" s="31" t="n">
+      <c r="K5" s="35" t="n">
         <f aca="false">G5+H5+J5</f>
         <v>15538</v>
       </c>
-      <c r="L5" s="24" t="s">
-        <v>248</v>
+      <c r="L5" s="29" t="s">
+        <v>304</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>249</v>
+        <v>305</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
-        <v>250</v>
+      <c r="A6" s="20" t="s">
+        <v>306</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>251</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>245</v>
-      </c>
-      <c r="D6" s="32" t="n">
+        <v>307</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>301</v>
+      </c>
+      <c r="D6" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="23" t="s">
-        <v>252</v>
-      </c>
-      <c r="F6" s="23" t="s">
-        <v>253</v>
+      <c r="E6" s="20" t="s">
+        <v>308</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>309</v>
       </c>
       <c r="G6" s="15" t="n">
         <f aca="false">機票價格!M5</f>
@@ -8072,42 +9017,42 @@
         <f aca="false">2*機票價格!O5</f>
         <v>1900</v>
       </c>
-      <c r="I6" s="33" t="n">
+      <c r="I6" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="27" t="n">
+      <c r="J6" s="31" t="n">
         <f aca="false">I6*總覽!$B$5</f>
         <v>0</v>
       </c>
-      <c r="K6" s="27" t="n">
+      <c r="K6" s="31" t="n">
         <f aca="false">G6+H6+J6</f>
         <v>11576</v>
       </c>
-      <c r="L6" s="23" t="s">
-        <v>248</v>
+      <c r="L6" s="20" t="s">
+        <v>304</v>
       </c>
       <c r="M6" s="16" t="s">
-        <v>254</v>
+        <v>310</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="s">
-        <v>255</v>
+      <c r="A7" s="20" t="s">
+        <v>311</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>256</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>257</v>
-      </c>
-      <c r="D7" s="32" t="n">
+        <v>312</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>313</v>
+      </c>
+      <c r="D7" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="23" t="s">
-        <v>258</v>
-      </c>
-      <c r="F7" s="23" t="s">
-        <v>253</v>
+      <c r="E7" s="20" t="s">
+        <v>314</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>309</v>
       </c>
       <c r="G7" s="15" t="n">
         <f aca="false">機票價格!L6+機票價格!L5</f>
@@ -8117,42 +9062,42 @@
         <f aca="false">機票價格!O5</f>
         <v>950</v>
       </c>
-      <c r="I7" s="33" t="n">
+      <c r="I7" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="27" t="n">
+      <c r="J7" s="31" t="n">
         <f aca="false">I7*總覽!$B$5</f>
         <v>0</v>
       </c>
-      <c r="K7" s="27" t="n">
+      <c r="K7" s="31" t="n">
         <f aca="false">G7+H7+J7</f>
         <v>15538</v>
       </c>
-      <c r="L7" s="23" t="s">
-        <v>248</v>
+      <c r="L7" s="20" t="s">
+        <v>304</v>
       </c>
       <c r="M7" s="16" t="s">
-        <v>259</v>
+        <v>315</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23" t="s">
-        <v>260</v>
+      <c r="A8" s="20" t="s">
+        <v>316</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>261</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>257</v>
-      </c>
-      <c r="D8" s="32" t="n">
+        <v>317</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>313</v>
+      </c>
+      <c r="D8" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="23" t="s">
-        <v>262</v>
-      </c>
-      <c r="F8" s="23" t="s">
-        <v>263</v>
+      <c r="E8" s="20" t="s">
+        <v>318</v>
+      </c>
+      <c r="F8" s="20" t="s">
+        <v>319</v>
       </c>
       <c r="G8" s="15" t="n">
         <f aca="false">機票價格!M7</f>
@@ -8162,42 +9107,42 @@
         <f aca="false">2*機票價格!O7</f>
         <v>0</v>
       </c>
-      <c r="I8" s="33" t="n">
+      <c r="I8" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="27" t="n">
+      <c r="J8" s="31" t="n">
         <f aca="false">I8*總覽!$B$5</f>
         <v>0</v>
       </c>
-      <c r="K8" s="27" t="n">
+      <c r="K8" s="31" t="n">
         <f aca="false">G8+H8+J8</f>
         <v>19586</v>
       </c>
-      <c r="L8" s="23" t="s">
-        <v>248</v>
+      <c r="L8" s="20" t="s">
+        <v>304</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>264</v>
+        <v>320</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="s">
-        <v>265</v>
+      <c r="A9" s="20" t="s">
+        <v>321</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>266</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>245</v>
-      </c>
-      <c r="D9" s="32" t="n">
+        <v>322</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>301</v>
+      </c>
+      <c r="D9" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="23" t="s">
-        <v>267</v>
-      </c>
-      <c r="F9" s="23" t="s">
-        <v>268</v>
+      <c r="E9" s="20" t="s">
+        <v>323</v>
+      </c>
+      <c r="F9" s="20" t="s">
+        <v>324</v>
       </c>
       <c r="G9" s="15" t="n">
         <f aca="false">機票價格!M8</f>
@@ -8207,43 +9152,43 @@
         <f aca="false">2*機票價格!O8</f>
         <v>0</v>
       </c>
-      <c r="I9" s="33" t="n">
+      <c r="I9" s="37" t="n">
         <f aca="false">2*(12580+500)-1690-680*2</f>
         <v>23110</v>
       </c>
-      <c r="J9" s="27" t="n">
+      <c r="J9" s="31" t="n">
         <f aca="false">I9*總覽!$B$5</f>
         <v>4853.1</v>
       </c>
-      <c r="K9" s="27" t="n">
+      <c r="K9" s="31" t="n">
         <f aca="false">G9+H9+J9</f>
         <v>21379.1</v>
       </c>
-      <c r="L9" s="23" t="s">
-        <v>269</v>
+      <c r="L9" s="20" t="s">
+        <v>325</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>270</v>
+        <v>326</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
-        <v>271</v>
+      <c r="A10" s="20" t="s">
+        <v>327</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>272</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>245</v>
-      </c>
-      <c r="D10" s="32" t="n">
+        <v>328</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>301</v>
+      </c>
+      <c r="D10" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="23" t="s">
-        <v>252</v>
-      </c>
-      <c r="F10" s="23" t="s">
-        <v>268</v>
+      <c r="E10" s="20" t="s">
+        <v>308</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>324</v>
       </c>
       <c r="G10" s="15" t="n">
         <f aca="false">機票價格!L5+機票價格!L8</f>
@@ -8253,43 +9198,43 @@
         <f aca="false">機票價格!O5</f>
         <v>950</v>
       </c>
-      <c r="I10" s="33" t="n">
+      <c r="I10" s="37" t="n">
         <f aca="false">12580+500-1690-680</f>
         <v>10710</v>
       </c>
-      <c r="J10" s="27" t="n">
+      <c r="J10" s="31" t="n">
         <f aca="false">I10*總覽!$B$5</f>
         <v>2249.1</v>
       </c>
-      <c r="K10" s="27" t="n">
+      <c r="K10" s="31" t="n">
         <f aca="false">G10+H10+J10</f>
         <v>18303.1</v>
       </c>
-      <c r="L10" s="23" t="s">
-        <v>248</v>
+      <c r="L10" s="20" t="s">
+        <v>304</v>
       </c>
       <c r="M10" s="16" t="s">
-        <v>273</v>
+        <v>329</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="s">
-        <v>274</v>
+      <c r="A11" s="20" t="s">
+        <v>330</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>275</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>245</v>
-      </c>
-      <c r="D11" s="32" t="n">
+        <v>331</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>301</v>
+      </c>
+      <c r="D11" s="36" t="n">
         <v>4</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>276</v>
+        <v>332</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>277</v>
+        <v>333</v>
       </c>
       <c r="G11" s="15" t="n">
         <f aca="false">機票價格!M12</f>
@@ -8299,28 +9244,28 @@
         <f aca="false">2*機票價格!O12</f>
         <v>2000</v>
       </c>
-      <c r="I11" s="33" t="n">
+      <c r="I11" s="37" t="n">
         <f aca="false">2*(12580+500)-1690-680*2</f>
         <v>23110</v>
       </c>
-      <c r="J11" s="27" t="n">
+      <c r="J11" s="31" t="n">
         <f aca="false">I11*總覽!$B$5</f>
         <v>4853.1</v>
       </c>
-      <c r="K11" s="27" t="n">
+      <c r="K11" s="31" t="n">
         <f aca="false">G11+H11+J11</f>
         <v>17625.1</v>
       </c>
-      <c r="L11" s="23" t="s">
-        <v>269</v>
+      <c r="L11" s="20" t="s">
+        <v>325</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>279</v>
+        <v>335</v>
       </c>
       <c r="C13" s="3" t="str">
         <f aca="false">INDEX(B5:B11,MATCH(MIN(K5:K11),K5:K11,0))</f>
@@ -8342,7 +9287,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -8362,13 +9307,13 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
-        <v>280</v>
+      <c r="A1" s="25" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>281</v>
+        <v>337</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8376,260 +9321,260 @@
         <v>11</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>30</v>
+        <v>92</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>282</v>
+        <v>338</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>283</v>
+        <v>339</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>284</v>
+        <v>340</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>285</v>
+        <v>341</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>286</v>
+        <v>342</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>287</v>
+        <v>343</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>288</v>
+        <v>344</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
-        <v>289</v>
+      <c r="A5" s="20" t="s">
+        <v>35</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>291</v>
-      </c>
-      <c r="D5" s="33" t="n">
+        <v>346</v>
+      </c>
+      <c r="D5" s="37" t="n">
         <v>1310</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>292</v>
-      </c>
-      <c r="F5" s="33" t="n">
+        <v>347</v>
+      </c>
+      <c r="F5" s="37" t="n">
         <v>9000</v>
       </c>
-      <c r="G5" s="33" t="n">
+      <c r="G5" s="37" t="n">
         <v>570</v>
       </c>
-      <c r="H5" s="34" t="n">
+      <c r="H5" s="38" t="n">
         <f aca="false">D5+F5+G5</f>
         <v>10880</v>
       </c>
-      <c r="I5" s="27" t="n">
+      <c r="I5" s="31" t="n">
         <f aca="false">H5*總覽!$B$5</f>
         <v>2284.8</v>
       </c>
-      <c r="J5" s="35" t="s">
-        <v>293</v>
+      <c r="J5" s="39" t="s">
+        <v>348</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
-        <v>294</v>
+      <c r="A6" s="20" t="s">
+        <v>47</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>295</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>296</v>
-      </c>
-      <c r="D6" s="33" t="n">
+        <v>349</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>350</v>
+      </c>
+      <c r="D6" s="37" t="n">
         <v>2300</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>297</v>
-      </c>
-      <c r="F6" s="33" t="n">
+        <v>351</v>
+      </c>
+      <c r="F6" s="37" t="n">
         <v>20000</v>
       </c>
-      <c r="G6" s="33" t="n">
+      <c r="G6" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="34" t="n">
+      <c r="H6" s="38" t="n">
         <f aca="false">D6+F6+G6</f>
         <v>22300</v>
       </c>
-      <c r="I6" s="27" t="n">
+      <c r="I6" s="31" t="n">
         <f aca="false">H6*總覽!$B$5</f>
         <v>4683</v>
       </c>
-      <c r="J6" s="35" t="s">
-        <v>298</v>
+      <c r="J6" s="39" t="s">
+        <v>352</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="s">
-        <v>299</v>
+      <c r="A7" s="20" t="s">
+        <v>49</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>300</v>
+        <v>353</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>301</v>
-      </c>
-      <c r="D7" s="33" t="n">
+        <v>354</v>
+      </c>
+      <c r="D7" s="37" t="n">
         <v>1200</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>302</v>
-      </c>
-      <c r="F7" s="33" t="n">
+        <v>355</v>
+      </c>
+      <c r="F7" s="37" t="n">
         <v>8000</v>
       </c>
-      <c r="G7" s="33" t="n">
+      <c r="G7" s="37" t="n">
         <v>4400</v>
       </c>
-      <c r="H7" s="34" t="n">
+      <c r="H7" s="38" t="n">
         <f aca="false">D7+F7+G7</f>
         <v>13600</v>
       </c>
-      <c r="I7" s="27" t="n">
+      <c r="I7" s="31" t="n">
         <f aca="false">H7*總覽!$B$5</f>
         <v>2856</v>
       </c>
-      <c r="J7" s="35" t="s">
-        <v>303</v>
+      <c r="J7" s="39" t="s">
+        <v>356</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23" t="s">
-        <v>304</v>
+      <c r="A8" s="20" t="s">
+        <v>357</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>305</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>306</v>
-      </c>
-      <c r="D8" s="33" t="n">
+        <v>358</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>359</v>
+      </c>
+      <c r="D8" s="37" t="n">
         <v>1900</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>307</v>
-      </c>
-      <c r="F8" s="36" t="n">
+        <v>360</v>
+      </c>
+      <c r="F8" s="40" t="n">
         <f aca="false">總覽!B7</f>
         <v>0</v>
       </c>
-      <c r="G8" s="33" t="n">
+      <c r="G8" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="34" t="n">
+      <c r="H8" s="38" t="n">
         <f aca="false">D8+F8+G8</f>
         <v>1900</v>
       </c>
-      <c r="I8" s="27" t="n">
+      <c r="I8" s="31" t="n">
         <f aca="false">H8*總覽!$B$5</f>
         <v>399</v>
       </c>
-      <c r="J8" s="37" t="s">
-        <v>308</v>
+      <c r="J8" s="41" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="s">
-        <v>309</v>
+      <c r="A9" s="20" t="s">
+        <v>66</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>310</v>
+        <v>362</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>311</v>
-      </c>
-      <c r="D9" s="33" t="n">
+        <v>363</v>
+      </c>
+      <c r="D9" s="37" t="n">
         <v>2690</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>292</v>
-      </c>
-      <c r="F9" s="33" t="n">
+        <v>347</v>
+      </c>
+      <c r="F9" s="37" t="n">
         <v>9000</v>
       </c>
-      <c r="G9" s="33" t="n">
+      <c r="G9" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="34" t="n">
+      <c r="H9" s="38" t="n">
         <f aca="false">D9+F9+G9</f>
         <v>11690</v>
       </c>
-      <c r="I9" s="27" t="n">
+      <c r="I9" s="31" t="n">
         <f aca="false">H9*總覽!$B$5</f>
         <v>2454.9</v>
       </c>
-      <c r="J9" s="35"/>
+      <c r="J9" s="39"/>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
-        <v>312</v>
+      <c r="A10" s="20" t="s">
+        <v>58</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>313</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>314</v>
-      </c>
-      <c r="D10" s="33" t="n">
+        <v>364</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>365</v>
+      </c>
+      <c r="D10" s="37" t="n">
         <v>1540</v>
       </c>
-      <c r="E10" s="23" t="s">
-        <v>315</v>
-      </c>
-      <c r="F10" s="33" t="n">
+      <c r="E10" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="33" t="n">
+      <c r="G10" s="37" t="n">
         <v>2200</v>
       </c>
-      <c r="H10" s="34" t="n">
+      <c r="H10" s="38" t="n">
         <f aca="false">D10+F10+G10</f>
         <v>3740</v>
       </c>
-      <c r="I10" s="27" t="n">
+      <c r="I10" s="31" t="n">
         <f aca="false">H10*總覽!$B$5</f>
         <v>785.4</v>
       </c>
-      <c r="J10" s="35" t="s">
-        <v>316</v>
+      <c r="J10" s="39" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="38" t="s">
+      <c r="A11" s="42" t="s">
         <v>25</v>
       </c>
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
-      <c r="D11" s="39" t="n">
+      <c r="D11" s="43" t="n">
         <f aca="false">SUM(D5:D10)</f>
         <v>10940</v>
       </c>
       <c r="E11" s="16"/>
-      <c r="F11" s="39" t="n">
+      <c r="F11" s="43" t="n">
         <f aca="false">SUM(F5:F10)</f>
         <v>46000</v>
       </c>
-      <c r="G11" s="39" t="n">
+      <c r="G11" s="43" t="n">
         <f aca="false">SUM(G5:G10)</f>
         <v>7170</v>
       </c>
-      <c r="H11" s="39" t="n">
+      <c r="H11" s="43" t="n">
         <f aca="false">SUM(H5:H10)</f>
         <v>64110</v>
       </c>
-      <c r="I11" s="40" t="n">
+      <c r="I11" s="44" t="n">
         <f aca="false">SUM(I5:I10)</f>
         <v>13463.1</v>
       </c>
@@ -8637,31 +9582,31 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>317</v>
-      </c>
-      <c r="H12" s="41" t="n">
+        <v>367</v>
+      </c>
+      <c r="H12" s="45" t="n">
         <v>5000</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>318</v>
+        <v>368</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>319</v>
-      </c>
-      <c r="H13" s="42" t="n">
+        <v>369</v>
+      </c>
+      <c r="H13" s="46" t="n">
         <f aca="false">H12*6</f>
         <v>30000</v>
       </c>
-      <c r="I13" s="43" t="n">
+      <c r="I13" s="47" t="n">
         <f aca="false">H13*總覽!$B$5</f>
         <v>6300</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>320</v>
+        <v>370</v>
       </c>
       <c r="I14" s="18" t="n">
         <f aca="false">I11+I13</f>
@@ -8679,7 +9624,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -8695,114 +9640,114 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>322</v>
+        <v>372</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>323</v>
+        <v>373</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>324</v>
-      </c>
-      <c r="B2" s="23" t="s">
-        <v>325</v>
-      </c>
-      <c r="C2" s="44" t="s">
-        <v>326</v>
+        <v>374</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>375</v>
+      </c>
+      <c r="C2" s="48" t="s">
+        <v>376</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>327</v>
+        <v>377</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>328</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>325</v>
-      </c>
-      <c r="C3" s="44" t="s">
-        <v>326</v>
+        <v>378</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>375</v>
+      </c>
+      <c r="C3" s="48" t="s">
+        <v>376</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>329</v>
+        <v>379</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>330</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>325</v>
-      </c>
-      <c r="C4" s="44" t="s">
-        <v>326</v>
+        <v>380</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>375</v>
+      </c>
+      <c r="C4" s="48" t="s">
+        <v>376</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>331</v>
+        <v>381</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>332</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>333</v>
-      </c>
-      <c r="C5" s="44" t="s">
-        <v>326</v>
+        <v>382</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>383</v>
+      </c>
+      <c r="C5" s="48" t="s">
+        <v>376</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>334</v>
+        <v>384</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>335</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>336</v>
-      </c>
-      <c r="C6" s="44" t="s">
-        <v>326</v>
+        <v>385</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>386</v>
+      </c>
+      <c r="C6" s="48" t="s">
+        <v>376</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>337</v>
+        <v>387</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>338</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>339</v>
-      </c>
-      <c r="C7" s="44" t="s">
-        <v>326</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>340</v>
+        <v>388</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>389</v>
+      </c>
+      <c r="C7" s="48" t="s">
+        <v>376</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>341</v>
+        <v>391</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>342</v>
-      </c>
-      <c r="C8" s="44" t="s">
-        <v>326</v>
+        <v>392</v>
+      </c>
+      <c r="C8" s="48" t="s">
+        <v>376</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>343</v>
+        <v>393</v>
       </c>
     </row>
   </sheetData>
@@ -8822,7 +9767,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -8836,138 +9781,138 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>344</v>
+        <v>394</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>345</v>
+        <v>395</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>346</v>
-      </c>
-      <c r="B2" s="45" t="s">
-        <v>347</v>
+        <v>396</v>
+      </c>
+      <c r="B2" s="49" t="s">
+        <v>397</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>348</v>
-      </c>
-      <c r="B3" s="45" t="s">
-        <v>349</v>
+        <v>398</v>
+      </c>
+      <c r="B3" s="49" t="s">
+        <v>399</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="46" t="s">
-        <v>350</v>
-      </c>
-      <c r="B4" s="45" t="s">
-        <v>351</v>
+      <c r="A4" s="50" t="s">
+        <v>400</v>
+      </c>
+      <c r="B4" s="49" t="s">
+        <v>401</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="46" t="s">
-        <v>352</v>
-      </c>
-      <c r="B5" s="45" t="s">
-        <v>353</v>
+      <c r="A5" s="50" t="s">
+        <v>402</v>
+      </c>
+      <c r="B5" s="49" t="s">
+        <v>403</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="46" t="s">
-        <v>354</v>
-      </c>
-      <c r="B6" s="45" t="s">
-        <v>355</v>
+      <c r="A6" s="50" t="s">
+        <v>404</v>
+      </c>
+      <c r="B6" s="49" t="s">
+        <v>405</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="46" t="s">
-        <v>356</v>
-      </c>
-      <c r="B7" s="45" t="s">
-        <v>357</v>
+      <c r="A7" s="50" t="s">
+        <v>406</v>
+      </c>
+      <c r="B7" s="49" t="s">
+        <v>407</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="46" t="s">
-        <v>358</v>
-      </c>
-      <c r="B8" s="45" t="s">
-        <v>359</v>
+      <c r="A8" s="50" t="s">
+        <v>408</v>
+      </c>
+      <c r="B8" s="49" t="s">
+        <v>409</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>360</v>
-      </c>
-      <c r="B9" s="45" t="s">
-        <v>361</v>
+        <v>410</v>
+      </c>
+      <c r="B9" s="49" t="s">
+        <v>411</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="46" t="s">
-        <v>362</v>
-      </c>
-      <c r="B10" s="45" t="s">
-        <v>363</v>
+      <c r="A10" s="50" t="s">
+        <v>412</v>
+      </c>
+      <c r="B10" s="49" t="s">
+        <v>413</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="46" t="s">
-        <v>364</v>
-      </c>
-      <c r="B11" s="45" t="s">
-        <v>365</v>
+      <c r="A11" s="50" t="s">
+        <v>414</v>
+      </c>
+      <c r="B11" s="49" t="s">
+        <v>415</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>366</v>
-      </c>
-      <c r="B12" s="45" t="s">
-        <v>367</v>
+        <v>416</v>
+      </c>
+      <c r="B12" s="49" t="s">
+        <v>417</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>368</v>
-      </c>
-      <c r="B13" s="45" t="s">
-        <v>369</v>
+        <v>418</v>
+      </c>
+      <c r="B13" s="49" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>370</v>
-      </c>
-      <c r="B14" s="45" t="s">
-        <v>371</v>
+        <v>420</v>
+      </c>
+      <c r="B14" s="49" t="s">
+        <v>421</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>372</v>
-      </c>
-      <c r="B15" s="45" t="s">
-        <v>373</v>
+        <v>422</v>
+      </c>
+      <c r="B15" s="49" t="s">
+        <v>423</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>374</v>
-      </c>
-      <c r="B16" s="45" t="s">
-        <v>375</v>
+        <v>424</v>
+      </c>
+      <c r="B16" s="49" t="s">
+        <v>425</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="B17" s="45" t="s">
-        <v>377</v>
+        <v>426</v>
+      </c>
+      <c r="B17" s="49" t="s">
+        <v>427</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 1/30-2/3 return flight availability to live price sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MqDR8ErShU29xSVraYyKeW
</commit_message>
<xml_diff>
--- a/japan-ginzan-plan.xlsx
+++ b/japan-ginzan-plan.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="441">
   <si>
     <r>
       <rPr>
@@ -439,7 +439,28 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">查詢，每人單程經濟艙，含稅，新台幣）</t>
+      <t xml:space="preserve">查詢；回程含 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/30–2/3</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">，每人單程經濟艙，含稅，新台幣）</t>
     </r>
   </si>
   <si>
@@ -777,7 +798,58 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">經濟艙查不到</t>
+    <t xml:space="preserve">唯一的直飛，經濟艙查不到</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">二</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">19:40 → 23:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有位；含行李</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">三</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">沒有直飛</t>
   </si>
   <si>
     <t xml:space="preserve">成田→桃園</t>
@@ -786,18 +858,72 @@
     <t xml:space="preserve">泰國獅航</t>
   </si>
   <si>
+    <t xml:space="preserve">18:15 → 21:10</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">有位；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">最便宜的晚班</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">酷航</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:45 → 22:55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:25 → 21:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:10 → 23:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:45 → 16:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">羽田→松山</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12:15 → 15:05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">有位；回松山最晚的平價班次</t>
+  </si>
+  <si>
     <t xml:space="preserve">17:25 → 20:20</t>
   </si>
   <si>
+    <t xml:space="preserve">19:45 → 23:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">有位；晚回又能搭捷運回家</t>
   </si>
   <si>
-    <t xml:space="preserve">酷航</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:45 → 22:55</t>
-  </si>
-  <si>
     <t xml:space="preserve">20:25 → 23:25</t>
   </si>
   <si>
@@ -844,9 +970,6 @@
   </si>
   <si>
     <t xml:space="preserve">20:20 → 23:25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">羽田→松山</t>
   </si>
   <si>
     <t xml:space="preserve">07:55 → 10:55</t>
@@ -7081,7 +7204,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -7458,7 +7581,7 @@
         <v>63</v>
       </c>
       <c r="E19" s="24" t="n">
-        <v>34279</v>
+        <v>34247</v>
       </c>
       <c r="F19" s="23" t="s">
         <v>61</v>
@@ -7469,88 +7592,86 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="C20" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="D20" s="20" t="s">
-        <v>73</v>
-      </c>
       <c r="E20" s="21" t="n">
-        <v>14542</v>
+        <v>16439</v>
       </c>
       <c r="F20" s="16" t="s">
         <v>39</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>74</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="E21" s="21" t="n">
-        <v>13212</v>
+        <v>20518</v>
       </c>
       <c r="F21" s="16" t="s">
         <v>39</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="B22" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="D22" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="E22" s="21" t="n">
-        <v>13149</v>
-      </c>
-      <c r="F22" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="G22" s="16" t="s">
-        <v>78</v>
+      <c r="A22" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="D22" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="E22" s="24"/>
+      <c r="F22" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="G22" s="23" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>80</v>
+        <v>54</v>
       </c>
       <c r="E23" s="21" t="n">
-        <v>18549</v>
+        <v>17309</v>
       </c>
       <c r="F23" s="16" t="s">
         <v>39</v>
@@ -7561,94 +7682,416 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="E24" s="21" t="n">
-        <v>21166</v>
+        <v>17246</v>
       </c>
       <c r="F24" s="16" t="s">
         <v>39</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>82</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E25" s="21" t="n">
-        <v>27583</v>
+        <v>10294</v>
       </c>
       <c r="F25" s="16" t="s">
         <v>39</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>43</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E26" s="21" t="n">
-        <v>15742</v>
+        <v>10752</v>
       </c>
       <c r="F26" s="16" t="s">
         <v>39</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>86</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D27" s="20" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E27" s="21" t="n">
-        <v>37120</v>
+        <v>13137</v>
       </c>
       <c r="F27" s="16" t="s">
         <v>39</v>
       </c>
       <c r="G27" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B28" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="E28" s="21" t="n">
+        <v>16591</v>
+      </c>
+      <c r="F28" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G28" s="16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D29" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="E29" s="21" t="n">
+        <v>16591</v>
+      </c>
+      <c r="F29" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G29" s="16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B30" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D30" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="E30" s="21" t="n">
+        <v>14855</v>
+      </c>
+      <c r="F30" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G30" s="16" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="D31" s="20" t="s">
         <v>88</v>
+      </c>
+      <c r="E31" s="21" t="n">
+        <v>16343</v>
+      </c>
+      <c r="F31" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G31" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="E32" s="21" t="n">
+        <v>10752</v>
+      </c>
+      <c r="F32" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G32" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B33" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D33" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="E33" s="21" t="n">
+        <v>10752</v>
+      </c>
+      <c r="F33" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G33" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="D34" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="E34" s="21" t="n">
+        <v>14542</v>
+      </c>
+      <c r="F34" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G34" s="16" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B35" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="E35" s="21" t="n">
+        <v>13212</v>
+      </c>
+      <c r="F35" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G35" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D36" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="E36" s="21" t="n">
+        <v>13149</v>
+      </c>
+      <c r="F36" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G36" s="16" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D37" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="E37" s="21" t="n">
+        <v>18549</v>
+      </c>
+      <c r="F37" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G37" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B38" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D38" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="E38" s="21" t="n">
+        <v>21166</v>
+      </c>
+      <c r="F38" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G38" s="16" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B39" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D39" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="E39" s="21" t="n">
+        <v>27583</v>
+      </c>
+      <c r="F39" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G39" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B40" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="D40" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="E40" s="21" t="n">
+        <v>15742</v>
+      </c>
+      <c r="F40" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G40" s="16" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B41" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D41" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="E41" s="21" t="n">
+        <v>37120</v>
+      </c>
+      <c r="F41" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G41" s="16" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -7679,12 +8122,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7692,156 +8135,156 @@
         <v>11</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="C5" s="28" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="E5" s="28" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16"/>
       <c r="B6" s="20" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16"/>
       <c r="B7" s="20" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16"/>
       <c r="B8" s="20" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16"/>
       <c r="B9" s="20" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16"/>
       <c r="B10" s="20" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16"/>
       <c r="B11" s="20" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="D11" s="16"/>
       <c r="E11" s="16" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="26" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="B12" s="27" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="C12" s="28" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="D12" s="27" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="E12" s="28" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16"/>
       <c r="B13" s="20" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="D13" s="16"/>
       <c r="E13" s="16" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16"/>
       <c r="B14" s="20" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
@@ -7849,83 +8292,83 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16"/>
       <c r="B15" s="20" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="E15" s="16"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16"/>
       <c r="B16" s="20" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="16"/>
       <c r="B17" s="20" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="D17" s="16"/>
       <c r="E17" s="16" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16"/>
       <c r="B18" s="20" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="26" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="C19" s="28" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="D19" s="28" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="E19" s="28" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16"/>
       <c r="B20" s="20" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="D20" s="16"/>
       <c r="E20" s="16"/>
@@ -7933,120 +8376,120 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16"/>
       <c r="B21" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>162</v>
+      </c>
+      <c r="D21" s="16" t="s">
         <v>148</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>149</v>
-      </c>
-      <c r="D21" s="16" t="s">
-        <v>135</v>
       </c>
       <c r="E21" s="16"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16"/>
       <c r="B22" s="20" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="16"/>
       <c r="B23" s="20" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="D23" s="16"/>
       <c r="E23" s="16" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="26" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="B24" s="27" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="C24" s="28" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="D24" s="28"/>
       <c r="E24" s="28" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16"/>
       <c r="B25" s="20" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="E25" s="16"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16"/>
       <c r="B26" s="20" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="E26" s="16" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12"/>
       <c r="B27" s="29" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="12" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16"/>
       <c r="B28" s="20" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="D28" s="16"/>
       <c r="E28" s="16" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16"/>
       <c r="B29" s="20" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
@@ -8054,38 +8497,38 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16"/>
       <c r="B30" s="20" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D30" s="16"/>
       <c r="E30" s="16" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="26" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="B31" s="27" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="C31" s="28" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="D31" s="28"/>
       <c r="E31" s="28" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16"/>
       <c r="B32" s="20" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
@@ -8093,38 +8536,38 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16"/>
       <c r="B33" s="20" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="E33" s="16"/>
     </row>
     <row r="34" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="16"/>
       <c r="B34" s="20" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="E34" s="16" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16"/>
       <c r="B35" s="20" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
@@ -8132,38 +8575,38 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16"/>
       <c r="B36" s="20" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="D36" s="16"/>
       <c r="E36" s="16" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16"/>
       <c r="B37" s="20" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="D37" s="16"/>
       <c r="E37" s="16" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="26" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="B38" s="27" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="C38" s="28" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="D38" s="28"/>
       <c r="E38" s="28"/>
@@ -8171,114 +8614,114 @@
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16"/>
       <c r="B39" s="20" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="D39" s="20" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="E39" s="16"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16"/>
       <c r="B40" s="20" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="E40" s="16"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="16"/>
       <c r="B41" s="20" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="E41" s="16"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="16"/>
       <c r="B42" s="20" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="D42" s="16"/>
       <c r="E42" s="16" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="16"/>
       <c r="B43" s="20" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="D43" s="20" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="E43" s="16"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="16"/>
       <c r="B44" s="20" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="E44" s="16" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="16"/>
       <c r="B45" s="20" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="D45" s="16"/>
       <c r="E45" s="16" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="16"/>
       <c r="B46" s="20" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="E46" s="16" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -8316,17 +8759,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>29</v>
@@ -8335,66 +8778,66 @@
         <v>30</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>44</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>4743</v>
@@ -8413,36 +8856,36 @@
         <v>9676</v>
       </c>
       <c r="N5" s="16" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="O5" s="21" t="n">
         <v>950</v>
       </c>
       <c r="P5" s="16" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>37</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>243</v>
+        <v>256</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>244</v>
+        <v>257</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>245</v>
+        <v>258</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>9845</v>
@@ -8461,36 +8904,36 @@
         <v>17878</v>
       </c>
       <c r="N6" s="16" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="O6" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P6" s="16" t="s">
-        <v>247</v>
+        <v>260</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>41</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>249</v>
+        <v>262</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>250</v>
+        <v>263</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>251</v>
+        <v>264</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="H7" s="21" t="n">
         <v>9720</v>
@@ -8509,36 +8952,36 @@
         <v>19586</v>
       </c>
       <c r="N7" s="16" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="O7" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P7" s="16" t="s">
-        <v>253</v>
+        <v>266</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>37</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>257</v>
+        <v>270</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="H8" s="21" t="n">
         <v>10361</v>
@@ -8557,36 +9000,36 @@
         <v>16526</v>
       </c>
       <c r="N8" s="16" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="O8" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P8" s="16" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>260</v>
+        <v>273</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>261</v>
+        <v>274</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>262</v>
+        <v>275</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>263</v>
+        <v>276</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="H9" s="21" t="n">
         <v>10361</v>
@@ -8605,36 +9048,36 @@
         <v>16526</v>
       </c>
       <c r="N9" s="16" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="O9" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P9" s="16" t="s">
-        <v>264</v>
+        <v>277</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
+        <v>278</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>268</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>279</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>280</v>
+      </c>
+      <c r="E10" s="20" t="s">
+        <v>281</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>271</v>
+      </c>
+      <c r="G10" s="16" t="s">
         <v>265</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>255</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>266</v>
-      </c>
-      <c r="D10" s="20" t="s">
-        <v>267</v>
-      </c>
-      <c r="E10" s="20" t="s">
-        <v>268</v>
-      </c>
-      <c r="F10" s="16" t="s">
-        <v>258</v>
-      </c>
-      <c r="G10" s="16" t="s">
-        <v>252</v>
       </c>
       <c r="H10" s="21" t="n">
         <v>10361</v>
@@ -8653,36 +9096,36 @@
         <v>16526</v>
       </c>
       <c r="N10" s="16" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="O10" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P10" s="16" t="s">
-        <v>264</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>269</v>
+        <v>282</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>270</v>
+        <v>283</v>
       </c>
       <c r="D11" s="20" t="s">
+        <v>284</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>285</v>
+      </c>
+      <c r="F11" s="16" t="s">
         <v>271</v>
       </c>
-      <c r="E11" s="20" t="s">
-        <v>272</v>
-      </c>
-      <c r="F11" s="16" t="s">
-        <v>258</v>
-      </c>
       <c r="G11" s="16" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="H11" s="21" t="n">
         <v>10361</v>
@@ -8701,36 +9144,36 @@
         <v>16526</v>
       </c>
       <c r="N11" s="16" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="O11" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P11" s="16" t="s">
-        <v>264</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>273</v>
+        <v>286</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>274</v>
+        <v>287</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>275</v>
+        <v>288</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="H12" s="21" t="n">
         <v>5386</v>
@@ -8750,36 +9193,36 @@
         <v>10772</v>
       </c>
       <c r="N12" s="16" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="O12" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="P12" s="16" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>278</v>
+        <v>291</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>279</v>
+        <v>292</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>281</v>
+        <v>294</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="H13" s="21" t="n">
         <v>3748</v>
@@ -8799,36 +9242,36 @@
         <v>7496</v>
       </c>
       <c r="N13" s="16" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="O13" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="P13" s="16" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>274</v>
+        <v>287</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>44</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>284</v>
+        <v>297</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="H14" s="21" t="n">
         <v>6702</v>
@@ -8848,18 +9291,18 @@
         <v>13404</v>
       </c>
       <c r="N14" s="16" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="O14" s="21" t="n">
         <v>950</v>
       </c>
       <c r="P14" s="16" t="s">
-        <v>285</v>
+        <v>298</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
     </row>
   </sheetData>
@@ -8896,17 +9339,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>288</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>289</v>
+        <v>302</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>10</v>
@@ -8918,51 +9361,51 @@
         <v>12</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>291</v>
+        <v>304</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>292</v>
+        <v>305</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>293</v>
+        <v>306</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>294</v>
+        <v>307</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>296</v>
+        <v>309</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="29" t="s">
-        <v>299</v>
+        <v>312</v>
       </c>
       <c r="B5" s="32" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="D5" s="33" t="n">
         <v>4</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>302</v>
+        <v>315</v>
       </c>
       <c r="F5" s="29" t="s">
-        <v>303</v>
+        <v>316</v>
       </c>
       <c r="G5" s="11" t="n">
         <f aca="false">機票價格!L6+機票價格!L5</f>
@@ -8984,30 +9427,30 @@
         <v>15538</v>
       </c>
       <c r="L5" s="29" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>305</v>
+        <v>318</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>306</v>
+        <v>319</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>307</v>
+        <v>320</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="D6" s="36" t="n">
         <v>4</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>309</v>
+        <v>322</v>
       </c>
       <c r="G6" s="15" t="n">
         <f aca="false">機票價格!M5</f>
@@ -9029,30 +9472,30 @@
         <v>11576</v>
       </c>
       <c r="L6" s="20" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="M6" s="16" t="s">
-        <v>310</v>
+        <v>323</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>311</v>
+        <v>324</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>312</v>
+        <v>325</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>313</v>
+        <v>326</v>
       </c>
       <c r="D7" s="36" t="n">
         <v>3</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>314</v>
+        <v>327</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>309</v>
+        <v>322</v>
       </c>
       <c r="G7" s="15" t="n">
         <f aca="false">機票價格!L6+機票價格!L5</f>
@@ -9074,30 +9517,30 @@
         <v>15538</v>
       </c>
       <c r="L7" s="20" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="M7" s="16" t="s">
-        <v>315</v>
+        <v>328</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>316</v>
+        <v>329</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>317</v>
+        <v>330</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>313</v>
+        <v>326</v>
       </c>
       <c r="D8" s="36" t="n">
         <v>3</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>318</v>
+        <v>331</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>319</v>
+        <v>332</v>
       </c>
       <c r="G8" s="15" t="n">
         <f aca="false">機票價格!M7</f>
@@ -9119,30 +9562,30 @@
         <v>19586</v>
       </c>
       <c r="L8" s="20" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>320</v>
+        <v>333</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>321</v>
+        <v>334</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>322</v>
+        <v>335</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="D9" s="36" t="n">
         <v>4</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>323</v>
+        <v>336</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>324</v>
+        <v>337</v>
       </c>
       <c r="G9" s="15" t="n">
         <f aca="false">機票價格!M8</f>
@@ -9165,30 +9608,30 @@
         <v>21379.1</v>
       </c>
       <c r="L9" s="20" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>326</v>
+        <v>339</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>327</v>
+        <v>340</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>328</v>
+        <v>341</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="D10" s="36" t="n">
         <v>4</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>324</v>
+        <v>337</v>
       </c>
       <c r="G10" s="15" t="n">
         <f aca="false">機票價格!L5+機票價格!L8</f>
@@ -9211,30 +9654,30 @@
         <v>18303.1</v>
       </c>
       <c r="L10" s="20" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="M10" s="16" t="s">
-        <v>329</v>
+        <v>342</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>330</v>
+        <v>343</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>331</v>
+        <v>344</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="D11" s="36" t="n">
         <v>4</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>332</v>
+        <v>345</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>333</v>
+        <v>346</v>
       </c>
       <c r="G11" s="15" t="n">
         <f aca="false">機票價格!M12</f>
@@ -9257,15 +9700,15 @@
         <v>17625.1</v>
       </c>
       <c r="L11" s="20" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>334</v>
+        <v>347</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>335</v>
+        <v>348</v>
       </c>
       <c r="C13" s="3" t="str">
         <f aca="false">INDEX(B5:B11,MATCH(MIN(K5:K11),K5:K11,0))</f>
@@ -9308,12 +9751,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>336</v>
+        <v>349</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>337</v>
+        <v>350</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9321,31 +9764,31 @@
         <v>11</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>338</v>
+        <v>351</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>339</v>
+        <v>352</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>340</v>
+        <v>353</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>341</v>
+        <v>354</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>342</v>
+        <v>355</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>343</v>
+        <v>356</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>344</v>
+        <v>357</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9353,16 +9796,16 @@
         <v>35</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>345</v>
+        <v>358</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>346</v>
+        <v>359</v>
       </c>
       <c r="D5" s="37" t="n">
         <v>1310</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>347</v>
+        <v>360</v>
       </c>
       <c r="F5" s="37" t="n">
         <v>9000</v>
@@ -9379,7 +9822,7 @@
         <v>2284.8</v>
       </c>
       <c r="J5" s="39" t="s">
-        <v>348</v>
+        <v>361</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9387,16 +9830,16 @@
         <v>47</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>349</v>
+        <v>362</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>350</v>
+        <v>363</v>
       </c>
       <c r="D6" s="37" t="n">
         <v>2300</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>351</v>
+        <v>364</v>
       </c>
       <c r="F6" s="37" t="n">
         <v>20000</v>
@@ -9413,7 +9856,7 @@
         <v>4683</v>
       </c>
       <c r="J6" s="39" t="s">
-        <v>352</v>
+        <v>365</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9421,16 +9864,16 @@
         <v>49</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>353</v>
+        <v>366</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>354</v>
+        <v>367</v>
       </c>
       <c r="D7" s="37" t="n">
         <v>1200</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>355</v>
+        <v>368</v>
       </c>
       <c r="F7" s="37" t="n">
         <v>8000</v>
@@ -9447,24 +9890,24 @@
         <v>2856</v>
       </c>
       <c r="J7" s="39" t="s">
-        <v>356</v>
+        <v>369</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>357</v>
+        <v>370</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>358</v>
+        <v>371</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>359</v>
+        <v>372</v>
       </c>
       <c r="D8" s="37" t="n">
         <v>1900</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>360</v>
+        <v>373</v>
       </c>
       <c r="F8" s="40" t="n">
         <f aca="false">總覽!B7</f>
@@ -9482,7 +9925,7 @@
         <v>399</v>
       </c>
       <c r="J8" s="41" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9490,16 +9933,16 @@
         <v>66</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>362</v>
+        <v>375</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="D9" s="37" t="n">
         <v>2690</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>347</v>
+        <v>360</v>
       </c>
       <c r="F9" s="37" t="n">
         <v>9000</v>
@@ -9522,10 +9965,10 @@
         <v>58</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>364</v>
+        <v>377</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>365</v>
+        <v>378</v>
       </c>
       <c r="D10" s="37" t="n">
         <v>1540</v>
@@ -9548,7 +9991,7 @@
         <v>785.4</v>
       </c>
       <c r="J10" s="39" t="s">
-        <v>366</v>
+        <v>379</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9582,18 +10025,18 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>367</v>
+        <v>380</v>
       </c>
       <c r="H12" s="45" t="n">
         <v>5000</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>368</v>
+        <v>381</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>369</v>
+        <v>382</v>
       </c>
       <c r="H13" s="46" t="n">
         <f aca="false">H12*6</f>
@@ -9606,7 +10049,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>370</v>
+        <v>383</v>
       </c>
       <c r="I14" s="18" t="n">
         <f aca="false">I11+I13</f>
@@ -9640,114 +10083,114 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>371</v>
+        <v>384</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>372</v>
+        <v>385</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>373</v>
+        <v>386</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>374</v>
+        <v>387</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>375</v>
+        <v>388</v>
       </c>
       <c r="C2" s="48" t="s">
-        <v>376</v>
+        <v>389</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>377</v>
+        <v>390</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>378</v>
+        <v>391</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>375</v>
+        <v>388</v>
       </c>
       <c r="C3" s="48" t="s">
-        <v>376</v>
+        <v>389</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>379</v>
+        <v>392</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>380</v>
+        <v>393</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>375</v>
+        <v>388</v>
       </c>
       <c r="C4" s="48" t="s">
-        <v>376</v>
+        <v>389</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>381</v>
+        <v>394</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>382</v>
+        <v>395</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>383</v>
+        <v>396</v>
       </c>
       <c r="C5" s="48" t="s">
-        <v>376</v>
+        <v>389</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>384</v>
+        <v>397</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>385</v>
+        <v>398</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>386</v>
+        <v>399</v>
       </c>
       <c r="C6" s="48" t="s">
-        <v>376</v>
+        <v>389</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>387</v>
+        <v>400</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>388</v>
+        <v>401</v>
       </c>
       <c r="B7" s="20" t="s">
+        <v>402</v>
+      </c>
+      <c r="C7" s="48" t="s">
         <v>389</v>
       </c>
-      <c r="C7" s="48" t="s">
-        <v>376</v>
-      </c>
       <c r="D7" s="20" t="s">
-        <v>390</v>
+        <v>403</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>391</v>
+        <v>404</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>392</v>
+        <v>405</v>
       </c>
       <c r="C8" s="48" t="s">
-        <v>376</v>
+        <v>389</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>393</v>
+        <v>406</v>
       </c>
     </row>
   </sheetData>
@@ -9781,138 +10224,138 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>394</v>
+        <v>407</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>395</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>396</v>
+        <v>409</v>
       </c>
       <c r="B2" s="49" t="s">
-        <v>397</v>
+        <v>410</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>398</v>
+        <v>411</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>399</v>
+        <v>412</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="50" t="s">
-        <v>400</v>
+        <v>413</v>
       </c>
       <c r="B4" s="49" t="s">
-        <v>401</v>
+        <v>414</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="50" t="s">
-        <v>402</v>
+        <v>415</v>
       </c>
       <c r="B5" s="49" t="s">
-        <v>403</v>
+        <v>416</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="50" t="s">
-        <v>404</v>
+        <v>417</v>
       </c>
       <c r="B6" s="49" t="s">
-        <v>405</v>
+        <v>418</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="50" t="s">
-        <v>406</v>
+        <v>419</v>
       </c>
       <c r="B7" s="49" t="s">
-        <v>407</v>
+        <v>420</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="50" t="s">
-        <v>408</v>
+        <v>421</v>
       </c>
       <c r="B8" s="49" t="s">
-        <v>409</v>
+        <v>422</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>410</v>
+        <v>423</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>411</v>
+        <v>424</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="50" t="s">
-        <v>412</v>
+        <v>425</v>
       </c>
       <c r="B10" s="49" t="s">
-        <v>413</v>
+        <v>426</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="50" t="s">
-        <v>414</v>
+        <v>427</v>
       </c>
       <c r="B11" s="49" t="s">
-        <v>415</v>
+        <v>428</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>416</v>
+        <v>429</v>
       </c>
       <c r="B12" s="49" t="s">
-        <v>417</v>
+        <v>430</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>418</v>
+        <v>431</v>
       </c>
       <c r="B13" s="49" t="s">
-        <v>419</v>
+        <v>432</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>420</v>
+        <v>433</v>
       </c>
       <c r="B14" s="49" t="s">
-        <v>421</v>
+        <v>434</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>422</v>
+        <v>435</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>423</v>
+        <v>436</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>424</v>
+        <v>437</v>
       </c>
       <c r="B16" s="49" t="s">
-        <v>425</v>
+        <v>438</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>426</v>
+        <v>439</v>
       </c>
       <c r="B17" s="49" t="s">
-        <v>427</v>
+        <v>440</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Sendai round-trip availability scan and combos (2026-10-10)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MqDR8ErShU29xSVraYyKeW
</commit_message>
<xml_diff>
--- a/japan-ginzan-plan.xlsx
+++ b/japan-ginzan-plan.xlsx
@@ -11,12 +11,13 @@
     <sheet name="總覽" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="即時查價 10-9" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="新方案 10-10" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="每日行程" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="機票價格" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="方案比較" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="行程預算" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="待辦清單" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="資料來源" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="仙台進出 10-10" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="每日行程" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="機票價格" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="方案比較" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="行程預算" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="待辦清單" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="資料來源" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="795" uniqueCount="516">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="565">
   <si>
     <r>
       <rPr>
@@ -3100,7 +3101,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">定案行程：早去晚回 </t>
+      <t xml:space="preserve">仙台進出：目前還買得到的直飛（</t>
     </r>
     <r>
       <rPr>
@@ -3111,7 +3112,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">6 </t>
+      <t xml:space="preserve">Google Flights 2026/10/10</t>
     </r>
     <r>
       <rPr>
@@ -3121,87 +3122,1182 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">，每人單程含稅，新台幣）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">去程查 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/22–1/28</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、回程查 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/30–2/3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。紅底＝只剩商務艙；沒列出的日期＝當天沒有直飛。虎航不含托運行李（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20kg </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">訂票時加購 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NT$950</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">方向</t>
+  </si>
+  <si>
+    <t xml:space="preserve">備註</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/22 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">五</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">經濟艙售完</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/23 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">六</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/24 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/25 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">一</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">含行李</t>
+  </si>
+  <si>
+    <t xml:space="preserve">含行李；去程最便宜的全服務航空</t>
+  </si>
+  <si>
+    <t xml:space="preserve">含行李；最早抵達</t>
+  </si>
+  <si>
+    <t xml:space="preserve">去程最便宜</t>
+  </si>
+  <si>
+    <t xml:space="preserve">回程唯一的平價選擇；落地晚</t>
+  </si>
+  <si>
+    <t xml:space="preserve">可行的組合（經濟艙去回）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">組合</t>
+  </si>
+  <si>
+    <t xml:space="preserve">去程價</t>
+  </si>
+  <si>
+    <t xml:space="preserve">回程價</t>
+  </si>
+  <si>
+    <t xml:space="preserve">行李加購</t>
+  </si>
+  <si>
+    <t xml:space="preserve">機票合計</t>
+  </si>
+  <si>
+    <t xml:space="preserve">說明</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ⓐ 虎航去＋虎航回（最便宜）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/28 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">四 虎航 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">14:35</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">二 虎航 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">19:40</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">最便宜；但去程下午、回程 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">23:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">落地</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Ⓑ 虎航去＋長榮回（推薦）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">二 長榮 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">16:15</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">請假 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">19:30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">落地，可以搭捷運回家</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Ⓒ 星宇去＋長榮回</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/28 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">四 星宇 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">11:50</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">兩段都含行李，去程比較早</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ⓓ 星宇去＋虎航回（早去）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/27 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">三 星宇 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">11:50</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">多請 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天，換到便宜的早一點出發</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Ⓔ 長榮去＋長榮回（早去）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/27 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">三 長榮 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10:15</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">最早抵達、全程含行李，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">天 </t>
     </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">夜</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Ⓕ 星宇去＋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/31 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">商務艙回</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/31 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日 長榮商務 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">16:15</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">維持原本日期，但回程只剩商務艙</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Ⓑ 行程：</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/28 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">四 – </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/2 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">二（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">夜，請假 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/28</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/29</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/1</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/2</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">住宿</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">虎航 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">14:35 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">桃園 → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18:45 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">仙台 → 仙台機場線到仙台站，晚餐吃牛舌</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">仙台</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">早上 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">JR </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">仙山線到山寺，爬雪中石階 → 山形 → 大石田 → 下午進銀山溫泉，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">16:45 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">拍瓦斯燈藍調時刻</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">♨ 銀山溫泉（已訂）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">清晨溫泉街拍照 → 大石田 → 山形 → 巴士到藏王溫泉，有點燈的話看樹冰夜景</t>
+  </si>
+  <si>
+    <t xml:space="preserve">藏王溫泉</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">早上搭纜車看樹冰 → 巴士到仙台（約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">小時）或在山形市區逛</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">仙台（或秋保、作並溫泉）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">松島遊覽船、瑞巖寺、烤牡蠣 → 下午回仙台逛一番町</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/2 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">二</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">仙台市區（仙台城跡、瑞鳳殿）→ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">14:30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">前往機場 → 長榮 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">16:15 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">起飛，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">19:30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">抵達桃園</t>
+    </r>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="13"/>
         <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5 </t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">定案行程：早去晚回 </t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="13"/>
         <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">夜（</t>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="13"/>
         <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2027/1/26 </t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天 </t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="13"/>
         <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">二 – </t>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="13"/>
         <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1/31 </t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">夜（</t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="13"/>
         <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">日，請假 </t>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2027/1/26 </t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="13"/>
         <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">二 – </t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="13"/>
         <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/31 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日，請假 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
@@ -3315,9 +4411,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">備註</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -5929,9 +7022,6 @@
     <t xml:space="preserve">機票</t>
   </si>
   <si>
-    <t xml:space="preserve">行李加購</t>
-  </si>
-  <si>
     <t xml:space="preserve">額外陸路（日圓）</t>
   </si>
   <si>
@@ -5944,9 +7034,6 @@
     <t xml:space="preserve">單程到銀山</t>
   </si>
   <si>
-    <t xml:space="preserve">說明</t>
-  </si>
-  <si>
     <t xml:space="preserve">★</t>
   </si>
   <si>
@@ -6771,9 +7858,6 @@
       </rPr>
       <t xml:space="preserve">¥1,200</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">藏王溫泉</t>
   </si>
   <si>
     <r>
@@ -8287,7 +9371,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -8433,6 +9517,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9133,6 +10225,183 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="90"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="B2" s="53" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>535</v>
+      </c>
+      <c r="B3" s="53" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="54" t="s">
+        <v>537</v>
+      </c>
+      <c r="B4" s="53" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="54" t="s">
+        <v>539</v>
+      </c>
+      <c r="B5" s="53" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="54" t="s">
+        <v>541</v>
+      </c>
+      <c r="B6" s="53" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="54" t="s">
+        <v>543</v>
+      </c>
+      <c r="B7" s="53" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="54" t="s">
+        <v>545</v>
+      </c>
+      <c r="B8" s="53" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>547</v>
+      </c>
+      <c r="B9" s="53" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="54" t="s">
+        <v>549</v>
+      </c>
+      <c r="B10" s="53" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="54" t="s">
+        <v>551</v>
+      </c>
+      <c r="B11" s="53" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="B12" s="53" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="B13" s="53" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>557</v>
+      </c>
+      <c r="B14" s="53" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>559</v>
+      </c>
+      <c r="B15" s="53" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>561</v>
+      </c>
+      <c r="B16" s="53" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="B17" s="53" t="s">
+        <v>564</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="https://www.starlux-airlines.com/flights/en/flights-from-taipei-to-sendai"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://flights.evaair.com/en/flights-from-taipei-to-sendai"/>
+    <hyperlink ref="B4" r:id="rId3" display="https://www.google.com/travel/flights/flights-from-taipei-city-to-sendai.html"/>
+    <hyperlink ref="B5" r:id="rId4" display="https://www.hotelscombined.com.tw/flight-routes/Taipei-City-Taiwan-Taoyuan-Intl-TPE/Sendai-SDJ.ksp"/>
+    <hyperlink ref="B6" r:id="rId5" display="https://www.skyscanner.com.tw/flights/airline-flights-to-airport/sdj/eva-air-br/cheap-flights-with-eva-air-br-flights-to-sendai"/>
+    <hyperlink ref="B7" r:id="rId6" display="https://www.trip.com/flights/airport-tsa-hnd/"/>
+    <hyperlink ref="B8" r:id="rId7" display="https://www.expedia.com.tw/en/lp/flights/tsa/hnd/taipei-to-tokyo"/>
+    <hyperlink ref="B9" r:id="rId8" display="https://www.haneda-tokyo.com/schedule/hnd-tsa-schedule.html"/>
+    <hyperlink ref="B10" r:id="rId9" display="https://www.hotelscombined.com.tw/flight-routes/Taipei-City-Taiwan-Taoyuan-Intl-TPE/Tokyo-Haneda-HND.ksp"/>
+    <hyperlink ref="B11" r:id="rId10" display="https://www.tw.kayak.com/%E8%88%AA%E7%8F%AD/%E5%8F%B0%E5%8C%97-TW1/%E6%9D%B1%E4%BA%AC-%E6%88%90%E7%94%B0%E5%9C%8B%E9%9A%9B%E6%A9%9F%E5%A0%B4-NRT"/>
+    <hyperlink ref="B12" r:id="rId11" display="https://www.tigerairtw.com/zh-tw/ready-to-go/fees"/>
+    <hyperlink ref="B13" r:id="rId12" display="https://ekitan.com/transit/shinkansen/section/sf-2590/st-737"/>
+    <hyperlink ref="B14" r:id="rId13" display="https://tohoku.letsgojp.com/archives/739243/"/>
+    <hyperlink ref="B15" r:id="rId14" display="https://travel.yamakobus.jp/zh-tw/timetable/routebus-yamagata-zaoline.html"/>
+    <hyperlink ref="B16" r:id="rId15" display="https://twoslowbyron.com/zao_ropeway/"/>
+    <hyperlink ref="B17" r:id="rId16" display="https://mimigo.tw/ginzan-onsen/"/>
+  </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -10555,6 +11824,847 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:I42"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="25" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="22" t="s">
+        <v>201</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="24" t="n">
+        <v>44798</v>
+      </c>
+      <c r="F5" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G5" s="23" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="22" t="s">
+        <v>203</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" s="24" t="n">
+        <v>44374</v>
+      </c>
+      <c r="F6" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G6" s="23" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>15599</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" s="16"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>27591</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="16"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="22" t="s">
+        <v>205</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="E9" s="24"/>
+      <c r="F9" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="G9" s="23" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>15599</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G10" s="16"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <v>22784</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>25171</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G12" s="16" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>15733</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="16" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" s="21" t="n">
+        <v>17781</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" s="21" t="n">
+        <v>14099</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G15" s="16" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" s="21" t="n">
+        <v>22784</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G16" s="16" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E17" s="24" t="n">
+        <v>44798</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G17" s="23" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" s="24"/>
+      <c r="F18" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="G18" s="23" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E19" s="24" t="n">
+        <v>33029</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G19" s="23" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="E20" s="24" t="n">
+        <v>34301</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G20" s="23" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="B21" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="E21" s="24" t="n">
+        <v>34301</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G21" s="23" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="E22" s="21" t="n">
+        <v>16466</v>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G22" s="16" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="E23" s="21" t="n">
+        <v>20549</v>
+      </c>
+      <c r="F23" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G23" s="16" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="B24" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="D24" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="E24" s="24"/>
+      <c r="F24" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="G24" s="23" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="33" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="H27" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="16" t="s">
+        <v>218</v>
+      </c>
+      <c r="B28" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" s="20" t="s">
+        <v>219</v>
+      </c>
+      <c r="D28" s="21" t="n">
+        <v>14099</v>
+      </c>
+      <c r="E28" s="20" t="s">
+        <v>220</v>
+      </c>
+      <c r="F28" s="21" t="n">
+        <v>16466</v>
+      </c>
+      <c r="G28" s="21" t="n">
+        <v>1900</v>
+      </c>
+      <c r="H28" s="32" t="n">
+        <f aca="false">D28+F28+G28</f>
+        <v>32465</v>
+      </c>
+      <c r="I28" s="16" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="26" t="s">
+        <v>222</v>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" s="27" t="s">
+        <v>219</v>
+      </c>
+      <c r="D29" s="28" t="n">
+        <v>14099</v>
+      </c>
+      <c r="E29" s="27" t="s">
+        <v>223</v>
+      </c>
+      <c r="F29" s="28" t="n">
+        <v>20549</v>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>950</v>
+      </c>
+      <c r="H29" s="30" t="n">
+        <f aca="false">D29+F29+G29</f>
+        <v>35598</v>
+      </c>
+      <c r="I29" s="12" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="16" t="s">
+        <v>225</v>
+      </c>
+      <c r="B30" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>226</v>
+      </c>
+      <c r="D30" s="21" t="n">
+        <v>22784</v>
+      </c>
+      <c r="E30" s="20" t="s">
+        <v>223</v>
+      </c>
+      <c r="F30" s="21" t="n">
+        <v>20549</v>
+      </c>
+      <c r="G30" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="32" t="n">
+        <f aca="false">D30+F30+G30</f>
+        <v>43333</v>
+      </c>
+      <c r="I30" s="16" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="16" t="s">
+        <v>228</v>
+      </c>
+      <c r="B31" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="D31" s="21" t="n">
+        <v>15733</v>
+      </c>
+      <c r="E31" s="20" t="s">
+        <v>220</v>
+      </c>
+      <c r="F31" s="21" t="n">
+        <v>16466</v>
+      </c>
+      <c r="G31" s="21" t="n">
+        <v>950</v>
+      </c>
+      <c r="H31" s="32" t="n">
+        <f aca="false">D31+F31+G31</f>
+        <v>33149</v>
+      </c>
+      <c r="I31" s="16" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="16" t="s">
+        <v>231</v>
+      </c>
+      <c r="B32" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" s="20" t="s">
+        <v>232</v>
+      </c>
+      <c r="D32" s="21" t="n">
+        <v>17781</v>
+      </c>
+      <c r="E32" s="20" t="s">
+        <v>223</v>
+      </c>
+      <c r="F32" s="21" t="n">
+        <v>20549</v>
+      </c>
+      <c r="G32" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="32" t="n">
+        <f aca="false">D32+F32+G32</f>
+        <v>38330</v>
+      </c>
+      <c r="I32" s="16" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="16" t="s">
+        <v>234</v>
+      </c>
+      <c r="B33" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C33" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="D33" s="21" t="n">
+        <v>15733</v>
+      </c>
+      <c r="E33" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="F33" s="21" t="n">
+        <v>33029</v>
+      </c>
+      <c r="G33" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="32" t="n">
+        <f aca="false">D33+F33+G33</f>
+        <v>48762</v>
+      </c>
+      <c r="I33" s="16" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="33" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="37" t="s">
+        <v>154</v>
+      </c>
+      <c r="B37" s="16" t="s">
+        <v>239</v>
+      </c>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="16" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="38" t="s">
+        <v>165</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="12" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="37" t="s">
+        <v>173</v>
+      </c>
+      <c r="B39" s="16" t="s">
+        <v>243</v>
+      </c>
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="16"/>
+      <c r="F39" s="16"/>
+      <c r="G39" s="16" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="37" t="s">
+        <v>183</v>
+      </c>
+      <c r="B40" s="16" t="s">
+        <v>245</v>
+      </c>
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="16"/>
+      <c r="F40" s="16"/>
+      <c r="G40" s="16" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="37" t="s">
+        <v>187</v>
+      </c>
+      <c r="B41" s="16" t="s">
+        <v>247</v>
+      </c>
+      <c r="C41" s="16"/>
+      <c r="D41" s="16"/>
+      <c r="E41" s="16"/>
+      <c r="F41" s="16"/>
+      <c r="G41" s="16" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="37" t="s">
+        <v>248</v>
+      </c>
+      <c r="B42" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="C42" s="16"/>
+      <c r="D42" s="16"/>
+      <c r="E42" s="16"/>
+      <c r="F42" s="16"/>
+      <c r="G42" s="20" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="B41:F41"/>
+    <mergeCell ref="B42:F42"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:E48"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -10567,12 +12677,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>197</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>198</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10589,39 +12699,39 @@
         <v>137</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="34" t="s">
-        <v>200</v>
+        <v>252</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>201</v>
+        <v>253</v>
       </c>
       <c r="C5" s="36" t="s">
-        <v>202</v>
+        <v>254</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>203</v>
+        <v>255</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>204</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16"/>
       <c r="B6" s="20" t="s">
-        <v>205</v>
+        <v>257</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>206</v>
+        <v>258</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>207</v>
+        <v>259</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>208</v>
+        <v>260</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10630,67 +12740,67 @@
         <v>147</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>209</v>
+        <v>261</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16" t="s">
-        <v>210</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16"/>
       <c r="B8" s="20" t="s">
-        <v>211</v>
+        <v>263</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>212</v>
+        <v>264</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>213</v>
+        <v>265</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>214</v>
+        <v>266</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16"/>
       <c r="B9" s="20" t="s">
-        <v>215</v>
+        <v>267</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>216</v>
+        <v>268</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16" t="s">
-        <v>217</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16"/>
       <c r="B10" s="20" t="s">
-        <v>218</v>
+        <v>270</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>219</v>
+        <v>271</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>220</v>
+        <v>272</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>221</v>
+        <v>273</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16"/>
       <c r="B11" s="20" t="s">
-        <v>222</v>
+        <v>274</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>223</v>
+        <v>275</v>
       </c>
       <c r="D11" s="16"/>
       <c r="E11" s="16" t="s">
-        <v>224</v>
+        <v>276</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10701,35 +12811,35 @@
         <v>155</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>225</v>
+        <v>277</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>226</v>
+        <v>278</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>227</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16"/>
       <c r="B13" s="20" t="s">
-        <v>228</v>
+        <v>280</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>229</v>
+        <v>281</v>
       </c>
       <c r="D13" s="16"/>
       <c r="E13" s="16" t="s">
-        <v>230</v>
+        <v>282</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16"/>
       <c r="B14" s="20" t="s">
-        <v>231</v>
+        <v>283</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>232</v>
+        <v>284</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
@@ -10737,20 +12847,20 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16"/>
       <c r="B15" s="20" t="s">
-        <v>233</v>
+        <v>285</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>234</v>
+        <v>286</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>235</v>
+        <v>287</v>
       </c>
       <c r="E15" s="16"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16"/>
       <c r="B16" s="20" t="s">
-        <v>215</v>
+        <v>267</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>151</v>
@@ -10759,7 +12869,7 @@
         <v>152</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>236</v>
+        <v>288</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10768,26 +12878,26 @@
         <v>180</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>237</v>
+        <v>289</v>
       </c>
       <c r="D17" s="16"/>
       <c r="E17" s="16" t="s">
-        <v>238</v>
+        <v>290</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16"/>
       <c r="B18" s="20" t="s">
-        <v>222</v>
+        <v>274</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>239</v>
+        <v>291</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>240</v>
+        <v>292</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>241</v>
+        <v>293</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10798,22 +12908,22 @@
         <v>155</v>
       </c>
       <c r="C19" s="36" t="s">
-        <v>242</v>
+        <v>294</v>
       </c>
       <c r="D19" s="36" t="s">
-        <v>243</v>
+        <v>295</v>
       </c>
       <c r="E19" s="36" t="s">
-        <v>244</v>
+        <v>296</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16"/>
       <c r="B20" s="20" t="s">
-        <v>231</v>
+        <v>283</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>245</v>
+        <v>297</v>
       </c>
       <c r="D20" s="16"/>
       <c r="E20" s="16"/>
@@ -10821,10 +12931,10 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16"/>
       <c r="B21" s="20" t="s">
-        <v>246</v>
+        <v>298</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>247</v>
+        <v>299</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>152</v>
@@ -10834,25 +12944,25 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16"/>
       <c r="B22" s="20" t="s">
-        <v>218</v>
+        <v>270</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>248</v>
+        <v>300</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>249</v>
+        <v>301</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>250</v>
+        <v>302</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="16"/>
       <c r="B23" s="20" t="s">
-        <v>222</v>
+        <v>274</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>251</v>
+        <v>303</v>
       </c>
       <c r="D23" s="16"/>
       <c r="E23" s="16" t="s">
@@ -10864,77 +12974,77 @@
         <v>165</v>
       </c>
       <c r="B24" s="35" t="s">
-        <v>252</v>
+        <v>304</v>
       </c>
       <c r="C24" s="36" t="s">
-        <v>253</v>
+        <v>305</v>
       </c>
       <c r="D24" s="36"/>
       <c r="E24" s="36" t="s">
-        <v>254</v>
+        <v>306</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16"/>
       <c r="B25" s="20" t="s">
-        <v>255</v>
+        <v>307</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>167</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>256</v>
+        <v>308</v>
       </c>
       <c r="E25" s="16"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16"/>
       <c r="B26" s="20" t="s">
-        <v>246</v>
+        <v>298</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>257</v>
+        <v>309</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>258</v>
+        <v>310</v>
       </c>
       <c r="E26" s="16" t="s">
-        <v>259</v>
+        <v>311</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12"/>
       <c r="B27" s="27" t="s">
-        <v>218</v>
+        <v>270</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>260</v>
+        <v>312</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="12" t="s">
-        <v>261</v>
+        <v>313</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16"/>
       <c r="B28" s="20" t="s">
-        <v>262</v>
+        <v>314</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>263</v>
+        <v>315</v>
       </c>
       <c r="D28" s="16"/>
       <c r="E28" s="16" t="s">
-        <v>264</v>
+        <v>316</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16"/>
       <c r="B29" s="20" t="s">
-        <v>265</v>
+        <v>317</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>266</v>
+        <v>318</v>
       </c>
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
@@ -10942,14 +13052,14 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16"/>
       <c r="B30" s="20" t="s">
-        <v>267</v>
+        <v>319</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>268</v>
+        <v>320</v>
       </c>
       <c r="D30" s="16"/>
       <c r="E30" s="16" t="s">
-        <v>269</v>
+        <v>321</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10964,16 +13074,16 @@
       </c>
       <c r="D31" s="36"/>
       <c r="E31" s="36" t="s">
-        <v>270</v>
+        <v>322</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16"/>
       <c r="B32" s="20" t="s">
-        <v>271</v>
+        <v>323</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>272</v>
+        <v>324</v>
       </c>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
@@ -10981,38 +13091,38 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16"/>
       <c r="B33" s="20" t="s">
-        <v>273</v>
+        <v>325</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>274</v>
+        <v>326</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>275</v>
+        <v>327</v>
       </c>
       <c r="E33" s="16"/>
     </row>
     <row r="34" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="16"/>
       <c r="B34" s="20" t="s">
-        <v>276</v>
+        <v>328</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>277</v>
+        <v>329</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>278</v>
+        <v>330</v>
       </c>
       <c r="E34" s="16" t="s">
-        <v>279</v>
+        <v>331</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16"/>
       <c r="B35" s="20" t="s">
-        <v>215</v>
+        <v>267</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>280</v>
+        <v>332</v>
       </c>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
@@ -11020,27 +13130,27 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16"/>
       <c r="B36" s="20" t="s">
-        <v>218</v>
+        <v>270</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>281</v>
+        <v>333</v>
       </c>
       <c r="D36" s="16"/>
       <c r="E36" s="16" t="s">
-        <v>282</v>
+        <v>334</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16"/>
       <c r="B37" s="20" t="s">
-        <v>265</v>
+        <v>317</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>283</v>
+        <v>335</v>
       </c>
       <c r="D37" s="16"/>
       <c r="E37" s="16" t="s">
-        <v>284</v>
+        <v>336</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11048,10 +13158,10 @@
         <v>183</v>
       </c>
       <c r="B38" s="35" t="s">
-        <v>271</v>
+        <v>323</v>
       </c>
       <c r="C38" s="36" t="s">
-        <v>285</v>
+        <v>337</v>
       </c>
       <c r="D38" s="36"/>
       <c r="E38" s="36"/>
@@ -11062,23 +13172,23 @@
         <v>155</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>286</v>
+        <v>338</v>
       </c>
       <c r="D39" s="20" t="s">
-        <v>287</v>
+        <v>339</v>
       </c>
       <c r="E39" s="16"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16"/>
       <c r="B40" s="20" t="s">
-        <v>288</v>
+        <v>340</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>289</v>
+        <v>341</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>290</v>
+        <v>342</v>
       </c>
       <c r="E40" s="16"/>
     </row>
@@ -11088,85 +13198,85 @@
         <v>166</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>291</v>
+        <v>343</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>292</v>
+        <v>344</v>
       </c>
       <c r="E41" s="16"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="16"/>
       <c r="B42" s="20" t="s">
-        <v>231</v>
+        <v>283</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>293</v>
+        <v>345</v>
       </c>
       <c r="D42" s="16"/>
       <c r="E42" s="16" t="s">
-        <v>294</v>
+        <v>346</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="16"/>
       <c r="B43" s="20" t="s">
-        <v>246</v>
+        <v>298</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>295</v>
+        <v>347</v>
       </c>
       <c r="D43" s="20" t="s">
-        <v>287</v>
+        <v>339</v>
       </c>
       <c r="E43" s="16"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="16"/>
       <c r="B44" s="20" t="s">
-        <v>296</v>
+        <v>348</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>297</v>
+        <v>349</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>213</v>
+        <v>265</v>
       </c>
       <c r="E44" s="16" t="s">
-        <v>298</v>
+        <v>350</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="16"/>
       <c r="B45" s="20" t="s">
-        <v>299</v>
+        <v>351</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>300</v>
+        <v>352</v>
       </c>
       <c r="D45" s="16"/>
       <c r="E45" s="16" t="s">
-        <v>301</v>
+        <v>353</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="16"/>
       <c r="B46" s="20" t="s">
-        <v>302</v>
+        <v>354</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>303</v>
+        <v>355</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>304</v>
+        <v>356</v>
       </c>
       <c r="E46" s="16" t="s">
-        <v>305</v>
+        <v>357</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>306</v>
+        <v>358</v>
       </c>
     </row>
   </sheetData>
@@ -11180,7 +13290,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -11204,17 +13314,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>307</v>
+        <v>359</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>308</v>
+        <v>360</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>309</v>
+        <v>361</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>29</v>
@@ -11223,66 +13333,66 @@
         <v>30</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>310</v>
+        <v>362</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>311</v>
+        <v>363</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>312</v>
+        <v>364</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>313</v>
+        <v>365</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>314</v>
+        <v>366</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>315</v>
+        <v>367</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>316</v>
+        <v>368</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>317</v>
+        <v>369</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>318</v>
+        <v>370</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>319</v>
+        <v>371</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>320</v>
+        <v>372</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>321</v>
+        <v>373</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>322</v>
+        <v>374</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>323</v>
+        <v>375</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>324</v>
+        <v>376</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>44</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>325</v>
+        <v>377</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>326</v>
+        <v>378</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>327</v>
+        <v>379</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>328</v>
+        <v>380</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>4743</v>
@@ -11290,8 +13400,8 @@
       <c r="I5" s="21" t="n">
         <v>9676</v>
       </c>
-      <c r="J5" s="37"/>
-      <c r="K5" s="37"/>
+      <c r="J5" s="39"/>
+      <c r="K5" s="39"/>
       <c r="L5" s="32" t="n">
         <f aca="false">IF(J5&gt;0,J5,H5)</f>
         <v>4743</v>
@@ -11301,36 +13411,36 @@
         <v>9676</v>
       </c>
       <c r="N5" s="16" t="s">
-        <v>329</v>
+        <v>381</v>
       </c>
       <c r="O5" s="21" t="n">
         <v>950</v>
       </c>
       <c r="P5" s="16" t="s">
-        <v>330</v>
+        <v>382</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>331</v>
+        <v>383</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>324</v>
+        <v>376</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>37</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>332</v>
+        <v>384</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>333</v>
+        <v>385</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>334</v>
+        <v>386</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>335</v>
+        <v>387</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>9845</v>
@@ -11338,8 +13448,8 @@
       <c r="I6" s="21" t="n">
         <v>17878</v>
       </c>
-      <c r="J6" s="37"/>
-      <c r="K6" s="37"/>
+      <c r="J6" s="39"/>
+      <c r="K6" s="39"/>
       <c r="L6" s="32" t="n">
         <f aca="false">IF(J6&gt;0,J6,H6)</f>
         <v>9845</v>
@@ -11349,36 +13459,36 @@
         <v>17878</v>
       </c>
       <c r="N6" s="16" t="s">
-        <v>336</v>
+        <v>388</v>
       </c>
       <c r="O6" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P6" s="16" t="s">
-        <v>337</v>
+        <v>389</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>338</v>
+        <v>390</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>324</v>
+        <v>376</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>41</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>339</v>
+        <v>391</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>340</v>
+        <v>392</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>341</v>
+        <v>393</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>342</v>
+        <v>394</v>
       </c>
       <c r="H7" s="21" t="n">
         <v>9720</v>
@@ -11386,8 +13496,8 @@
       <c r="I7" s="21" t="n">
         <v>19586</v>
       </c>
-      <c r="J7" s="37"/>
-      <c r="K7" s="37"/>
+      <c r="J7" s="39"/>
+      <c r="K7" s="39"/>
       <c r="L7" s="32" t="n">
         <f aca="false">IF(J7&gt;0,J7,H7)</f>
         <v>9720</v>
@@ -11397,36 +13507,36 @@
         <v>19586</v>
       </c>
       <c r="N7" s="16" t="s">
-        <v>336</v>
+        <v>388</v>
       </c>
       <c r="O7" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P7" s="16" t="s">
-        <v>343</v>
+        <v>395</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>344</v>
+        <v>396</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>345</v>
+        <v>397</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>37</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>346</v>
+        <v>398</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>347</v>
+        <v>399</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>348</v>
+        <v>400</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>342</v>
+        <v>394</v>
       </c>
       <c r="H8" s="21" t="n">
         <v>10361</v>
@@ -11434,8 +13544,8 @@
       <c r="I8" s="21" t="n">
         <v>16526</v>
       </c>
-      <c r="J8" s="37"/>
-      <c r="K8" s="37"/>
+      <c r="J8" s="39"/>
+      <c r="K8" s="39"/>
       <c r="L8" s="32" t="n">
         <f aca="false">IF(J8&gt;0,J8,H8)</f>
         <v>10361</v>
@@ -11445,36 +13555,36 @@
         <v>16526</v>
       </c>
       <c r="N8" s="16" t="s">
-        <v>336</v>
+        <v>388</v>
       </c>
       <c r="O8" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P8" s="16" t="s">
-        <v>349</v>
+        <v>401</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>350</v>
+        <v>402</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>345</v>
+        <v>397</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>351</v>
+        <v>403</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>352</v>
+        <v>404</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>353</v>
+        <v>405</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>348</v>
+        <v>400</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>342</v>
+        <v>394</v>
       </c>
       <c r="H9" s="21" t="n">
         <v>10361</v>
@@ -11482,8 +13592,8 @@
       <c r="I9" s="21" t="n">
         <v>16526</v>
       </c>
-      <c r="J9" s="37"/>
-      <c r="K9" s="37"/>
+      <c r="J9" s="39"/>
+      <c r="K9" s="39"/>
       <c r="L9" s="32" t="n">
         <f aca="false">IF(J9&gt;0,J9,H9)</f>
         <v>10361</v>
@@ -11493,36 +13603,36 @@
         <v>16526</v>
       </c>
       <c r="N9" s="16" t="s">
-        <v>336</v>
+        <v>388</v>
       </c>
       <c r="O9" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P9" s="16" t="s">
-        <v>354</v>
+        <v>406</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>355</v>
+        <v>407</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>345</v>
+        <v>397</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>356</v>
+        <v>408</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>357</v>
+        <v>409</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>358</v>
+        <v>410</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>348</v>
+        <v>400</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>342</v>
+        <v>394</v>
       </c>
       <c r="H10" s="21" t="n">
         <v>10361</v>
@@ -11530,8 +13640,8 @@
       <c r="I10" s="21" t="n">
         <v>16526</v>
       </c>
-      <c r="J10" s="37"/>
-      <c r="K10" s="37"/>
+      <c r="J10" s="39"/>
+      <c r="K10" s="39"/>
       <c r="L10" s="32" t="n">
         <f aca="false">IF(J10&gt;0,J10,H10)</f>
         <v>10361</v>
@@ -11541,36 +13651,36 @@
         <v>16526</v>
       </c>
       <c r="N10" s="16" t="s">
-        <v>336</v>
+        <v>388</v>
       </c>
       <c r="O10" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P10" s="16" t="s">
-        <v>354</v>
+        <v>406</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>359</v>
+        <v>411</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>345</v>
+        <v>397</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>360</v>
+        <v>412</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>361</v>
+        <v>413</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>362</v>
+        <v>414</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>348</v>
+        <v>400</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>342</v>
+        <v>394</v>
       </c>
       <c r="H11" s="21" t="n">
         <v>10361</v>
@@ -11578,8 +13688,8 @@
       <c r="I11" s="21" t="n">
         <v>16526</v>
       </c>
-      <c r="J11" s="37"/>
-      <c r="K11" s="37"/>
+      <c r="J11" s="39"/>
+      <c r="K11" s="39"/>
       <c r="L11" s="32" t="n">
         <f aca="false">IF(J11&gt;0,J11,H11)</f>
         <v>10361</v>
@@ -11589,36 +13699,36 @@
         <v>16526</v>
       </c>
       <c r="N11" s="16" t="s">
-        <v>336</v>
+        <v>388</v>
       </c>
       <c r="O11" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P11" s="16" t="s">
-        <v>354</v>
+        <v>406</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>363</v>
+        <v>415</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>364</v>
+        <v>416</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>93</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>365</v>
+        <v>417</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>366</v>
+        <v>418</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>366</v>
+        <v>418</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>342</v>
+        <v>394</v>
       </c>
       <c r="H12" s="21" t="n">
         <v>5386</v>
@@ -11627,8 +13737,8 @@
         <f aca="false">H12*2</f>
         <v>10772</v>
       </c>
-      <c r="J12" s="37"/>
-      <c r="K12" s="37"/>
+      <c r="J12" s="39"/>
+      <c r="K12" s="39"/>
       <c r="L12" s="32" t="n">
         <f aca="false">IF(J12&gt;0,J12,H12)</f>
         <v>5386</v>
@@ -11638,36 +13748,36 @@
         <v>10772</v>
       </c>
       <c r="N12" s="16" t="s">
-        <v>329</v>
+        <v>381</v>
       </c>
       <c r="O12" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="P12" s="16" t="s">
-        <v>367</v>
+        <v>419</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>368</v>
+        <v>420</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>369</v>
+        <v>421</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>370</v>
+        <v>422</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>371</v>
+        <v>423</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>366</v>
+        <v>418</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>366</v>
+        <v>418</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>342</v>
+        <v>394</v>
       </c>
       <c r="H13" s="21" t="n">
         <v>3748</v>
@@ -11676,8 +13786,8 @@
         <f aca="false">H13*2</f>
         <v>7496</v>
       </c>
-      <c r="J13" s="37"/>
-      <c r="K13" s="37"/>
+      <c r="J13" s="39"/>
+      <c r="K13" s="39"/>
       <c r="L13" s="32" t="n">
         <f aca="false">IF(J13&gt;0,J13,H13)</f>
         <v>3748</v>
@@ -11687,36 +13797,36 @@
         <v>7496</v>
       </c>
       <c r="N13" s="16" t="s">
-        <v>329</v>
+        <v>381</v>
       </c>
       <c r="O13" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="P13" s="16" t="s">
-        <v>372</v>
+        <v>424</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>373</v>
+        <v>425</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>364</v>
+        <v>416</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>44</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>374</v>
+        <v>426</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>366</v>
+        <v>418</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>366</v>
+        <v>418</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>342</v>
+        <v>394</v>
       </c>
       <c r="H14" s="21" t="n">
         <v>6702</v>
@@ -11725,8 +13835,8 @@
         <f aca="false">H14*2</f>
         <v>13404</v>
       </c>
-      <c r="J14" s="37"/>
-      <c r="K14" s="37"/>
+      <c r="J14" s="39"/>
+      <c r="K14" s="39"/>
       <c r="L14" s="32" t="n">
         <f aca="false">IF(J14&gt;0,J14,H14)</f>
         <v>6702</v>
@@ -11736,18 +13846,18 @@
         <v>13404</v>
       </c>
       <c r="N14" s="16" t="s">
-        <v>329</v>
+        <v>381</v>
       </c>
       <c r="O14" s="21" t="n">
         <v>950</v>
       </c>
       <c r="P14" s="16" t="s">
-        <v>375</v>
+        <v>427</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>376</v>
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -11761,7 +13871,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -11784,17 +13894,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>377</v>
+        <v>429</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>378</v>
+        <v>430</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>379</v>
+        <v>431</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>10</v>
@@ -11812,45 +13922,45 @@
         <v>107</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>380</v>
+        <v>432</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>381</v>
+        <v>215</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>382</v>
+        <v>433</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>383</v>
+        <v>434</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>384</v>
+        <v>435</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>385</v>
+        <v>436</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>386</v>
+        <v>217</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>387</v>
+        <v>437</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>388</v>
+        <v>438</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>389</v>
-      </c>
-      <c r="D5" s="38" t="n">
+        <v>439</v>
+      </c>
+      <c r="D5" s="40" t="n">
         <v>4</v>
       </c>
       <c r="E5" s="27" t="s">
-        <v>390</v>
+        <v>440</v>
       </c>
       <c r="F5" s="27" t="s">
-        <v>391</v>
+        <v>441</v>
       </c>
       <c r="G5" s="11" t="n">
         <f aca="false">機票價格!L6+機票價格!L5</f>
@@ -11872,30 +13982,30 @@
         <v>15538</v>
       </c>
       <c r="L5" s="27" t="s">
-        <v>392</v>
+        <v>442</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>393</v>
+        <v>443</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>394</v>
+        <v>444</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>395</v>
+        <v>445</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="D6" s="39" t="n">
+        <v>439</v>
+      </c>
+      <c r="D6" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>396</v>
+        <v>446</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>397</v>
+        <v>447</v>
       </c>
       <c r="G6" s="15" t="n">
         <f aca="false">機票價格!M5</f>
@@ -11917,30 +14027,30 @@
         <v>11576</v>
       </c>
       <c r="L6" s="20" t="s">
-        <v>392</v>
+        <v>442</v>
       </c>
       <c r="M6" s="16" t="s">
-        <v>398</v>
+        <v>448</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>399</v>
+        <v>449</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>401</v>
-      </c>
-      <c r="D7" s="39" t="n">
+        <v>451</v>
+      </c>
+      <c r="D7" s="41" t="n">
         <v>3</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>402</v>
+        <v>452</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>397</v>
+        <v>447</v>
       </c>
       <c r="G7" s="15" t="n">
         <f aca="false">機票價格!L6+機票價格!L5</f>
@@ -11962,30 +14072,30 @@
         <v>15538</v>
       </c>
       <c r="L7" s="20" t="s">
-        <v>392</v>
+        <v>442</v>
       </c>
       <c r="M7" s="16" t="s">
-        <v>403</v>
+        <v>453</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>404</v>
+        <v>454</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>405</v>
+        <v>455</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>401</v>
-      </c>
-      <c r="D8" s="39" t="n">
+        <v>451</v>
+      </c>
+      <c r="D8" s="41" t="n">
         <v>3</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>406</v>
+        <v>456</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>407</v>
+        <v>457</v>
       </c>
       <c r="G8" s="15" t="n">
         <f aca="false">機票價格!M7</f>
@@ -12007,30 +14117,30 @@
         <v>19586</v>
       </c>
       <c r="L8" s="20" t="s">
-        <v>392</v>
+        <v>442</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>408</v>
+        <v>458</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>409</v>
+        <v>459</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>410</v>
+        <v>460</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="D9" s="39" t="n">
+        <v>439</v>
+      </c>
+      <c r="D9" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>411</v>
+        <v>461</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>412</v>
+        <v>462</v>
       </c>
       <c r="G9" s="15" t="n">
         <f aca="false">機票價格!M8</f>
@@ -12053,30 +14163,30 @@
         <v>21379.1</v>
       </c>
       <c r="L9" s="20" t="s">
-        <v>413</v>
+        <v>463</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>414</v>
+        <v>464</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>415</v>
+        <v>465</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>416</v>
+        <v>466</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="D10" s="39" t="n">
+        <v>439</v>
+      </c>
+      <c r="D10" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>396</v>
+        <v>446</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>412</v>
+        <v>462</v>
       </c>
       <c r="G10" s="15" t="n">
         <f aca="false">機票價格!L5+機票價格!L8</f>
@@ -12099,30 +14209,30 @@
         <v>18303.1</v>
       </c>
       <c r="L10" s="20" t="s">
-        <v>392</v>
+        <v>442</v>
       </c>
       <c r="M10" s="16" t="s">
-        <v>417</v>
+        <v>467</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>418</v>
+        <v>468</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>419</v>
+        <v>469</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>389</v>
-      </c>
-      <c r="D11" s="39" t="n">
+        <v>439</v>
+      </c>
+      <c r="D11" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>420</v>
+        <v>470</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>421</v>
+        <v>471</v>
       </c>
       <c r="G11" s="15" t="n">
         <f aca="false">機票價格!M12</f>
@@ -12145,15 +14255,15 @@
         <v>17625.1</v>
       </c>
       <c r="L11" s="20" t="s">
-        <v>413</v>
+        <v>463</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>422</v>
+        <v>472</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>423</v>
+        <v>473</v>
       </c>
       <c r="C13" s="3" t="str">
         <f aca="false">INDEX(B5:B11,MATCH(MIN(K5:K11),K5:K11,0))</f>
@@ -12175,7 +14285,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -12196,12 +14306,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>424</v>
+        <v>474</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>425</v>
+        <v>475</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12212,28 +14322,28 @@
         <v>136</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>426</v>
+        <v>476</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>427</v>
+        <v>477</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>428</v>
+        <v>478</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>429</v>
+        <v>479</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>430</v>
+        <v>480</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>431</v>
+        <v>481</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>432</v>
+        <v>482</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12241,16 +14351,16 @@
         <v>35</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>433</v>
+        <v>483</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>434</v>
+        <v>484</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>1310</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>435</v>
+        <v>485</v>
       </c>
       <c r="F5" s="31" t="n">
         <v>9000</v>
@@ -12258,7 +14368,7 @@
       <c r="G5" s="31" t="n">
         <v>570</v>
       </c>
-      <c r="H5" s="40" t="n">
+      <c r="H5" s="42" t="n">
         <f aca="false">D5+F5+G5</f>
         <v>10880</v>
       </c>
@@ -12266,8 +14376,8 @@
         <f aca="false">H5*總覽!$B$5</f>
         <v>2284.8</v>
       </c>
-      <c r="J5" s="41" t="s">
-        <v>436</v>
+      <c r="J5" s="43" t="s">
+        <v>486</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12275,16 +14385,16 @@
         <v>47</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>437</v>
+        <v>487</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>438</v>
+        <v>488</v>
       </c>
       <c r="D6" s="31" t="n">
         <v>2300</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>439</v>
+        <v>244</v>
       </c>
       <c r="F6" s="31" t="n">
         <v>20000</v>
@@ -12292,7 +14402,7 @@
       <c r="G6" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="40" t="n">
+      <c r="H6" s="42" t="n">
         <f aca="false">D6+F6+G6</f>
         <v>22300</v>
       </c>
@@ -12300,8 +14410,8 @@
         <f aca="false">H6*總覽!$B$5</f>
         <v>4683</v>
       </c>
-      <c r="J6" s="41" t="s">
-        <v>440</v>
+      <c r="J6" s="43" t="s">
+        <v>489</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12309,16 +14419,16 @@
         <v>49</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>441</v>
+        <v>490</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>442</v>
+        <v>491</v>
       </c>
       <c r="D7" s="31" t="n">
         <v>1200</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>443</v>
+        <v>492</v>
       </c>
       <c r="F7" s="31" t="n">
         <v>8000</v>
@@ -12326,7 +14436,7 @@
       <c r="G7" s="31" t="n">
         <v>4400</v>
       </c>
-      <c r="H7" s="40" t="n">
+      <c r="H7" s="42" t="n">
         <f aca="false">D7+F7+G7</f>
         <v>13600</v>
       </c>
@@ -12334,34 +14444,34 @@
         <f aca="false">H7*總覽!$B$5</f>
         <v>2856</v>
       </c>
-      <c r="J7" s="41" t="s">
-        <v>444</v>
+      <c r="J7" s="43" t="s">
+        <v>493</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>445</v>
+        <v>494</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>446</v>
+        <v>495</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>447</v>
+        <v>496</v>
       </c>
       <c r="D8" s="31" t="n">
         <v>1900</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>448</v>
-      </c>
-      <c r="F8" s="42" t="n">
+        <v>497</v>
+      </c>
+      <c r="F8" s="44" t="n">
         <f aca="false">總覽!B7</f>
         <v>0</v>
       </c>
       <c r="G8" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="40" t="n">
+      <c r="H8" s="42" t="n">
         <f aca="false">D8+F8+G8</f>
         <v>1900</v>
       </c>
@@ -12369,8 +14479,8 @@
         <f aca="false">H8*總覽!$B$5</f>
         <v>399</v>
       </c>
-      <c r="J8" s="43" t="s">
-        <v>449</v>
+      <c r="J8" s="45" t="s">
+        <v>498</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12378,16 +14488,16 @@
         <v>66</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>450</v>
+        <v>499</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>451</v>
+        <v>500</v>
       </c>
       <c r="D9" s="31" t="n">
         <v>2690</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>435</v>
+        <v>485</v>
       </c>
       <c r="F9" s="31" t="n">
         <v>9000</v>
@@ -12395,7 +14505,7 @@
       <c r="G9" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="40" t="n">
+      <c r="H9" s="42" t="n">
         <f aca="false">D9+F9+G9</f>
         <v>11690</v>
       </c>
@@ -12403,17 +14513,17 @@
         <f aca="false">H9*總覽!$B$5</f>
         <v>2454.9</v>
       </c>
-      <c r="J9" s="41"/>
+      <c r="J9" s="43"/>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>452</v>
+        <v>501</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>453</v>
+        <v>502</v>
       </c>
       <c r="D10" s="31" t="n">
         <v>1540</v>
@@ -12427,7 +14537,7 @@
       <c r="G10" s="31" t="n">
         <v>2200</v>
       </c>
-      <c r="H10" s="40" t="n">
+      <c r="H10" s="42" t="n">
         <f aca="false">D10+F10+G10</f>
         <v>3740</v>
       </c>
@@ -12435,34 +14545,34 @@
         <f aca="false">H10*總覽!$B$5</f>
         <v>785.4</v>
       </c>
-      <c r="J10" s="41" t="s">
-        <v>454</v>
+      <c r="J10" s="43" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="44" t="s">
+      <c r="A11" s="46" t="s">
         <v>25</v>
       </c>
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
-      <c r="D11" s="45" t="n">
+      <c r="D11" s="47" t="n">
         <f aca="false">SUM(D5:D10)</f>
         <v>10940</v>
       </c>
       <c r="E11" s="16"/>
-      <c r="F11" s="45" t="n">
+      <c r="F11" s="47" t="n">
         <f aca="false">SUM(F5:F10)</f>
         <v>46000</v>
       </c>
-      <c r="G11" s="45" t="n">
+      <c r="G11" s="47" t="n">
         <f aca="false">SUM(G5:G10)</f>
         <v>7170</v>
       </c>
-      <c r="H11" s="45" t="n">
+      <c r="H11" s="47" t="n">
         <f aca="false">SUM(H5:H10)</f>
         <v>64110</v>
       </c>
-      <c r="I11" s="46" t="n">
+      <c r="I11" s="48" t="n">
         <f aca="false">SUM(I5:I10)</f>
         <v>13463.1</v>
       </c>
@@ -12470,31 +14580,31 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>455</v>
-      </c>
-      <c r="H12" s="47" t="n">
+        <v>504</v>
+      </c>
+      <c r="H12" s="49" t="n">
         <v>5000</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>456</v>
+        <v>505</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>457</v>
-      </c>
-      <c r="H13" s="48" t="n">
+        <v>506</v>
+      </c>
+      <c r="H13" s="50" t="n">
         <f aca="false">H12*6</f>
         <v>30000</v>
       </c>
-      <c r="I13" s="49" t="n">
+      <c r="I13" s="51" t="n">
         <f aca="false">H13*總覽!$B$5</f>
         <v>6300</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>458</v>
+        <v>507</v>
       </c>
       <c r="I14" s="18" t="n">
         <f aca="false">I11+I13</f>
@@ -12512,7 +14622,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -12528,114 +14638,114 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>459</v>
+        <v>508</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>460</v>
+        <v>509</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>461</v>
+        <v>510</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>462</v>
+        <v>511</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>463</v>
-      </c>
-      <c r="C2" s="50" t="s">
-        <v>464</v>
+        <v>512</v>
+      </c>
+      <c r="C2" s="52" t="s">
+        <v>513</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>465</v>
+        <v>514</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>466</v>
+        <v>515</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>463</v>
-      </c>
-      <c r="C3" s="50" t="s">
-        <v>464</v>
+        <v>512</v>
+      </c>
+      <c r="C3" s="52" t="s">
+        <v>513</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>467</v>
+        <v>516</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>468</v>
+        <v>517</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>463</v>
-      </c>
-      <c r="C4" s="50" t="s">
-        <v>464</v>
+        <v>512</v>
+      </c>
+      <c r="C4" s="52" t="s">
+        <v>513</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>469</v>
+        <v>518</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>470</v>
+        <v>519</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>471</v>
-      </c>
-      <c r="C5" s="50" t="s">
-        <v>464</v>
+        <v>520</v>
+      </c>
+      <c r="C5" s="52" t="s">
+        <v>513</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>472</v>
+        <v>521</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>473</v>
+        <v>522</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>474</v>
-      </c>
-      <c r="C6" s="50" t="s">
-        <v>464</v>
+        <v>523</v>
+      </c>
+      <c r="C6" s="52" t="s">
+        <v>513</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>475</v>
+        <v>524</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>476</v>
+        <v>525</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>477</v>
-      </c>
-      <c r="C7" s="50" t="s">
-        <v>464</v>
+        <v>526</v>
+      </c>
+      <c r="C7" s="52" t="s">
+        <v>513</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>478</v>
+        <v>527</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>479</v>
+        <v>528</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>480</v>
-      </c>
-      <c r="C8" s="50" t="s">
-        <v>464</v>
+        <v>529</v>
+      </c>
+      <c r="C8" s="52" t="s">
+        <v>513</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>481</v>
+        <v>530</v>
       </c>
     </row>
   </sheetData>
@@ -12653,181 +14763,4 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:B17"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="90"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
-        <v>482</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
-        <v>484</v>
-      </c>
-      <c r="B2" s="51" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
-        <v>486</v>
-      </c>
-      <c r="B3" s="51" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="52" t="s">
-        <v>488</v>
-      </c>
-      <c r="B4" s="51" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="52" t="s">
-        <v>490</v>
-      </c>
-      <c r="B5" s="51" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="52" t="s">
-        <v>492</v>
-      </c>
-      <c r="B6" s="51" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="52" t="s">
-        <v>494</v>
-      </c>
-      <c r="B7" s="51" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="52" t="s">
-        <v>496</v>
-      </c>
-      <c r="B8" s="51" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>498</v>
-      </c>
-      <c r="B9" s="51" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="52" t="s">
-        <v>500</v>
-      </c>
-      <c r="B10" s="51" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="52" t="s">
-        <v>502</v>
-      </c>
-      <c r="B11" s="51" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>504</v>
-      </c>
-      <c r="B12" s="51" t="s">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>506</v>
-      </c>
-      <c r="B13" s="51" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>508</v>
-      </c>
-      <c r="B14" s="51" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>510</v>
-      </c>
-      <c r="B15" s="51" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>512</v>
-      </c>
-      <c r="B16" s="51" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>514</v>
-      </c>
-      <c r="B17" s="51" t="s">
-        <v>515</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="https://www.starlux-airlines.com/flights/en/flights-from-taipei-to-sendai"/>
-    <hyperlink ref="B3" r:id="rId2" display="https://flights.evaair.com/en/flights-from-taipei-to-sendai"/>
-    <hyperlink ref="B4" r:id="rId3" display="https://www.google.com/travel/flights/flights-from-taipei-city-to-sendai.html"/>
-    <hyperlink ref="B5" r:id="rId4" display="https://www.hotelscombined.com.tw/flight-routes/Taipei-City-Taiwan-Taoyuan-Intl-TPE/Sendai-SDJ.ksp"/>
-    <hyperlink ref="B6" r:id="rId5" display="https://www.skyscanner.com.tw/flights/airline-flights-to-airport/sdj/eva-air-br/cheap-flights-with-eva-air-br-flights-to-sendai"/>
-    <hyperlink ref="B7" r:id="rId6" display="https://www.trip.com/flights/airport-tsa-hnd/"/>
-    <hyperlink ref="B8" r:id="rId7" display="https://www.expedia.com.tw/en/lp/flights/tsa/hnd/taipei-to-tokyo"/>
-    <hyperlink ref="B9" r:id="rId8" display="https://www.haneda-tokyo.com/schedule/hnd-tsa-schedule.html"/>
-    <hyperlink ref="B10" r:id="rId9" display="https://www.hotelscombined.com.tw/flight-routes/Taipei-City-Taiwan-Taoyuan-Intl-TPE/Tokyo-Haneda-HND.ksp"/>
-    <hyperlink ref="B11" r:id="rId10" display="https://www.tw.kayak.com/%E8%88%AA%E7%8F%AD/%E5%8F%B0%E5%8C%97-TW1/%E6%9D%B1%E4%BA%AC-%E6%88%90%E7%94%B0%E5%9C%8B%E9%9A%9B%E6%A9%9F%E5%A0%B4-NRT"/>
-    <hyperlink ref="B12" r:id="rId11" display="https://www.tigerairtw.com/zh-tw/ready-to-go/fees"/>
-    <hyperlink ref="B13" r:id="rId12" display="https://ekitan.com/transit/shinkansen/section/sf-2590/st-737"/>
-    <hyperlink ref="B14" r:id="rId13" display="https://tohoku.letsgojp.com/archives/739243/"/>
-    <hyperlink ref="B15" r:id="rId14" display="https://travel.yamakobus.jp/zh-tw/timetable/routebus-yamagata-zaoline.html"/>
-    <hyperlink ref="B16" r:id="rId15" display="https://twoslowbyron.com/zao_ropeway/"/>
-    <hyperlink ref="B17" r:id="rId16" display="https://mimigo.tw/ginzan-onsen/"/>
-  </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Starlux official fare-bucket availability to Sendai sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MqDR8ErShU29xSVraYyKeW
</commit_message>
<xml_diff>
--- a/japan-ginzan-plan.xlsx
+++ b/japan-ginzan-plan.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="565">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="570">
   <si>
     <r>
       <rPr>
@@ -3171,7 +3171,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">。紅底＝只剩商務艙；沒列出的日期＝當天沒有直飛。虎航不含托運行李（</t>
+      <t xml:space="preserve">。紅底＝只剩商務艙或已售完；沒列出的日期＝當天沒有直飛。航空公司不公開剩餘座位數；星宇官網 </t>
     </r>
     <r>
       <rPr>
@@ -3181,6 +3181,25 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">1/28–2/3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">仙台回程經濟艙全部售完。虎航不含托運行李（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">20kg </t>
     </r>
     <r>
@@ -3306,16 +3325,96 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">星宇官網：只剩「全額」票價，便宜票價已售完，快滿了</t>
+  </si>
+  <si>
     <t xml:space="preserve">含行李</t>
   </si>
   <si>
-    <t xml:space="preserve">含行李；去程最便宜的全服務航空</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">星宇官網：超值 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15,733</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／基本 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">17,480</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／全額 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">22,784 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">三種票價都還有，座位最充足</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">含行李；最早抵達</t>
   </si>
   <si>
     <t xml:space="preserve">去程最便宜</t>
+  </si>
+  <si>
+    <t xml:space="preserve">星宇官網：只剩「全額」票價，快滿了</t>
+  </si>
+  <si>
+    <t xml:space="preserve">售完</t>
+  </si>
+  <si>
+    <t xml:space="preserve">星宇官網：整班已售完（含商務艙）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">星宇官網：經濟艙已售完</t>
   </si>
   <si>
     <t xml:space="preserve">回程唯一的平價選擇；落地晚</t>
@@ -10239,138 +10338,138 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>531</v>
+        <v>536</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>532</v>
+        <v>537</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>533</v>
+        <v>538</v>
       </c>
       <c r="B2" s="53" t="s">
-        <v>534</v>
+        <v>539</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>535</v>
+        <v>540</v>
       </c>
       <c r="B3" s="53" t="s">
-        <v>536</v>
+        <v>541</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="54" t="s">
-        <v>537</v>
+        <v>542</v>
       </c>
       <c r="B4" s="53" t="s">
-        <v>538</v>
+        <v>543</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="54" t="s">
-        <v>539</v>
+        <v>544</v>
       </c>
       <c r="B5" s="53" t="s">
-        <v>540</v>
+        <v>545</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="54" t="s">
-        <v>541</v>
+        <v>546</v>
       </c>
       <c r="B6" s="53" t="s">
-        <v>542</v>
+        <v>547</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="54" t="s">
-        <v>543</v>
+        <v>548</v>
       </c>
       <c r="B7" s="53" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="54" t="s">
-        <v>545</v>
+        <v>550</v>
       </c>
       <c r="B8" s="53" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>547</v>
+        <v>552</v>
       </c>
       <c r="B9" s="53" t="s">
-        <v>548</v>
+        <v>553</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="54" t="s">
-        <v>549</v>
+        <v>554</v>
       </c>
       <c r="B10" s="53" t="s">
-        <v>550</v>
+        <v>555</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="54" t="s">
-        <v>551</v>
+        <v>556</v>
       </c>
       <c r="B11" s="53" t="s">
-        <v>552</v>
+        <v>557</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="B12" s="53" t="s">
-        <v>554</v>
+        <v>559</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>555</v>
+        <v>560</v>
       </c>
       <c r="B13" s="53" t="s">
-        <v>556</v>
+        <v>561</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>557</v>
+        <v>562</v>
       </c>
       <c r="B14" s="53" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>559</v>
+        <v>564</v>
       </c>
       <c r="B15" s="53" t="s">
-        <v>560</v>
+        <v>565</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>561</v>
+        <v>566</v>
       </c>
       <c r="B16" s="53" t="s">
-        <v>562</v>
+        <v>567</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>563</v>
+        <v>568</v>
       </c>
       <c r="B17" s="53" t="s">
-        <v>564</v>
+        <v>569</v>
       </c>
     </row>
   </sheetData>
@@ -12042,10 +12141,10 @@
         <v>39</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
         <v>47</v>
       </c>
@@ -12065,7 +12164,7 @@
         <v>39</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12088,7 +12187,7 @@
         <v>39</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12111,7 +12210,7 @@
         <v>39</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12134,7 +12233,7 @@
         <v>39</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12217,14 +12316,12 @@
       <c r="D20" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="E20" s="24" t="n">
-        <v>34301</v>
-      </c>
+      <c r="E20" s="24"/>
       <c r="F20" s="23" t="s">
-        <v>61</v>
+        <v>212</v>
       </c>
       <c r="G20" s="23" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12247,7 +12344,7 @@
         <v>61</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12270,7 +12367,7 @@
         <v>39</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12293,7 +12390,7 @@
         <v>39</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12319,12 +12416,12 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="33" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="B27" s="8" t="s">
         <v>104</v>
@@ -12333,39 +12430,39 @@
         <v>105</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="E27" s="8" t="s">
         <v>107</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="B28" s="16" t="n">
         <v>4</v>
       </c>
       <c r="C28" s="20" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="D28" s="21" t="n">
         <v>14099</v>
       </c>
       <c r="E28" s="20" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="F28" s="21" t="n">
         <v>16466</v>
@@ -12378,24 +12475,24 @@
         <v>32465</v>
       </c>
       <c r="I28" s="16" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="26" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="B29" s="12" t="n">
         <v>4</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="D29" s="28" t="n">
         <v>14099</v>
       </c>
       <c r="E29" s="27" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="F29" s="28" t="n">
         <v>20549</v>
@@ -12408,24 +12505,24 @@
         <v>35598</v>
       </c>
       <c r="I29" s="12" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B30" s="16" t="n">
         <v>4</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="D30" s="21" t="n">
         <v>22784</v>
       </c>
       <c r="E30" s="20" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="F30" s="21" t="n">
         <v>20549</v>
@@ -12438,24 +12535,24 @@
         <v>43333</v>
       </c>
       <c r="I30" s="16" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="16" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B31" s="16" t="n">
         <v>5</v>
       </c>
       <c r="C31" s="20" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="D31" s="21" t="n">
         <v>15733</v>
       </c>
       <c r="E31" s="20" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="F31" s="21" t="n">
         <v>16466</v>
@@ -12468,24 +12565,24 @@
         <v>33149</v>
       </c>
       <c r="I31" s="16" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="B32" s="16" t="n">
         <v>5</v>
       </c>
       <c r="C32" s="20" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="D32" s="21" t="n">
         <v>17781</v>
       </c>
       <c r="E32" s="20" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="F32" s="21" t="n">
         <v>20549</v>
@@ -12498,24 +12595,24 @@
         <v>38330</v>
       </c>
       <c r="I32" s="16" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B33" s="16" t="n">
         <v>4</v>
       </c>
       <c r="C33" s="20" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="D33" s="21" t="n">
         <v>15733</v>
       </c>
       <c r="E33" s="20" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="F33" s="21" t="n">
         <v>33029</v>
@@ -12528,12 +12625,12 @@
         <v>48762</v>
       </c>
       <c r="I33" s="16" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="33" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12548,7 +12645,7 @@
       <c r="E36" s="8"/>
       <c r="F36" s="8"/>
       <c r="G36" s="8" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12556,14 +12653,14 @@
         <v>154</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C37" s="16"/>
       <c r="D37" s="16"/>
       <c r="E37" s="16"/>
       <c r="F37" s="16"/>
       <c r="G37" s="16" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12571,14 +12668,14 @@
         <v>165</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="C38" s="12"/>
       <c r="D38" s="12"/>
       <c r="E38" s="12"/>
       <c r="F38" s="12"/>
       <c r="G38" s="12" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12586,14 +12683,14 @@
         <v>173</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="C39" s="16"/>
       <c r="D39" s="16"/>
       <c r="E39" s="16"/>
       <c r="F39" s="16"/>
       <c r="G39" s="16" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12601,14 +12698,14 @@
         <v>183</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="C40" s="16"/>
       <c r="D40" s="16"/>
       <c r="E40" s="16"/>
       <c r="F40" s="16"/>
       <c r="G40" s="16" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12616,22 +12713,22 @@
         <v>187</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C41" s="16"/>
       <c r="D41" s="16"/>
       <c r="E41" s="16"/>
       <c r="F41" s="16"/>
       <c r="G41" s="16" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="37" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C42" s="16"/>
       <c r="D42" s="16"/>
@@ -12677,12 +12774,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12704,34 +12801,34 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="34" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="C5" s="36" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16"/>
       <c r="B6" s="20" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12740,67 +12837,67 @@
         <v>147</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16"/>
       <c r="B8" s="20" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16"/>
       <c r="B9" s="20" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16"/>
       <c r="B10" s="20" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16"/>
       <c r="B11" s="20" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="D11" s="16"/>
       <c r="E11" s="16" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12811,35 +12908,35 @@
         <v>155</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16"/>
       <c r="B13" s="20" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="D13" s="16"/>
       <c r="E13" s="16" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16"/>
       <c r="B14" s="20" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
@@ -12847,20 +12944,20 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16"/>
       <c r="B15" s="20" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="E15" s="16"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16"/>
       <c r="B16" s="20" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>151</v>
@@ -12869,7 +12966,7 @@
         <v>152</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12878,26 +12975,26 @@
         <v>180</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="D17" s="16"/>
       <c r="E17" s="16" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16"/>
       <c r="B18" s="20" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12908,22 +13005,22 @@
         <v>155</v>
       </c>
       <c r="C19" s="36" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="D19" s="36" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="E19" s="36" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16"/>
       <c r="B20" s="20" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="D20" s="16"/>
       <c r="E20" s="16"/>
@@ -12931,10 +13028,10 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16"/>
       <c r="B21" s="20" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>152</v>
@@ -12944,25 +13041,25 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16"/>
       <c r="B22" s="20" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="16"/>
       <c r="B23" s="20" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="D23" s="16"/>
       <c r="E23" s="16" t="s">
@@ -12974,77 +13071,77 @@
         <v>165</v>
       </c>
       <c r="B24" s="35" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="C24" s="36" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="D24" s="36"/>
       <c r="E24" s="36" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16"/>
       <c r="B25" s="20" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>167</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="E25" s="16"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16"/>
       <c r="B26" s="20" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="E26" s="16" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12"/>
       <c r="B27" s="27" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="12" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16"/>
       <c r="B28" s="20" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="D28" s="16"/>
       <c r="E28" s="16" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16"/>
       <c r="B29" s="20" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
@@ -13052,14 +13149,14 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16"/>
       <c r="B30" s="20" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="D30" s="16"/>
       <c r="E30" s="16" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13074,16 +13171,16 @@
       </c>
       <c r="D31" s="36"/>
       <c r="E31" s="36" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16"/>
       <c r="B32" s="20" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
@@ -13091,38 +13188,38 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16"/>
       <c r="B33" s="20" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="E33" s="16"/>
     </row>
     <row r="34" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="16"/>
       <c r="B34" s="20" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="E34" s="16" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16"/>
       <c r="B35" s="20" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
@@ -13130,27 +13227,27 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16"/>
       <c r="B36" s="20" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="D36" s="16"/>
       <c r="E36" s="16" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16"/>
       <c r="B37" s="20" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="D37" s="16"/>
       <c r="E37" s="16" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13158,10 +13255,10 @@
         <v>183</v>
       </c>
       <c r="B38" s="35" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="C38" s="36" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="D38" s="36"/>
       <c r="E38" s="36"/>
@@ -13172,23 +13269,23 @@
         <v>155</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="D39" s="20" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="E39" s="16"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16"/>
       <c r="B40" s="20" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="E40" s="16"/>
     </row>
@@ -13198,85 +13295,85 @@
         <v>166</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="E41" s="16"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="16"/>
       <c r="B42" s="20" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="D42" s="16"/>
       <c r="E42" s="16" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="16"/>
       <c r="B43" s="20" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="D43" s="20" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="E43" s="16"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="16"/>
       <c r="B44" s="20" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="E44" s="16" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="16"/>
       <c r="B45" s="20" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="D45" s="16"/>
       <c r="E45" s="16" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="16"/>
       <c r="B46" s="20" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="E46" s="16" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
     </row>
   </sheetData>
@@ -13314,17 +13411,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>29</v>
@@ -13333,66 +13430,66 @@
         <v>30</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>44</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>4743</v>
@@ -13411,36 +13508,36 @@
         <v>9676</v>
       </c>
       <c r="N5" s="16" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="O5" s="21" t="n">
         <v>950</v>
       </c>
       <c r="P5" s="16" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>37</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>9845</v>
@@ -13459,36 +13556,36 @@
         <v>17878</v>
       </c>
       <c r="N6" s="16" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="O6" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P6" s="16" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>41</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="H7" s="21" t="n">
         <v>9720</v>
@@ -13507,36 +13604,36 @@
         <v>19586</v>
       </c>
       <c r="N7" s="16" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="O7" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P7" s="16" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>37</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="E8" s="20" t="s">
+        <v>404</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>405</v>
+      </c>
+      <c r="G8" s="16" t="s">
         <v>399</v>
-      </c>
-      <c r="F8" s="16" t="s">
-        <v>400</v>
-      </c>
-      <c r="G8" s="16" t="s">
-        <v>394</v>
       </c>
       <c r="H8" s="21" t="n">
         <v>10361</v>
@@ -13555,36 +13652,36 @@
         <v>16526</v>
       </c>
       <c r="N8" s="16" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="O8" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P8" s="16" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
+        <v>407</v>
+      </c>
+      <c r="B9" s="16" t="s">
         <v>402</v>
       </c>
-      <c r="B9" s="16" t="s">
-        <v>397</v>
-      </c>
       <c r="C9" s="16" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="E9" s="20" t="s">
+        <v>410</v>
+      </c>
+      <c r="F9" s="16" t="s">
         <v>405</v>
       </c>
-      <c r="F9" s="16" t="s">
-        <v>400</v>
-      </c>
       <c r="G9" s="16" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="H9" s="21" t="n">
         <v>10361</v>
@@ -13603,36 +13700,36 @@
         <v>16526</v>
       </c>
       <c r="N9" s="16" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="O9" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P9" s="16" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="H10" s="21" t="n">
         <v>10361</v>
@@ -13651,36 +13748,36 @@
         <v>16526</v>
       </c>
       <c r="N10" s="16" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="O10" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P10" s="16" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="H11" s="21" t="n">
         <v>10361</v>
@@ -13699,36 +13796,36 @@
         <v>16526</v>
       </c>
       <c r="N11" s="16" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="O11" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P11" s="16" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>93</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="H12" s="21" t="n">
         <v>5386</v>
@@ -13748,36 +13845,36 @@
         <v>10772</v>
       </c>
       <c r="N12" s="16" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="O12" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="P12" s="16" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="D13" s="20" t="s">
+        <v>428</v>
+      </c>
+      <c r="E13" s="16" t="s">
         <v>423</v>
       </c>
-      <c r="E13" s="16" t="s">
-        <v>418</v>
-      </c>
       <c r="F13" s="16" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="H13" s="21" t="n">
         <v>3748</v>
@@ -13797,36 +13894,36 @@
         <v>7496</v>
       </c>
       <c r="N13" s="16" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="O13" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="P13" s="16" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>44</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="H14" s="21" t="n">
         <v>6702</v>
@@ -13846,18 +13943,18 @@
         <v>13404</v>
       </c>
       <c r="N14" s="16" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="O14" s="21" t="n">
         <v>950</v>
       </c>
       <c r="P14" s="16" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
     </row>
   </sheetData>
@@ -13894,17 +13991,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>10</v>
@@ -13922,45 +14019,45 @@
         <v>107</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
       <c r="D5" s="40" t="n">
         <v>4</v>
       </c>
       <c r="E5" s="27" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
       <c r="F5" s="27" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
       <c r="G5" s="11" t="n">
         <f aca="false">機票價格!L6+機票價格!L5</f>
@@ -13982,30 +14079,30 @@
         <v>15538</v>
       </c>
       <c r="L5" s="27" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
+        <v>449</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>450</v>
+      </c>
+      <c r="C6" s="20" t="s">
         <v>444</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>445</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>439</v>
       </c>
       <c r="D6" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="G6" s="15" t="n">
         <f aca="false">機票價格!M5</f>
@@ -14027,30 +14124,30 @@
         <v>11576</v>
       </c>
       <c r="L6" s="20" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="M6" s="16" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
       <c r="D7" s="41" t="n">
         <v>3</v>
       </c>
       <c r="E7" s="20" t="s">
+        <v>457</v>
+      </c>
+      <c r="F7" s="20" t="s">
         <v>452</v>
-      </c>
-      <c r="F7" s="20" t="s">
-        <v>447</v>
       </c>
       <c r="G7" s="15" t="n">
         <f aca="false">機票價格!L6+機票價格!L5</f>
@@ -14072,30 +14169,30 @@
         <v>15538</v>
       </c>
       <c r="L7" s="20" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="M7" s="16" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
       <c r="D8" s="41" t="n">
         <v>3</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="G8" s="15" t="n">
         <f aca="false">機票價格!M7</f>
@@ -14117,30 +14214,30 @@
         <v>19586</v>
       </c>
       <c r="L8" s="20" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>459</v>
+        <v>464</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
       <c r="D9" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
       <c r="G9" s="15" t="n">
         <f aca="false">機票價格!M8</f>
@@ -14163,30 +14260,30 @@
         <v>21379.1</v>
       </c>
       <c r="L9" s="20" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>466</v>
+        <v>471</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
       <c r="D10" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
       <c r="G10" s="15" t="n">
         <f aca="false">機票價格!L5+機票價格!L8</f>
@@ -14209,30 +14306,30 @@
         <v>18303.1</v>
       </c>
       <c r="L10" s="20" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="M10" s="16" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
       <c r="D11" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>470</v>
+        <v>475</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
       <c r="G11" s="15" t="n">
         <f aca="false">機票價格!M12</f>
@@ -14255,15 +14352,15 @@
         <v>17625.1</v>
       </c>
       <c r="L11" s="20" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="C13" s="3" t="str">
         <f aca="false">INDEX(B5:B11,MATCH(MIN(K5:K11),K5:K11,0))</f>
@@ -14306,12 +14403,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14322,25 +14419,25 @@
         <v>136</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>481</v>
+        <v>486</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
       <c r="J4" s="8" t="s">
         <v>200</v>
@@ -14351,16 +14448,16 @@
         <v>35</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>1310</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="F5" s="31" t="n">
         <v>9000</v>
@@ -14377,7 +14474,7 @@
         <v>2284.8</v>
       </c>
       <c r="J5" s="43" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14385,16 +14482,16 @@
         <v>47</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="D6" s="31" t="n">
         <v>2300</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="F6" s="31" t="n">
         <v>20000</v>
@@ -14411,7 +14508,7 @@
         <v>4683</v>
       </c>
       <c r="J6" s="43" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14419,16 +14516,16 @@
         <v>49</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="D7" s="31" t="n">
         <v>1200</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="F7" s="31" t="n">
         <v>8000</v>
@@ -14445,24 +14542,24 @@
         <v>2856</v>
       </c>
       <c r="J7" s="43" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>496</v>
+        <v>501</v>
       </c>
       <c r="D8" s="31" t="n">
         <v>1900</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="F8" s="44" t="n">
         <f aca="false">總覽!B7</f>
@@ -14480,7 +14577,7 @@
         <v>399</v>
       </c>
       <c r="J8" s="45" t="s">
-        <v>498</v>
+        <v>503</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14488,16 +14585,16 @@
         <v>66</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>499</v>
+        <v>504</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
       <c r="D9" s="31" t="n">
         <v>2690</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="F9" s="31" t="n">
         <v>9000</v>
@@ -14520,10 +14617,10 @@
         <v>58</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="D10" s="31" t="n">
         <v>1540</v>
@@ -14546,7 +14643,7 @@
         <v>785.4</v>
       </c>
       <c r="J10" s="43" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14580,18 +14677,18 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="H12" s="49" t="n">
         <v>5000</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>506</v>
+        <v>511</v>
       </c>
       <c r="H13" s="50" t="n">
         <f aca="false">H12*6</f>
@@ -14604,7 +14701,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="I14" s="18" t="n">
         <f aca="false">I11+I13</f>
@@ -14638,13 +14735,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>509</v>
+        <v>514</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>510</v>
+        <v>515</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>200</v>
@@ -14652,100 +14749,100 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="C2" s="52" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>514</v>
+        <v>519</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>515</v>
+        <v>520</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="C3" s="52" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>516</v>
+        <v>521</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
+        <v>522</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>517</v>
       </c>
-      <c r="B4" s="20" t="s">
-        <v>512</v>
-      </c>
       <c r="C4" s="52" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>518</v>
+        <v>523</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>519</v>
+        <v>524</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>520</v>
+        <v>525</v>
       </c>
       <c r="C5" s="52" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>521</v>
+        <v>526</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>522</v>
+        <v>527</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="C6" s="52" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>524</v>
+        <v>529</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>526</v>
+        <v>531</v>
       </c>
       <c r="C7" s="52" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>528</v>
+        <v>533</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>529</v>
+        <v>534</v>
       </c>
       <c r="C8" s="52" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>530</v>
+        <v>535</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add non-Sendai return options (Akita, Aomori, Hanamaki, Niigata) with live fares
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MqDR8ErShU29xSVraYyKeW
</commit_message>
<xml_diff>
--- a/japan-ginzan-plan.xlsx
+++ b/japan-ginzan-plan.xlsx
@@ -12,12 +12,13 @@
     <sheet name="即時查價 10-9" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="新方案 10-10" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="仙台進出 10-10" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="每日行程" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="機票價格" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="方案比較" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="行程預算" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="待辦清單" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="資料來源" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="非仙台回程 10-10" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="每日行程" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="機票價格" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="方案比較" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="行程預算" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="待辦清單" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="資料來源" sheetId="11" state="visible" r:id="rId13"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="608">
   <si>
     <r>
       <rPr>
@@ -4284,6 +4285,1627 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">抵達桃園</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">仙台進、其他東北機場回（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Google Flights 2026/10/10</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">，每人單程經濟艙含稅，新台幣）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">去程皆以 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/27</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（三）星宇 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">11:50 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">桃園→仙台（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NT$15,733</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">，含行李，目前位子最多）計算；也可以改搭長榮 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10:15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NT$17,781</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）。福島、山形機場 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/30–2/1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">沒有直飛。陸路交通為估計值。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">回程航班</t>
+  </si>
+  <si>
+    <t xml:space="preserve">陸路交通（日圓，估）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">旅遊天數</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Ⓐ 秋田回（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/31 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">虎航 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">14:10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秋田→桃園 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">17:25</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">夜</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">只請 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天最省假；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">從銀山溫泉到乳頭溫泉住一晚，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/31 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">搭秋田新幹線到秋田再去機場。落地 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">17:25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">，不算晚回</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Ⓑ 青森回（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/1 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">一）★</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">長榮 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15:30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">青森→桃園 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">19:00</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">夜</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">全程都是全服務航空、含行李；回程票價最便宜；多玩乳頭溫泉＋青森（酸湯溫泉／八甲田）；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">19:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">落地</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Ⓒ 花卷回（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">六）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">虎航 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">17:50 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">花卷→桃園 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">21:10</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">夜</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">行程最短；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">要 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">9:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">前離開銀山溫泉，車程約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">小時，班次少有風險</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Ⓓ 新潟回（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">一）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">虎航 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">19:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">新潟→桃園 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">22:30</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">機票最便宜，但 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">22:30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">才落地，羽越線冬天常因大雪誤點</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Ⓔ 青森回（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/31 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">請 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天也能晚一點回來，但 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/30–1/31 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">要長途移動</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">參考：仙台回（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">二）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">長榮 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">16:15 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">仙台→桃園 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">19:30</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">夜</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">仙台回程經濟艙最早只有 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/2</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Ⓑ 青森回 行程：</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/27 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">三 – </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/1 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">一（請假 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/27</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/28</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/29</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/1</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">星宇 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">11:50 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">桃園 → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">16:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">仙台 → 巴士或 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">JR </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">到山形 → 巴士到藏王溫泉（約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">小時）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">早上搭纜車看樹冰 → 下午山寺 → 山形</t>
+  </si>
+  <si>
+    <t xml:space="preserve">山形</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">山形 → 大石田 → 銀山溫泉，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">16:45 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">拍瓦斯燈藍調時刻</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">清晨拍照 → 大石田 → 新庄 → 奧羽本線 → 大曲 → 秋田新幹線到田澤湖 → 巴士到乳頭溫泉（約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">小時，中午前出發）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">乳頭溫泉鄉（鶴之湯等）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">乳頭溫泉 → 田澤湖 → 秋田新幹線到盛岡 → 隼號到新青森（約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">小時）→ 青森市區（睡魔之家、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">A-FACTORY</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、海鮮）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">青森市（或酸湯溫泉）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">上午青森魚菜中心吃自選海鮮丼 → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">13:30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">搭巴士到機場（約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">35 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分鐘）→ 長榮 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15:30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">起飛，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">19:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">抵達桃園</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Ⓐ 秋田回：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/27–1/29 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">同上；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">銀山溫泉 → 乳頭溫泉；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/31 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">乳頭 → 田澤湖 → 秋田新幹線到秋田（約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">小時）→ 巴士到機場（約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分鐘）→ 虎航 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">14:10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">起飛。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">陸路參考：新庄—大曲之間的奧羽本線班次很少（院內站每天約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">班），出發前務必查 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">JR </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">東日本時刻表；八甲田纜車冬季 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">9:00–15:40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">，常因強風停駛。</t>
     </r>
   </si>
   <si>
@@ -10329,6 +11951,149 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="8" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>552</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>553</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="16" t="s">
+        <v>554</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>555</v>
+      </c>
+      <c r="C2" s="52" t="s">
+        <v>556</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="16" t="s">
+        <v>558</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>555</v>
+      </c>
+      <c r="C3" s="52" t="s">
+        <v>556</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="16" t="s">
+        <v>560</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>555</v>
+      </c>
+      <c r="C4" s="52" t="s">
+        <v>556</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
+        <v>562</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>563</v>
+      </c>
+      <c r="C5" s="52" t="s">
+        <v>556</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="s">
+        <v>565</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="C6" s="52" t="s">
+        <v>556</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>568</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>569</v>
+      </c>
+      <c r="C7" s="52" t="s">
+        <v>556</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>571</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>572</v>
+      </c>
+      <c r="C8" s="52" t="s">
+        <v>556</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>573</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C2:C8" type="list">
+      <formula1>"未開始,進行中,完成"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:B17"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -10338,138 +12103,138 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>536</v>
+        <v>574</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>537</v>
+        <v>575</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>538</v>
+        <v>576</v>
       </c>
       <c r="B2" s="53" t="s">
-        <v>539</v>
+        <v>577</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>540</v>
+        <v>578</v>
       </c>
       <c r="B3" s="53" t="s">
-        <v>541</v>
+        <v>579</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="54" t="s">
-        <v>542</v>
+        <v>580</v>
       </c>
       <c r="B4" s="53" t="s">
-        <v>543</v>
+        <v>581</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="54" t="s">
-        <v>544</v>
+        <v>582</v>
       </c>
       <c r="B5" s="53" t="s">
-        <v>545</v>
+        <v>583</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="54" t="s">
-        <v>546</v>
+        <v>584</v>
       </c>
       <c r="B6" s="53" t="s">
-        <v>547</v>
+        <v>585</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="54" t="s">
-        <v>548</v>
+        <v>586</v>
       </c>
       <c r="B7" s="53" t="s">
-        <v>549</v>
+        <v>587</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="54" t="s">
-        <v>550</v>
+        <v>588</v>
       </c>
       <c r="B8" s="53" t="s">
-        <v>551</v>
+        <v>589</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>552</v>
+        <v>590</v>
       </c>
       <c r="B9" s="53" t="s">
-        <v>553</v>
+        <v>591</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="54" t="s">
-        <v>554</v>
+        <v>592</v>
       </c>
       <c r="B10" s="53" t="s">
-        <v>555</v>
+        <v>593</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="54" t="s">
-        <v>556</v>
+        <v>594</v>
       </c>
       <c r="B11" s="53" t="s">
-        <v>557</v>
+        <v>595</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>558</v>
+        <v>596</v>
       </c>
       <c r="B12" s="53" t="s">
-        <v>559</v>
+        <v>597</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>560</v>
+        <v>598</v>
       </c>
       <c r="B13" s="53" t="s">
-        <v>561</v>
+        <v>599</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>562</v>
+        <v>600</v>
       </c>
       <c r="B14" s="53" t="s">
-        <v>563</v>
+        <v>601</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>564</v>
+        <v>602</v>
       </c>
       <c r="B15" s="53" t="s">
-        <v>565</v>
+        <v>603</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>566</v>
+        <v>604</v>
       </c>
       <c r="B16" s="53" t="s">
-        <v>567</v>
+        <v>605</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>568</v>
+        <v>606</v>
       </c>
       <c r="B17" s="53" t="s">
-        <v>569</v>
+        <v>607</v>
       </c>
     </row>
   </sheetData>
@@ -12762,6 +14527,425 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:J22"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="52"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="25" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
+        <v>260</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>261</v>
+      </c>
+      <c r="C5" s="21" t="n">
+        <v>11147</v>
+      </c>
+      <c r="D5" s="21" t="n">
+        <v>950</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>15733</v>
+      </c>
+      <c r="F5" s="31" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G5" s="32" t="n">
+        <f aca="false">C5+D5+E5+F5*總覽!$B$5</f>
+        <v>30350</v>
+      </c>
+      <c r="H5" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="J5" s="16" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="26" t="s">
+        <v>264</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C6" s="28" t="n">
+        <v>11999</v>
+      </c>
+      <c r="D6" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="28" t="n">
+        <v>15733</v>
+      </c>
+      <c r="F6" s="29" t="n">
+        <v>22000</v>
+      </c>
+      <c r="G6" s="30" t="n">
+        <f aca="false">C6+D6+E6+F6*總覽!$B$5</f>
+        <v>32352</v>
+      </c>
+      <c r="H6" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" s="27" t="s">
+        <v>266</v>
+      </c>
+      <c r="J6" s="12" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>268</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>269</v>
+      </c>
+      <c r="C7" s="21" t="n">
+        <v>11995</v>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>950</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>15733</v>
+      </c>
+      <c r="F7" s="31" t="n">
+        <v>6500</v>
+      </c>
+      <c r="G7" s="32" t="n">
+        <f aca="false">C7+D7+E7+F7*總覽!$B$5</f>
+        <v>30043</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="J7" s="16" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>272</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>273</v>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>10890</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>950</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>15733</v>
+      </c>
+      <c r="F8" s="31" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G8" s="32" t="n">
+        <f aca="false">C8+D8+E8+F8*總覽!$B$5</f>
+        <v>29463</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="I8" s="20" t="s">
+        <v>266</v>
+      </c>
+      <c r="J8" s="16" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
+        <v>275</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>265</v>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>14987</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>15733</v>
+      </c>
+      <c r="F9" s="31" t="n">
+        <v>16000</v>
+      </c>
+      <c r="G9" s="32" t="n">
+        <f aca="false">C9+D9+E9+F9*總覽!$B$5</f>
+        <v>34080</v>
+      </c>
+      <c r="H9" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="I9" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="J9" s="16" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="16" t="s">
+        <v>277</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>278</v>
+      </c>
+      <c r="C10" s="21" t="n">
+        <v>20549</v>
+      </c>
+      <c r="D10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>15733</v>
+      </c>
+      <c r="F10" s="31" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G10" s="32" t="n">
+        <f aca="false">C10+D10+E10+F10*總覽!$B$5</f>
+        <v>36912</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" s="20" t="s">
+        <v>279</v>
+      </c>
+      <c r="J10" s="16" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="33" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="J13" s="8"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="37" t="s">
+        <v>139</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>282</v>
+      </c>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="J14" s="16"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="37" t="s">
+        <v>154</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>283</v>
+      </c>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="J15" s="16"/>
+    </row>
+    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="38" t="s">
+        <v>165</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="J16" s="12"/>
+    </row>
+    <row r="17" customFormat="false" ht="39.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="37" t="s">
+        <v>173</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>286</v>
+      </c>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16" t="s">
+        <v>287</v>
+      </c>
+      <c r="J17" s="16"/>
+    </row>
+    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="37" t="s">
+        <v>183</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>288</v>
+      </c>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16" t="s">
+        <v>289</v>
+      </c>
+      <c r="J18" s="16"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="37" t="s">
+        <v>187</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>290</v>
+      </c>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="J19" s="16"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
+        <v>292</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B19:H19"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:E48"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -12774,12 +14958,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>255</v>
+        <v>293</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>256</v>
+        <v>294</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12801,34 +14985,34 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="34" t="s">
-        <v>257</v>
+        <v>295</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>258</v>
+        <v>296</v>
       </c>
       <c r="C5" s="36" t="s">
-        <v>259</v>
+        <v>297</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>260</v>
+        <v>298</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>261</v>
+        <v>299</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16"/>
       <c r="B6" s="20" t="s">
-        <v>262</v>
+        <v>300</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>263</v>
+        <v>301</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>264</v>
+        <v>302</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>265</v>
+        <v>303</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12837,67 +15021,67 @@
         <v>147</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>266</v>
+        <v>304</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16" t="s">
-        <v>267</v>
+        <v>305</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16"/>
       <c r="B8" s="20" t="s">
-        <v>268</v>
+        <v>306</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>269</v>
+        <v>307</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>270</v>
+        <v>308</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>271</v>
+        <v>309</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16"/>
       <c r="B9" s="20" t="s">
-        <v>272</v>
+        <v>310</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>273</v>
+        <v>311</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16" t="s">
-        <v>274</v>
+        <v>312</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16"/>
       <c r="B10" s="20" t="s">
-        <v>275</v>
+        <v>313</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>276</v>
+        <v>314</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>277</v>
+        <v>315</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>278</v>
+        <v>316</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16"/>
       <c r="B11" s="20" t="s">
-        <v>279</v>
+        <v>317</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>280</v>
+        <v>318</v>
       </c>
       <c r="D11" s="16"/>
       <c r="E11" s="16" t="s">
-        <v>281</v>
+        <v>319</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12908,35 +15092,35 @@
         <v>155</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>282</v>
+        <v>320</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>283</v>
+        <v>321</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>284</v>
+        <v>322</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16"/>
       <c r="B13" s="20" t="s">
-        <v>285</v>
+        <v>323</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>286</v>
+        <v>324</v>
       </c>
       <c r="D13" s="16"/>
       <c r="E13" s="16" t="s">
-        <v>287</v>
+        <v>325</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16"/>
       <c r="B14" s="20" t="s">
-        <v>288</v>
+        <v>326</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>289</v>
+        <v>327</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
@@ -12944,20 +15128,20 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16"/>
       <c r="B15" s="20" t="s">
-        <v>290</v>
+        <v>328</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>291</v>
+        <v>329</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>292</v>
+        <v>330</v>
       </c>
       <c r="E15" s="16"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16"/>
       <c r="B16" s="20" t="s">
-        <v>272</v>
+        <v>310</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>151</v>
@@ -12966,7 +15150,7 @@
         <v>152</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>293</v>
+        <v>331</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12975,26 +15159,26 @@
         <v>180</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>294</v>
+        <v>332</v>
       </c>
       <c r="D17" s="16"/>
       <c r="E17" s="16" t="s">
-        <v>295</v>
+        <v>333</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16"/>
       <c r="B18" s="20" t="s">
-        <v>279</v>
+        <v>317</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>296</v>
+        <v>334</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>297</v>
+        <v>335</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>298</v>
+        <v>336</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13005,22 +15189,22 @@
         <v>155</v>
       </c>
       <c r="C19" s="36" t="s">
-        <v>299</v>
+        <v>337</v>
       </c>
       <c r="D19" s="36" t="s">
-        <v>300</v>
+        <v>338</v>
       </c>
       <c r="E19" s="36" t="s">
-        <v>301</v>
+        <v>339</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16"/>
       <c r="B20" s="20" t="s">
-        <v>288</v>
+        <v>326</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>302</v>
+        <v>340</v>
       </c>
       <c r="D20" s="16"/>
       <c r="E20" s="16"/>
@@ -13028,10 +15212,10 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16"/>
       <c r="B21" s="20" t="s">
-        <v>303</v>
+        <v>341</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>304</v>
+        <v>342</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>152</v>
@@ -13041,25 +15225,25 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16"/>
       <c r="B22" s="20" t="s">
-        <v>275</v>
+        <v>313</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>305</v>
+        <v>343</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>306</v>
+        <v>344</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>307</v>
+        <v>345</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="16"/>
       <c r="B23" s="20" t="s">
-        <v>279</v>
+        <v>317</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>308</v>
+        <v>346</v>
       </c>
       <c r="D23" s="16"/>
       <c r="E23" s="16" t="s">
@@ -13071,77 +15255,77 @@
         <v>165</v>
       </c>
       <c r="B24" s="35" t="s">
-        <v>309</v>
+        <v>347</v>
       </c>
       <c r="C24" s="36" t="s">
-        <v>310</v>
+        <v>348</v>
       </c>
       <c r="D24" s="36"/>
       <c r="E24" s="36" t="s">
-        <v>311</v>
+        <v>349</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16"/>
       <c r="B25" s="20" t="s">
-        <v>312</v>
+        <v>350</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>167</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>313</v>
+        <v>351</v>
       </c>
       <c r="E25" s="16"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16"/>
       <c r="B26" s="20" t="s">
-        <v>303</v>
+        <v>341</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>314</v>
+        <v>352</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>315</v>
+        <v>353</v>
       </c>
       <c r="E26" s="16" t="s">
-        <v>316</v>
+        <v>354</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12"/>
       <c r="B27" s="27" t="s">
-        <v>275</v>
+        <v>313</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>317</v>
+        <v>355</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="12" t="s">
-        <v>318</v>
+        <v>356</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16"/>
       <c r="B28" s="20" t="s">
-        <v>319</v>
+        <v>357</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>320</v>
+        <v>358</v>
       </c>
       <c r="D28" s="16"/>
       <c r="E28" s="16" t="s">
-        <v>321</v>
+        <v>359</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16"/>
       <c r="B29" s="20" t="s">
-        <v>322</v>
+        <v>360</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>323</v>
+        <v>361</v>
       </c>
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
@@ -13149,14 +15333,14 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16"/>
       <c r="B30" s="20" t="s">
-        <v>324</v>
+        <v>362</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>325</v>
+        <v>363</v>
       </c>
       <c r="D30" s="16"/>
       <c r="E30" s="16" t="s">
-        <v>326</v>
+        <v>364</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13171,16 +15355,16 @@
       </c>
       <c r="D31" s="36"/>
       <c r="E31" s="36" t="s">
-        <v>327</v>
+        <v>365</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16"/>
       <c r="B32" s="20" t="s">
-        <v>328</v>
+        <v>366</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>329</v>
+        <v>367</v>
       </c>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
@@ -13188,38 +15372,38 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16"/>
       <c r="B33" s="20" t="s">
-        <v>330</v>
+        <v>368</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>331</v>
+        <v>369</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>332</v>
+        <v>370</v>
       </c>
       <c r="E33" s="16"/>
     </row>
     <row r="34" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="16"/>
       <c r="B34" s="20" t="s">
-        <v>333</v>
+        <v>371</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>334</v>
+        <v>372</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>335</v>
+        <v>373</v>
       </c>
       <c r="E34" s="16" t="s">
-        <v>336</v>
+        <v>374</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16"/>
       <c r="B35" s="20" t="s">
-        <v>272</v>
+        <v>310</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>337</v>
+        <v>375</v>
       </c>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
@@ -13227,27 +15411,27 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16"/>
       <c r="B36" s="20" t="s">
-        <v>275</v>
+        <v>313</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>338</v>
+        <v>376</v>
       </c>
       <c r="D36" s="16"/>
       <c r="E36" s="16" t="s">
-        <v>339</v>
+        <v>377</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16"/>
       <c r="B37" s="20" t="s">
-        <v>322</v>
+        <v>360</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>340</v>
+        <v>378</v>
       </c>
       <c r="D37" s="16"/>
       <c r="E37" s="16" t="s">
-        <v>341</v>
+        <v>379</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13255,10 +15439,10 @@
         <v>183</v>
       </c>
       <c r="B38" s="35" t="s">
-        <v>328</v>
+        <v>366</v>
       </c>
       <c r="C38" s="36" t="s">
-        <v>342</v>
+        <v>380</v>
       </c>
       <c r="D38" s="36"/>
       <c r="E38" s="36"/>
@@ -13269,23 +15453,23 @@
         <v>155</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>343</v>
+        <v>381</v>
       </c>
       <c r="D39" s="20" t="s">
-        <v>344</v>
+        <v>382</v>
       </c>
       <c r="E39" s="16"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16"/>
       <c r="B40" s="20" t="s">
-        <v>345</v>
+        <v>383</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>346</v>
+        <v>384</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>347</v>
+        <v>385</v>
       </c>
       <c r="E40" s="16"/>
     </row>
@@ -13295,85 +15479,85 @@
         <v>166</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>348</v>
+        <v>386</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>349</v>
+        <v>387</v>
       </c>
       <c r="E41" s="16"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="16"/>
       <c r="B42" s="20" t="s">
-        <v>288</v>
+        <v>326</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>350</v>
+        <v>388</v>
       </c>
       <c r="D42" s="16"/>
       <c r="E42" s="16" t="s">
-        <v>351</v>
+        <v>389</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="16"/>
       <c r="B43" s="20" t="s">
-        <v>303</v>
+        <v>341</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>352</v>
+        <v>390</v>
       </c>
       <c r="D43" s="20" t="s">
-        <v>344</v>
+        <v>382</v>
       </c>
       <c r="E43" s="16"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="16"/>
       <c r="B44" s="20" t="s">
-        <v>353</v>
+        <v>391</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>354</v>
+        <v>392</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>270</v>
+        <v>308</v>
       </c>
       <c r="E44" s="16" t="s">
-        <v>355</v>
+        <v>393</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="16"/>
       <c r="B45" s="20" t="s">
-        <v>356</v>
+        <v>394</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>357</v>
+        <v>395</v>
       </c>
       <c r="D45" s="16"/>
       <c r="E45" s="16" t="s">
-        <v>358</v>
+        <v>396</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="16"/>
       <c r="B46" s="20" t="s">
-        <v>359</v>
+        <v>397</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>360</v>
+        <v>398</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>361</v>
+        <v>399</v>
       </c>
       <c r="E46" s="16" t="s">
-        <v>362</v>
+        <v>400</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>363</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -13387,7 +15571,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -13411,17 +15595,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>364</v>
+        <v>402</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>365</v>
+        <v>403</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>366</v>
+        <v>404</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>29</v>
@@ -13430,66 +15614,66 @@
         <v>30</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>367</v>
+        <v>405</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>368</v>
+        <v>406</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>369</v>
+        <v>407</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>370</v>
+        <v>408</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>371</v>
+        <v>409</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>372</v>
+        <v>410</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>373</v>
+        <v>411</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>374</v>
+        <v>412</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>375</v>
+        <v>413</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>376</v>
+        <v>414</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>377</v>
+        <v>415</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>378</v>
+        <v>416</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>379</v>
+        <v>417</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>380</v>
+        <v>418</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>381</v>
+        <v>419</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>44</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>382</v>
+        <v>420</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>383</v>
+        <v>421</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>384</v>
+        <v>422</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>385</v>
+        <v>423</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>4743</v>
@@ -13508,36 +15692,36 @@
         <v>9676</v>
       </c>
       <c r="N5" s="16" t="s">
-        <v>386</v>
+        <v>424</v>
       </c>
       <c r="O5" s="21" t="n">
         <v>950</v>
       </c>
       <c r="P5" s="16" t="s">
-        <v>387</v>
+        <v>425</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>388</v>
+        <v>426</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>381</v>
+        <v>419</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>37</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>389</v>
+        <v>427</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>390</v>
+        <v>428</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>391</v>
+        <v>429</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>392</v>
+        <v>430</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>9845</v>
@@ -13556,36 +15740,36 @@
         <v>17878</v>
       </c>
       <c r="N6" s="16" t="s">
-        <v>393</v>
+        <v>431</v>
       </c>
       <c r="O6" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P6" s="16" t="s">
-        <v>394</v>
+        <v>432</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>395</v>
+        <v>433</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>381</v>
+        <v>419</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>41</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>396</v>
+        <v>434</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>397</v>
+        <v>435</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>398</v>
+        <v>436</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>399</v>
+        <v>437</v>
       </c>
       <c r="H7" s="21" t="n">
         <v>9720</v>
@@ -13604,36 +15788,36 @@
         <v>19586</v>
       </c>
       <c r="N7" s="16" t="s">
-        <v>393</v>
+        <v>431</v>
       </c>
       <c r="O7" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P7" s="16" t="s">
-        <v>400</v>
+        <v>438</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>401</v>
+        <v>439</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>402</v>
+        <v>440</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>37</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>403</v>
+        <v>441</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>404</v>
+        <v>442</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>405</v>
+        <v>443</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>399</v>
+        <v>437</v>
       </c>
       <c r="H8" s="21" t="n">
         <v>10361</v>
@@ -13652,36 +15836,36 @@
         <v>16526</v>
       </c>
       <c r="N8" s="16" t="s">
-        <v>393</v>
+        <v>431</v>
       </c>
       <c r="O8" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P8" s="16" t="s">
-        <v>406</v>
+        <v>444</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>407</v>
+        <v>445</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>402</v>
+        <v>440</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>408</v>
+        <v>446</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>409</v>
+        <v>447</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>410</v>
+        <v>448</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>405</v>
+        <v>443</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>399</v>
+        <v>437</v>
       </c>
       <c r="H9" s="21" t="n">
         <v>10361</v>
@@ -13700,36 +15884,36 @@
         <v>16526</v>
       </c>
       <c r="N9" s="16" t="s">
-        <v>393</v>
+        <v>431</v>
       </c>
       <c r="O9" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P9" s="16" t="s">
-        <v>411</v>
+        <v>449</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>412</v>
+        <v>450</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>402</v>
+        <v>440</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>413</v>
+        <v>451</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>414</v>
+        <v>452</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>415</v>
+        <v>453</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>405</v>
+        <v>443</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>399</v>
+        <v>437</v>
       </c>
       <c r="H10" s="21" t="n">
         <v>10361</v>
@@ -13748,36 +15932,36 @@
         <v>16526</v>
       </c>
       <c r="N10" s="16" t="s">
-        <v>393</v>
+        <v>431</v>
       </c>
       <c r="O10" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P10" s="16" t="s">
-        <v>411</v>
+        <v>449</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>416</v>
+        <v>454</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>402</v>
+        <v>440</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>417</v>
+        <v>455</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>418</v>
+        <v>456</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>419</v>
+        <v>457</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>405</v>
+        <v>443</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>399</v>
+        <v>437</v>
       </c>
       <c r="H11" s="21" t="n">
         <v>10361</v>
@@ -13796,36 +15980,36 @@
         <v>16526</v>
       </c>
       <c r="N11" s="16" t="s">
-        <v>393</v>
+        <v>431</v>
       </c>
       <c r="O11" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P11" s="16" t="s">
-        <v>411</v>
+        <v>449</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>420</v>
+        <v>458</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>421</v>
+        <v>459</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>93</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>422</v>
+        <v>460</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>423</v>
+        <v>461</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>423</v>
+        <v>461</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>399</v>
+        <v>437</v>
       </c>
       <c r="H12" s="21" t="n">
         <v>5386</v>
@@ -13845,36 +16029,36 @@
         <v>10772</v>
       </c>
       <c r="N12" s="16" t="s">
-        <v>386</v>
+        <v>424</v>
       </c>
       <c r="O12" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="P12" s="16" t="s">
-        <v>424</v>
+        <v>462</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>425</v>
+        <v>463</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>426</v>
+        <v>464</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>427</v>
+        <v>465</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>428</v>
+        <v>466</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>423</v>
+        <v>461</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>423</v>
+        <v>461</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>399</v>
+        <v>437</v>
       </c>
       <c r="H13" s="21" t="n">
         <v>3748</v>
@@ -13894,36 +16078,36 @@
         <v>7496</v>
       </c>
       <c r="N13" s="16" t="s">
-        <v>386</v>
+        <v>424</v>
       </c>
       <c r="O13" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="P13" s="16" t="s">
-        <v>429</v>
+        <v>467</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>430</v>
+        <v>468</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>421</v>
+        <v>459</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>44</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>431</v>
+        <v>469</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>423</v>
+        <v>461</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>423</v>
+        <v>461</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>399</v>
+        <v>437</v>
       </c>
       <c r="H14" s="21" t="n">
         <v>6702</v>
@@ -13943,18 +16127,18 @@
         <v>13404</v>
       </c>
       <c r="N14" s="16" t="s">
-        <v>386</v>
+        <v>424</v>
       </c>
       <c r="O14" s="21" t="n">
         <v>950</v>
       </c>
       <c r="P14" s="16" t="s">
-        <v>432</v>
+        <v>470</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>433</v>
+        <v>471</v>
       </c>
     </row>
   </sheetData>
@@ -13968,7 +16152,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -13991,17 +16175,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>434</v>
+        <v>472</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>435</v>
+        <v>473</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>436</v>
+        <v>474</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>10</v>
@@ -14019,22 +16203,22 @@
         <v>107</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>437</v>
+        <v>475</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>220</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>438</v>
+        <v>476</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>439</v>
+        <v>477</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>440</v>
+        <v>478</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>441</v>
+        <v>479</v>
       </c>
       <c r="M4" s="8" t="s">
         <v>222</v>
@@ -14042,22 +16226,22 @@
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>442</v>
+        <v>480</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>443</v>
+        <v>481</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>444</v>
+        <v>482</v>
       </c>
       <c r="D5" s="40" t="n">
         <v>4</v>
       </c>
       <c r="E5" s="27" t="s">
-        <v>445</v>
+        <v>483</v>
       </c>
       <c r="F5" s="27" t="s">
-        <v>446</v>
+        <v>484</v>
       </c>
       <c r="G5" s="11" t="n">
         <f aca="false">機票價格!L6+機票價格!L5</f>
@@ -14079,30 +16263,30 @@
         <v>15538</v>
       </c>
       <c r="L5" s="27" t="s">
-        <v>447</v>
+        <v>485</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>448</v>
+        <v>486</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>449</v>
+        <v>487</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>450</v>
+        <v>488</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>444</v>
+        <v>482</v>
       </c>
       <c r="D6" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>451</v>
+        <v>489</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>452</v>
+        <v>490</v>
       </c>
       <c r="G6" s="15" t="n">
         <f aca="false">機票價格!M5</f>
@@ -14124,30 +16308,30 @@
         <v>11576</v>
       </c>
       <c r="L6" s="20" t="s">
-        <v>447</v>
+        <v>485</v>
       </c>
       <c r="M6" s="16" t="s">
-        <v>453</v>
+        <v>491</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>454</v>
+        <v>492</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>455</v>
+        <v>493</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>456</v>
+        <v>494</v>
       </c>
       <c r="D7" s="41" t="n">
         <v>3</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>457</v>
+        <v>495</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>452</v>
+        <v>490</v>
       </c>
       <c r="G7" s="15" t="n">
         <f aca="false">機票價格!L6+機票價格!L5</f>
@@ -14169,30 +16353,30 @@
         <v>15538</v>
       </c>
       <c r="L7" s="20" t="s">
-        <v>447</v>
+        <v>485</v>
       </c>
       <c r="M7" s="16" t="s">
-        <v>458</v>
+        <v>496</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>459</v>
+        <v>497</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>460</v>
+        <v>498</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>456</v>
+        <v>494</v>
       </c>
       <c r="D8" s="41" t="n">
         <v>3</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>461</v>
+        <v>499</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>462</v>
+        <v>500</v>
       </c>
       <c r="G8" s="15" t="n">
         <f aca="false">機票價格!M7</f>
@@ -14214,30 +16398,30 @@
         <v>19586</v>
       </c>
       <c r="L8" s="20" t="s">
-        <v>447</v>
+        <v>485</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>463</v>
+        <v>501</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>464</v>
+        <v>502</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>465</v>
+        <v>503</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>444</v>
+        <v>482</v>
       </c>
       <c r="D9" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>466</v>
+        <v>504</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>467</v>
+        <v>505</v>
       </c>
       <c r="G9" s="15" t="n">
         <f aca="false">機票價格!M8</f>
@@ -14260,30 +16444,30 @@
         <v>21379.1</v>
       </c>
       <c r="L9" s="20" t="s">
-        <v>468</v>
+        <v>506</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>469</v>
+        <v>507</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>470</v>
+        <v>508</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>471</v>
+        <v>509</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>444</v>
+        <v>482</v>
       </c>
       <c r="D10" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>451</v>
+        <v>489</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>467</v>
+        <v>505</v>
       </c>
       <c r="G10" s="15" t="n">
         <f aca="false">機票價格!L5+機票價格!L8</f>
@@ -14306,30 +16490,30 @@
         <v>18303.1</v>
       </c>
       <c r="L10" s="20" t="s">
-        <v>447</v>
+        <v>485</v>
       </c>
       <c r="M10" s="16" t="s">
-        <v>472</v>
+        <v>510</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>473</v>
+        <v>511</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>474</v>
+        <v>512</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>444</v>
+        <v>482</v>
       </c>
       <c r="D11" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>475</v>
+        <v>513</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>476</v>
+        <v>514</v>
       </c>
       <c r="G11" s="15" t="n">
         <f aca="false">機票價格!M12</f>
@@ -14352,15 +16536,15 @@
         <v>17625.1</v>
       </c>
       <c r="L11" s="20" t="s">
-        <v>468</v>
+        <v>506</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>477</v>
+        <v>515</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>478</v>
+        <v>516</v>
       </c>
       <c r="C13" s="3" t="str">
         <f aca="false">INDEX(B5:B11,MATCH(MIN(K5:K11),K5:K11,0))</f>
@@ -14382,7 +16566,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -14403,12 +16587,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>479</v>
+        <v>517</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>480</v>
+        <v>518</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14419,25 +16603,25 @@
         <v>136</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>481</v>
+        <v>519</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>482</v>
+        <v>520</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>483</v>
+        <v>521</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>484</v>
+        <v>522</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>485</v>
+        <v>523</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>486</v>
+        <v>524</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>487</v>
+        <v>525</v>
       </c>
       <c r="J4" s="8" t="s">
         <v>200</v>
@@ -14448,16 +16632,16 @@
         <v>35</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>488</v>
+        <v>526</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>489</v>
+        <v>527</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>1310</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>490</v>
+        <v>528</v>
       </c>
       <c r="F5" s="31" t="n">
         <v>9000</v>
@@ -14474,7 +16658,7 @@
         <v>2284.8</v>
       </c>
       <c r="J5" s="43" t="s">
-        <v>491</v>
+        <v>529</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14482,10 +16666,10 @@
         <v>47</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>492</v>
+        <v>530</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>493</v>
+        <v>531</v>
       </c>
       <c r="D6" s="31" t="n">
         <v>2300</v>
@@ -14508,7 +16692,7 @@
         <v>4683</v>
       </c>
       <c r="J6" s="43" t="s">
-        <v>494</v>
+        <v>532</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14516,16 +16700,16 @@
         <v>49</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>495</v>
+        <v>533</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>496</v>
+        <v>534</v>
       </c>
       <c r="D7" s="31" t="n">
         <v>1200</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>497</v>
+        <v>535</v>
       </c>
       <c r="F7" s="31" t="n">
         <v>8000</v>
@@ -14542,24 +16726,24 @@
         <v>2856</v>
       </c>
       <c r="J7" s="43" t="s">
-        <v>498</v>
+        <v>536</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>499</v>
+        <v>537</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>500</v>
+        <v>538</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>501</v>
+        <v>539</v>
       </c>
       <c r="D8" s="31" t="n">
         <v>1900</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>502</v>
+        <v>540</v>
       </c>
       <c r="F8" s="44" t="n">
         <f aca="false">總覽!B7</f>
@@ -14577,7 +16761,7 @@
         <v>399</v>
       </c>
       <c r="J8" s="45" t="s">
-        <v>503</v>
+        <v>541</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14585,16 +16769,16 @@
         <v>66</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>504</v>
+        <v>542</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>505</v>
+        <v>543</v>
       </c>
       <c r="D9" s="31" t="n">
         <v>2690</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>490</v>
+        <v>528</v>
       </c>
       <c r="F9" s="31" t="n">
         <v>9000</v>
@@ -14617,10 +16801,10 @@
         <v>58</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>506</v>
+        <v>544</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>507</v>
+        <v>545</v>
       </c>
       <c r="D10" s="31" t="n">
         <v>1540</v>
@@ -14643,7 +16827,7 @@
         <v>785.4</v>
       </c>
       <c r="J10" s="43" t="s">
-        <v>508</v>
+        <v>546</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14677,18 +16861,18 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>509</v>
+        <v>547</v>
       </c>
       <c r="H12" s="49" t="n">
         <v>5000</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>510</v>
+        <v>548</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>511</v>
+        <v>549</v>
       </c>
       <c r="H13" s="50" t="n">
         <f aca="false">H12*6</f>
@@ -14701,7 +16885,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>512</v>
+        <v>550</v>
       </c>
       <c r="I14" s="18" t="n">
         <f aca="false">I11+I13</f>
@@ -14717,147 +16901,4 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
-        <v>513</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>514</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>515</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="s">
-        <v>516</v>
-      </c>
-      <c r="B2" s="20" t="s">
-        <v>517</v>
-      </c>
-      <c r="C2" s="52" t="s">
-        <v>518</v>
-      </c>
-      <c r="D2" s="16" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="16" t="s">
-        <v>520</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>517</v>
-      </c>
-      <c r="C3" s="52" t="s">
-        <v>518</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
-        <v>522</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>517</v>
-      </c>
-      <c r="C4" s="52" t="s">
-        <v>518</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="s">
-        <v>524</v>
-      </c>
-      <c r="B5" s="20" t="s">
-        <v>525</v>
-      </c>
-      <c r="C5" s="52" t="s">
-        <v>518</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="s">
-        <v>527</v>
-      </c>
-      <c r="B6" s="20" t="s">
-        <v>528</v>
-      </c>
-      <c r="C6" s="52" t="s">
-        <v>518</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
-        <v>530</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>531</v>
-      </c>
-      <c r="C7" s="52" t="s">
-        <v>518</v>
-      </c>
-      <c r="D7" s="20" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="s">
-        <v>533</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>534</v>
-      </c>
-      <c r="C8" s="52" t="s">
-        <v>518</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>535</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C2:C8" type="list">
-      <formula1>"未開始,進行中,完成"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add 2026-10-13 full rescan of bookable Sendai/Tohoku flights
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MqDR8ErShU29xSVraYyKeW
</commit_message>
<xml_diff>
--- a/japan-ginzan-plan.xlsx
+++ b/japan-ginzan-plan.xlsx
@@ -13,12 +13,13 @@
     <sheet name="新方案 10-10" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="仙台進出 10-10" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="非仙台回程 10-10" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="每日行程" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="機票價格" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="方案比較" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="行程預算" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="待辦清單" sheetId="10" state="visible" r:id="rId12"/>
-    <sheet name="資料來源" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="即時查價 10-13" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="每日行程" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="機票價格" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="方案比較" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="行程預算" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="待辦清單" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="資料來源" sheetId="12" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="608">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1241" uniqueCount="631">
   <si>
     <r>
       <rPr>
@@ -5907,6 +5908,236 @@
       </rPr>
       <t xml:space="preserve">，常因強風停駛。</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">目前還能買的直飛（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Google Flights</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">＋星宇官網，</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026/10/13 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">查詢；每人單程含稅，新台幣）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">不含東京。去程查 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/22–1/28</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、回程查 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/30–2/2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。紅底＝只剩商務艙。沒列出的日期＝當天沒有直飛或已售完。航空公司不公開剩餘座位數。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">起飛 → 抵達（當地）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">經濟艙已售完</t>
+  </si>
+  <si>
+    <t xml:space="preserve">不含托運行李</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">星宇官網：最便宜的「超值」票已售完，剩基本 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">17,480</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／全額 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">22,784</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">桃園→新潟</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:55 → 18:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">桃園→秋田</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08:30 → 12:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">桃園→花卷</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12:15 → 16:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">桃園→青森</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09:55 → 14:20</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">星宇官網確認有經濟艙（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">¥79,370</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">新潟→桃園</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:00 → 22:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">秋田→桃園</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14:10 → 17:25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">花卷→桃園</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:50 → 21:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">青森→桃園</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15:30 → 19:00</t>
   </si>
   <si>
     <r>
@@ -11951,6 +12182,343 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:J14"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="36"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="25" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>542</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>543</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>544</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>545</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>546</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>547</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>548</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>549</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>550</v>
+      </c>
+      <c r="D5" s="31" t="n">
+        <v>1310</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>551</v>
+      </c>
+      <c r="F5" s="31" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G5" s="31" t="n">
+        <v>570</v>
+      </c>
+      <c r="H5" s="42" t="n">
+        <f aca="false">D5+F5+G5</f>
+        <v>10880</v>
+      </c>
+      <c r="I5" s="32" t="n">
+        <f aca="false">H5*總覽!$B$5</f>
+        <v>2284.8</v>
+      </c>
+      <c r="J5" s="43" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>553</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>554</v>
+      </c>
+      <c r="D6" s="31" t="n">
+        <v>2300</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="F6" s="31" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G6" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="42" t="n">
+        <f aca="false">D6+F6+G6</f>
+        <v>22300</v>
+      </c>
+      <c r="I6" s="32" t="n">
+        <f aca="false">H6*總覽!$B$5</f>
+        <v>4683</v>
+      </c>
+      <c r="J6" s="43" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>556</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>557</v>
+      </c>
+      <c r="D7" s="31" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>558</v>
+      </c>
+      <c r="F7" s="31" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G7" s="31" t="n">
+        <v>4400</v>
+      </c>
+      <c r="H7" s="42" t="n">
+        <f aca="false">D7+F7+G7</f>
+        <v>13600</v>
+      </c>
+      <c r="I7" s="32" t="n">
+        <f aca="false">H7*總覽!$B$5</f>
+        <v>2856</v>
+      </c>
+      <c r="J7" s="43" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="20" t="s">
+        <v>560</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>561</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>562</v>
+      </c>
+      <c r="D8" s="31" t="n">
+        <v>1900</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>563</v>
+      </c>
+      <c r="F8" s="44" t="n">
+        <f aca="false">總覽!B7</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="42" t="n">
+        <f aca="false">D8+F8+G8</f>
+        <v>1900</v>
+      </c>
+      <c r="I8" s="32" t="n">
+        <f aca="false">H8*總覽!$B$5</f>
+        <v>399</v>
+      </c>
+      <c r="J8" s="45" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>565</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>566</v>
+      </c>
+      <c r="D9" s="31" t="n">
+        <v>2690</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>551</v>
+      </c>
+      <c r="F9" s="31" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G9" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="42" t="n">
+        <f aca="false">D9+F9+G9</f>
+        <v>11690</v>
+      </c>
+      <c r="I9" s="32" t="n">
+        <f aca="false">H9*總覽!$B$5</f>
+        <v>2454.9</v>
+      </c>
+      <c r="J9" s="43"/>
+    </row>
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>567</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>568</v>
+      </c>
+      <c r="D10" s="31" t="n">
+        <v>1540</v>
+      </c>
+      <c r="E10" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="31" t="n">
+        <v>2200</v>
+      </c>
+      <c r="H10" s="42" t="n">
+        <f aca="false">D10+F10+G10</f>
+        <v>3740</v>
+      </c>
+      <c r="I10" s="32" t="n">
+        <f aca="false">H10*總覽!$B$5</f>
+        <v>785.4</v>
+      </c>
+      <c r="J10" s="43" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="46" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="47" t="n">
+        <f aca="false">SUM(D5:D10)</f>
+        <v>10940</v>
+      </c>
+      <c r="E11" s="16"/>
+      <c r="F11" s="47" t="n">
+        <f aca="false">SUM(F5:F10)</f>
+        <v>46000</v>
+      </c>
+      <c r="G11" s="47" t="n">
+        <f aca="false">SUM(G5:G10)</f>
+        <v>7170</v>
+      </c>
+      <c r="H11" s="47" t="n">
+        <f aca="false">SUM(H5:H10)</f>
+        <v>64110</v>
+      </c>
+      <c r="I11" s="48" t="n">
+        <f aca="false">SUM(I5:I10)</f>
+        <v>13463.1</v>
+      </c>
+      <c r="J11" s="16"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="H12" s="49" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="H13" s="50" t="n">
+        <f aca="false">H12*6</f>
+        <v>30000</v>
+      </c>
+      <c r="I13" s="51" t="n">
+        <f aca="false">H13*總覽!$B$5</f>
+        <v>6300</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="I14" s="18" t="n">
+        <f aca="false">I11+I13</f>
+        <v>19763.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -11962,13 +12530,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>551</v>
+        <v>574</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>552</v>
+        <v>575</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>553</v>
+        <v>576</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>200</v>
@@ -11976,100 +12544,100 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>554</v>
+        <v>577</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>555</v>
+        <v>578</v>
       </c>
       <c r="C2" s="52" t="s">
-        <v>556</v>
+        <v>579</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>557</v>
+        <v>580</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>558</v>
+        <v>581</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>555</v>
+        <v>578</v>
       </c>
       <c r="C3" s="52" t="s">
-        <v>556</v>
+        <v>579</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>559</v>
+        <v>582</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>560</v>
+        <v>583</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>555</v>
+        <v>578</v>
       </c>
       <c r="C4" s="52" t="s">
-        <v>556</v>
+        <v>579</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>561</v>
+        <v>584</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>562</v>
+        <v>585</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>563</v>
+        <v>586</v>
       </c>
       <c r="C5" s="52" t="s">
-        <v>556</v>
+        <v>579</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>564</v>
+        <v>587</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>565</v>
+        <v>588</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>566</v>
+        <v>589</v>
       </c>
       <c r="C6" s="52" t="s">
-        <v>556</v>
+        <v>579</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>567</v>
+        <v>590</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>568</v>
+        <v>591</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>569</v>
+        <v>592</v>
       </c>
       <c r="C7" s="52" t="s">
-        <v>556</v>
+        <v>579</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>570</v>
+        <v>593</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>571</v>
+        <v>594</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>572</v>
+        <v>595</v>
       </c>
       <c r="C8" s="52" t="s">
-        <v>556</v>
+        <v>579</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>573</v>
+        <v>596</v>
       </c>
     </row>
   </sheetData>
@@ -12089,7 +12657,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -12103,138 +12671,138 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>574</v>
+        <v>597</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>575</v>
+        <v>598</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>576</v>
+        <v>599</v>
       </c>
       <c r="B2" s="53" t="s">
-        <v>577</v>
+        <v>600</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>578</v>
+        <v>601</v>
       </c>
       <c r="B3" s="53" t="s">
-        <v>579</v>
+        <v>602</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="54" t="s">
-        <v>580</v>
+        <v>603</v>
       </c>
       <c r="B4" s="53" t="s">
-        <v>581</v>
+        <v>604</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="54" t="s">
-        <v>582</v>
+        <v>605</v>
       </c>
       <c r="B5" s="53" t="s">
-        <v>583</v>
+        <v>606</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="54" t="s">
-        <v>584</v>
+        <v>607</v>
       </c>
       <c r="B6" s="53" t="s">
-        <v>585</v>
+        <v>608</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="54" t="s">
-        <v>586</v>
+        <v>609</v>
       </c>
       <c r="B7" s="53" t="s">
-        <v>587</v>
+        <v>610</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="54" t="s">
-        <v>588</v>
+        <v>611</v>
       </c>
       <c r="B8" s="53" t="s">
-        <v>589</v>
+        <v>612</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>590</v>
+        <v>613</v>
       </c>
       <c r="B9" s="53" t="s">
-        <v>591</v>
+        <v>614</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="54" t="s">
-        <v>592</v>
+        <v>615</v>
       </c>
       <c r="B10" s="53" t="s">
-        <v>593</v>
+        <v>616</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="54" t="s">
-        <v>594</v>
+        <v>617</v>
       </c>
       <c r="B11" s="53" t="s">
-        <v>595</v>
+        <v>618</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>596</v>
+        <v>619</v>
       </c>
       <c r="B12" s="53" t="s">
-        <v>597</v>
+        <v>620</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>598</v>
+        <v>621</v>
       </c>
       <c r="B13" s="53" t="s">
-        <v>599</v>
+        <v>622</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>600</v>
+        <v>623</v>
       </c>
       <c r="B14" s="53" t="s">
-        <v>601</v>
+        <v>624</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>602</v>
+        <v>625</v>
       </c>
       <c r="B15" s="53" t="s">
-        <v>603</v>
+        <v>626</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>604</v>
+        <v>627</v>
       </c>
       <c r="B16" s="53" t="s">
-        <v>605</v>
+        <v>628</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>606</v>
+        <v>629</v>
       </c>
       <c r="B17" s="53" t="s">
-        <v>607</v>
+        <v>630</v>
       </c>
     </row>
   </sheetData>
@@ -14946,6 +15514,842 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:G39"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="50"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="25" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>295</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="22" t="s">
+        <v>201</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="24" t="n">
+        <v>44798</v>
+      </c>
+      <c r="F5" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G5" s="23" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>22784</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" s="16"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>27591</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" s="16"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="22" t="s">
+        <v>204</v>
+      </c>
+      <c r="B8" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="24" t="n">
+        <v>44374</v>
+      </c>
+      <c r="F8" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G8" s="23" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>15599</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>25171</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G10" s="16"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <v>22784</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G11" s="16"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>15599</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G12" s="16" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>20266</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="16"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" s="21" t="n">
+        <v>17480</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="24" t="n">
+        <v>44798</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G15" s="23" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" s="21" t="n">
+        <v>22784</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G16" s="16"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17" s="21" t="n">
+        <v>14099</v>
+      </c>
+      <c r="F17" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G17" s="16" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>299</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>300</v>
+      </c>
+      <c r="E18" s="21" t="n">
+        <v>12799</v>
+      </c>
+      <c r="F18" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G18" s="16" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>301</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="E19" s="21" t="n">
+        <v>14599</v>
+      </c>
+      <c r="F19" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G19" s="16" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>301</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="E20" s="21" t="n">
+        <v>13099</v>
+      </c>
+      <c r="F20" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G20" s="16" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>304</v>
+      </c>
+      <c r="E21" s="21" t="n">
+        <v>17099</v>
+      </c>
+      <c r="F21" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G21" s="16" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>305</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="E22" s="21" t="n">
+        <v>25171</v>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G22" s="16"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>305</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="E23" s="21" t="n">
+        <v>25171</v>
+      </c>
+      <c r="F23" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G23" s="16"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>305</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="E24" s="21" t="n">
+        <v>25171</v>
+      </c>
+      <c r="F24" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G24" s="16"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>305</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="E25" s="21" t="n">
+        <v>20266</v>
+      </c>
+      <c r="F25" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G25" s="16"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>305</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="E26" s="21" t="n">
+        <v>25171</v>
+      </c>
+      <c r="F26" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G26" s="16"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B27" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D27" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E27" s="24" t="n">
+        <v>33270</v>
+      </c>
+      <c r="F27" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G27" s="23" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B28" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="D28" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="E28" s="24" t="n">
+        <v>34552</v>
+      </c>
+      <c r="F28" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G28" s="23" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C29" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="D29" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="E29" s="24" t="n">
+        <v>34552</v>
+      </c>
+      <c r="F29" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G29" s="23" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="B30" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D30" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E30" s="24" t="n">
+        <v>33270</v>
+      </c>
+      <c r="F30" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="G30" s="23" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="E31" s="21" t="n">
+        <v>16144</v>
+      </c>
+      <c r="F31" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G31" s="16" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="E32" s="21" t="n">
+        <v>16585</v>
+      </c>
+      <c r="F32" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G32" s="16" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B33" s="16" t="s">
+        <v>308</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D33" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="E33" s="21" t="n">
+        <v>10970</v>
+      </c>
+      <c r="F33" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G33" s="16" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" s="16" t="s">
+        <v>310</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D34" s="20" t="s">
+        <v>311</v>
+      </c>
+      <c r="E34" s="21" t="n">
+        <v>11228</v>
+      </c>
+      <c r="F34" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G34" s="16" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B35" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D35" s="20" t="s">
+        <v>313</v>
+      </c>
+      <c r="E35" s="21" t="n">
+        <v>12082</v>
+      </c>
+      <c r="F35" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G35" s="16" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B36" s="16" t="s">
+        <v>314</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D36" s="20" t="s">
+        <v>315</v>
+      </c>
+      <c r="E36" s="21" t="n">
+        <v>20631</v>
+      </c>
+      <c r="F36" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G36" s="16"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37" s="16" t="s">
+        <v>314</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D37" s="20" t="s">
+        <v>315</v>
+      </c>
+      <c r="E37" s="21" t="n">
+        <v>15099</v>
+      </c>
+      <c r="F37" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G37" s="16"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B38" s="16" t="s">
+        <v>314</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D38" s="20" t="s">
+        <v>315</v>
+      </c>
+      <c r="E38" s="21" t="n">
+        <v>15099</v>
+      </c>
+      <c r="F38" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G38" s="16"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="B39" s="16" t="s">
+        <v>314</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D39" s="20" t="s">
+        <v>315</v>
+      </c>
+      <c r="E39" s="21" t="n">
+        <v>15099</v>
+      </c>
+      <c r="F39" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G39" s="16"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:E48"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -14958,12 +16362,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>293</v>
+        <v>316</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>294</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14985,34 +16389,34 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="34" t="s">
-        <v>295</v>
+        <v>318</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>296</v>
+        <v>319</v>
       </c>
       <c r="C5" s="36" t="s">
-        <v>297</v>
+        <v>320</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>298</v>
+        <v>321</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>299</v>
+        <v>322</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16"/>
       <c r="B6" s="20" t="s">
-        <v>300</v>
+        <v>323</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>301</v>
+        <v>324</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>302</v>
+        <v>325</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>303</v>
+        <v>326</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15021,67 +16425,67 @@
         <v>147</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>304</v>
+        <v>327</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16" t="s">
-        <v>305</v>
+        <v>328</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16"/>
       <c r="B8" s="20" t="s">
-        <v>306</v>
+        <v>329</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>307</v>
+        <v>330</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>308</v>
+        <v>331</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>309</v>
+        <v>332</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16"/>
       <c r="B9" s="20" t="s">
-        <v>310</v>
+        <v>333</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>311</v>
+        <v>334</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16" t="s">
-        <v>312</v>
+        <v>335</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16"/>
       <c r="B10" s="20" t="s">
-        <v>313</v>
+        <v>336</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>314</v>
+        <v>337</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>315</v>
+        <v>338</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>316</v>
+        <v>339</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16"/>
       <c r="B11" s="20" t="s">
-        <v>317</v>
+        <v>340</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>318</v>
+        <v>341</v>
       </c>
       <c r="D11" s="16"/>
       <c r="E11" s="16" t="s">
-        <v>319</v>
+        <v>342</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15092,35 +16496,35 @@
         <v>155</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>320</v>
+        <v>343</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>321</v>
+        <v>344</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>322</v>
+        <v>345</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16"/>
       <c r="B13" s="20" t="s">
-        <v>323</v>
+        <v>346</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>324</v>
+        <v>347</v>
       </c>
       <c r="D13" s="16"/>
       <c r="E13" s="16" t="s">
-        <v>325</v>
+        <v>348</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16"/>
       <c r="B14" s="20" t="s">
-        <v>326</v>
+        <v>349</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>327</v>
+        <v>350</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
@@ -15128,20 +16532,20 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16"/>
       <c r="B15" s="20" t="s">
-        <v>328</v>
+        <v>351</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>329</v>
+        <v>352</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>330</v>
+        <v>353</v>
       </c>
       <c r="E15" s="16"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16"/>
       <c r="B16" s="20" t="s">
-        <v>310</v>
+        <v>333</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>151</v>
@@ -15150,7 +16554,7 @@
         <v>152</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>331</v>
+        <v>354</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15159,26 +16563,26 @@
         <v>180</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>332</v>
+        <v>355</v>
       </c>
       <c r="D17" s="16"/>
       <c r="E17" s="16" t="s">
-        <v>333</v>
+        <v>356</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16"/>
       <c r="B18" s="20" t="s">
-        <v>317</v>
+        <v>340</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>334</v>
+        <v>357</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>335</v>
+        <v>358</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>336</v>
+        <v>359</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15189,22 +16593,22 @@
         <v>155</v>
       </c>
       <c r="C19" s="36" t="s">
-        <v>337</v>
+        <v>360</v>
       </c>
       <c r="D19" s="36" t="s">
-        <v>338</v>
+        <v>361</v>
       </c>
       <c r="E19" s="36" t="s">
-        <v>339</v>
+        <v>362</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16"/>
       <c r="B20" s="20" t="s">
-        <v>326</v>
+        <v>349</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>340</v>
+        <v>363</v>
       </c>
       <c r="D20" s="16"/>
       <c r="E20" s="16"/>
@@ -15212,10 +16616,10 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16"/>
       <c r="B21" s="20" t="s">
-        <v>341</v>
+        <v>364</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>342</v>
+        <v>365</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>152</v>
@@ -15225,25 +16629,25 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16"/>
       <c r="B22" s="20" t="s">
-        <v>313</v>
+        <v>336</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>343</v>
+        <v>366</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>344</v>
+        <v>367</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>345</v>
+        <v>368</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="16"/>
       <c r="B23" s="20" t="s">
-        <v>317</v>
+        <v>340</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>346</v>
+        <v>369</v>
       </c>
       <c r="D23" s="16"/>
       <c r="E23" s="16" t="s">
@@ -15255,77 +16659,77 @@
         <v>165</v>
       </c>
       <c r="B24" s="35" t="s">
-        <v>347</v>
+        <v>370</v>
       </c>
       <c r="C24" s="36" t="s">
-        <v>348</v>
+        <v>371</v>
       </c>
       <c r="D24" s="36"/>
       <c r="E24" s="36" t="s">
-        <v>349</v>
+        <v>372</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16"/>
       <c r="B25" s="20" t="s">
-        <v>350</v>
+        <v>373</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>167</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>351</v>
+        <v>374</v>
       </c>
       <c r="E25" s="16"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16"/>
       <c r="B26" s="20" t="s">
-        <v>341</v>
+        <v>364</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>352</v>
+        <v>375</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>353</v>
+        <v>376</v>
       </c>
       <c r="E26" s="16" t="s">
-        <v>354</v>
+        <v>377</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12"/>
       <c r="B27" s="27" t="s">
-        <v>313</v>
+        <v>336</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>355</v>
+        <v>378</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="12" t="s">
-        <v>356</v>
+        <v>379</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16"/>
       <c r="B28" s="20" t="s">
-        <v>357</v>
+        <v>380</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>358</v>
+        <v>381</v>
       </c>
       <c r="D28" s="16"/>
       <c r="E28" s="16" t="s">
-        <v>359</v>
+        <v>382</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16"/>
       <c r="B29" s="20" t="s">
-        <v>360</v>
+        <v>383</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>361</v>
+        <v>384</v>
       </c>
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
@@ -15333,14 +16737,14 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16"/>
       <c r="B30" s="20" t="s">
-        <v>362</v>
+        <v>385</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>363</v>
+        <v>386</v>
       </c>
       <c r="D30" s="16"/>
       <c r="E30" s="16" t="s">
-        <v>364</v>
+        <v>387</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15355,16 +16759,16 @@
       </c>
       <c r="D31" s="36"/>
       <c r="E31" s="36" t="s">
-        <v>365</v>
+        <v>388</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16"/>
       <c r="B32" s="20" t="s">
-        <v>366</v>
+        <v>389</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>367</v>
+        <v>390</v>
       </c>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
@@ -15372,38 +16776,38 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16"/>
       <c r="B33" s="20" t="s">
-        <v>368</v>
+        <v>391</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>369</v>
+        <v>392</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>370</v>
+        <v>393</v>
       </c>
       <c r="E33" s="16"/>
     </row>
     <row r="34" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="16"/>
       <c r="B34" s="20" t="s">
-        <v>371</v>
+        <v>394</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>372</v>
+        <v>395</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>373</v>
+        <v>396</v>
       </c>
       <c r="E34" s="16" t="s">
-        <v>374</v>
+        <v>397</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16"/>
       <c r="B35" s="20" t="s">
-        <v>310</v>
+        <v>333</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>375</v>
+        <v>398</v>
       </c>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
@@ -15411,27 +16815,27 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16"/>
       <c r="B36" s="20" t="s">
-        <v>313</v>
+        <v>336</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>376</v>
+        <v>399</v>
       </c>
       <c r="D36" s="16"/>
       <c r="E36" s="16" t="s">
-        <v>377</v>
+        <v>400</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16"/>
       <c r="B37" s="20" t="s">
-        <v>360</v>
+        <v>383</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>378</v>
+        <v>401</v>
       </c>
       <c r="D37" s="16"/>
       <c r="E37" s="16" t="s">
-        <v>379</v>
+        <v>402</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15439,10 +16843,10 @@
         <v>183</v>
       </c>
       <c r="B38" s="35" t="s">
-        <v>366</v>
+        <v>389</v>
       </c>
       <c r="C38" s="36" t="s">
-        <v>380</v>
+        <v>403</v>
       </c>
       <c r="D38" s="36"/>
       <c r="E38" s="36"/>
@@ -15453,23 +16857,23 @@
         <v>155</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>381</v>
+        <v>404</v>
       </c>
       <c r="D39" s="20" t="s">
-        <v>382</v>
+        <v>405</v>
       </c>
       <c r="E39" s="16"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16"/>
       <c r="B40" s="20" t="s">
-        <v>383</v>
+        <v>406</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>384</v>
+        <v>407</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>385</v>
+        <v>408</v>
       </c>
       <c r="E40" s="16"/>
     </row>
@@ -15479,85 +16883,85 @@
         <v>166</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>386</v>
+        <v>409</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>387</v>
+        <v>410</v>
       </c>
       <c r="E41" s="16"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="16"/>
       <c r="B42" s="20" t="s">
-        <v>326</v>
+        <v>349</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>388</v>
+        <v>411</v>
       </c>
       <c r="D42" s="16"/>
       <c r="E42" s="16" t="s">
-        <v>389</v>
+        <v>412</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="16"/>
       <c r="B43" s="20" t="s">
-        <v>341</v>
+        <v>364</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>390</v>
+        <v>413</v>
       </c>
       <c r="D43" s="20" t="s">
-        <v>382</v>
+        <v>405</v>
       </c>
       <c r="E43" s="16"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="16"/>
       <c r="B44" s="20" t="s">
-        <v>391</v>
+        <v>414</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>392</v>
+        <v>415</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>308</v>
+        <v>331</v>
       </c>
       <c r="E44" s="16" t="s">
-        <v>393</v>
+        <v>416</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="16"/>
       <c r="B45" s="20" t="s">
-        <v>394</v>
+        <v>417</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>395</v>
+        <v>418</v>
       </c>
       <c r="D45" s="16"/>
       <c r="E45" s="16" t="s">
-        <v>396</v>
+        <v>419</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="16"/>
       <c r="B46" s="20" t="s">
-        <v>397</v>
+        <v>420</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>398</v>
+        <v>421</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>399</v>
+        <v>422</v>
       </c>
       <c r="E46" s="16" t="s">
-        <v>400</v>
+        <v>423</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>401</v>
+        <v>424</v>
       </c>
     </row>
   </sheetData>
@@ -15571,7 +16975,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -15595,17 +16999,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>402</v>
+        <v>425</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>403</v>
+        <v>426</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>404</v>
+        <v>427</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>29</v>
@@ -15614,66 +17018,66 @@
         <v>30</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>405</v>
+        <v>428</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>406</v>
+        <v>429</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>407</v>
+        <v>430</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>408</v>
+        <v>431</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>409</v>
+        <v>432</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>410</v>
+        <v>433</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>411</v>
+        <v>434</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>412</v>
+        <v>435</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>413</v>
+        <v>436</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>414</v>
+        <v>437</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>415</v>
+        <v>438</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>416</v>
+        <v>439</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>417</v>
+        <v>440</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>418</v>
+        <v>441</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>419</v>
+        <v>442</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>44</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>420</v>
+        <v>443</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>421</v>
+        <v>444</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>422</v>
+        <v>445</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>423</v>
+        <v>446</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>4743</v>
@@ -15692,36 +17096,36 @@
         <v>9676</v>
       </c>
       <c r="N5" s="16" t="s">
-        <v>424</v>
+        <v>447</v>
       </c>
       <c r="O5" s="21" t="n">
         <v>950</v>
       </c>
       <c r="P5" s="16" t="s">
-        <v>425</v>
+        <v>448</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>426</v>
+        <v>449</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>419</v>
+        <v>442</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>37</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>427</v>
+        <v>450</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>428</v>
+        <v>451</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>429</v>
+        <v>452</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>430</v>
+        <v>453</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>9845</v>
@@ -15740,36 +17144,36 @@
         <v>17878</v>
       </c>
       <c r="N6" s="16" t="s">
-        <v>431</v>
+        <v>454</v>
       </c>
       <c r="O6" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P6" s="16" t="s">
-        <v>432</v>
+        <v>455</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>433</v>
+        <v>456</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>419</v>
+        <v>442</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>41</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>434</v>
+        <v>457</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>435</v>
+        <v>458</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>436</v>
+        <v>459</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>437</v>
+        <v>460</v>
       </c>
       <c r="H7" s="21" t="n">
         <v>9720</v>
@@ -15788,36 +17192,36 @@
         <v>19586</v>
       </c>
       <c r="N7" s="16" t="s">
-        <v>431</v>
+        <v>454</v>
       </c>
       <c r="O7" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P7" s="16" t="s">
-        <v>438</v>
+        <v>461</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>439</v>
+        <v>462</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>440</v>
+        <v>463</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>37</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>441</v>
+        <v>464</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>442</v>
+        <v>465</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>443</v>
+        <v>466</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>437</v>
+        <v>460</v>
       </c>
       <c r="H8" s="21" t="n">
         <v>10361</v>
@@ -15836,36 +17240,36 @@
         <v>16526</v>
       </c>
       <c r="N8" s="16" t="s">
-        <v>431</v>
+        <v>454</v>
       </c>
       <c r="O8" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P8" s="16" t="s">
-        <v>444</v>
+        <v>467</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>445</v>
+        <v>468</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>440</v>
+        <v>463</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>446</v>
+        <v>469</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>447</v>
+        <v>470</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>448</v>
+        <v>471</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>443</v>
+        <v>466</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>437</v>
+        <v>460</v>
       </c>
       <c r="H9" s="21" t="n">
         <v>10361</v>
@@ -15884,36 +17288,36 @@
         <v>16526</v>
       </c>
       <c r="N9" s="16" t="s">
-        <v>431</v>
+        <v>454</v>
       </c>
       <c r="O9" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P9" s="16" t="s">
-        <v>449</v>
+        <v>472</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>450</v>
+        <v>473</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>440</v>
+        <v>463</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>451</v>
+        <v>474</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>452</v>
+        <v>475</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>453</v>
+        <v>476</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>443</v>
+        <v>466</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>437</v>
+        <v>460</v>
       </c>
       <c r="H10" s="21" t="n">
         <v>10361</v>
@@ -15932,36 +17336,36 @@
         <v>16526</v>
       </c>
       <c r="N10" s="16" t="s">
-        <v>431</v>
+        <v>454</v>
       </c>
       <c r="O10" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P10" s="16" t="s">
-        <v>449</v>
+        <v>472</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>454</v>
+        <v>477</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>440</v>
+        <v>463</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>455</v>
+        <v>478</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>456</v>
+        <v>479</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>457</v>
+        <v>480</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>443</v>
+        <v>466</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>437</v>
+        <v>460</v>
       </c>
       <c r="H11" s="21" t="n">
         <v>10361</v>
@@ -15980,36 +17384,36 @@
         <v>16526</v>
       </c>
       <c r="N11" s="16" t="s">
-        <v>431</v>
+        <v>454</v>
       </c>
       <c r="O11" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P11" s="16" t="s">
-        <v>449</v>
+        <v>472</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>458</v>
+        <v>481</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>459</v>
+        <v>482</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>93</v>
       </c>
       <c r="D12" s="20" t="s">
+        <v>483</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>484</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>484</v>
+      </c>
+      <c r="G12" s="16" t="s">
         <v>460</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>461</v>
-      </c>
-      <c r="F12" s="16" t="s">
-        <v>461</v>
-      </c>
-      <c r="G12" s="16" t="s">
-        <v>437</v>
       </c>
       <c r="H12" s="21" t="n">
         <v>5386</v>
@@ -16029,36 +17433,36 @@
         <v>10772</v>
       </c>
       <c r="N12" s="16" t="s">
-        <v>424</v>
+        <v>447</v>
       </c>
       <c r="O12" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="P12" s="16" t="s">
-        <v>462</v>
+        <v>485</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>463</v>
+        <v>486</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>464</v>
+        <v>487</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>465</v>
+        <v>488</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>466</v>
+        <v>489</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>461</v>
+        <v>484</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>461</v>
+        <v>484</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>437</v>
+        <v>460</v>
       </c>
       <c r="H13" s="21" t="n">
         <v>3748</v>
@@ -16078,36 +17482,36 @@
         <v>7496</v>
       </c>
       <c r="N13" s="16" t="s">
-        <v>424</v>
+        <v>447</v>
       </c>
       <c r="O13" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="P13" s="16" t="s">
-        <v>467</v>
+        <v>490</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>468</v>
+        <v>491</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>459</v>
+        <v>482</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>44</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>469</v>
+        <v>492</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>461</v>
+        <v>484</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>461</v>
+        <v>484</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>437</v>
+        <v>460</v>
       </c>
       <c r="H14" s="21" t="n">
         <v>6702</v>
@@ -16127,18 +17531,18 @@
         <v>13404</v>
       </c>
       <c r="N14" s="16" t="s">
-        <v>424</v>
+        <v>447</v>
       </c>
       <c r="O14" s="21" t="n">
         <v>950</v>
       </c>
       <c r="P14" s="16" t="s">
-        <v>470</v>
+        <v>493</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>471</v>
+        <v>494</v>
       </c>
     </row>
   </sheetData>
@@ -16152,7 +17556,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -16175,17 +17579,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>472</v>
+        <v>495</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>473</v>
+        <v>496</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>474</v>
+        <v>497</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>10</v>
@@ -16203,22 +17607,22 @@
         <v>107</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>475</v>
+        <v>498</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>220</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>476</v>
+        <v>499</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>477</v>
+        <v>500</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>478</v>
+        <v>501</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>479</v>
+        <v>502</v>
       </c>
       <c r="M4" s="8" t="s">
         <v>222</v>
@@ -16226,22 +17630,22 @@
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>480</v>
+        <v>503</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>481</v>
+        <v>504</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>482</v>
+        <v>505</v>
       </c>
       <c r="D5" s="40" t="n">
         <v>4</v>
       </c>
       <c r="E5" s="27" t="s">
-        <v>483</v>
+        <v>506</v>
       </c>
       <c r="F5" s="27" t="s">
-        <v>484</v>
+        <v>507</v>
       </c>
       <c r="G5" s="11" t="n">
         <f aca="false">機票價格!L6+機票價格!L5</f>
@@ -16263,30 +17667,30 @@
         <v>15538</v>
       </c>
       <c r="L5" s="27" t="s">
-        <v>485</v>
+        <v>508</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>486</v>
+        <v>509</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>487</v>
+        <v>510</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>488</v>
+        <v>511</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>482</v>
+        <v>505</v>
       </c>
       <c r="D6" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>489</v>
+        <v>512</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>490</v>
+        <v>513</v>
       </c>
       <c r="G6" s="15" t="n">
         <f aca="false">機票價格!M5</f>
@@ -16308,30 +17712,30 @@
         <v>11576</v>
       </c>
       <c r="L6" s="20" t="s">
-        <v>485</v>
+        <v>508</v>
       </c>
       <c r="M6" s="16" t="s">
-        <v>491</v>
+        <v>514</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>492</v>
+        <v>515</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>493</v>
+        <v>516</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>494</v>
+        <v>517</v>
       </c>
       <c r="D7" s="41" t="n">
         <v>3</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>495</v>
+        <v>518</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>490</v>
+        <v>513</v>
       </c>
       <c r="G7" s="15" t="n">
         <f aca="false">機票價格!L6+機票價格!L5</f>
@@ -16353,30 +17757,30 @@
         <v>15538</v>
       </c>
       <c r="L7" s="20" t="s">
-        <v>485</v>
+        <v>508</v>
       </c>
       <c r="M7" s="16" t="s">
-        <v>496</v>
+        <v>519</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>497</v>
+        <v>520</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>498</v>
+        <v>521</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>494</v>
+        <v>517</v>
       </c>
       <c r="D8" s="41" t="n">
         <v>3</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>499</v>
+        <v>522</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>500</v>
+        <v>523</v>
       </c>
       <c r="G8" s="15" t="n">
         <f aca="false">機票價格!M7</f>
@@ -16398,30 +17802,30 @@
         <v>19586</v>
       </c>
       <c r="L8" s="20" t="s">
-        <v>485</v>
+        <v>508</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>501</v>
+        <v>524</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>502</v>
+        <v>525</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>503</v>
+        <v>526</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>482</v>
+        <v>505</v>
       </c>
       <c r="D9" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>504</v>
+        <v>527</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>505</v>
+        <v>528</v>
       </c>
       <c r="G9" s="15" t="n">
         <f aca="false">機票價格!M8</f>
@@ -16444,30 +17848,30 @@
         <v>21379.1</v>
       </c>
       <c r="L9" s="20" t="s">
-        <v>506</v>
+        <v>529</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>507</v>
+        <v>530</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>508</v>
+        <v>531</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>509</v>
+        <v>532</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>482</v>
+        <v>505</v>
       </c>
       <c r="D10" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>489</v>
+        <v>512</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>505</v>
+        <v>528</v>
       </c>
       <c r="G10" s="15" t="n">
         <f aca="false">機票價格!L5+機票價格!L8</f>
@@ -16490,30 +17894,30 @@
         <v>18303.1</v>
       </c>
       <c r="L10" s="20" t="s">
-        <v>485</v>
+        <v>508</v>
       </c>
       <c r="M10" s="16" t="s">
-        <v>510</v>
+        <v>533</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>511</v>
+        <v>534</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>512</v>
+        <v>535</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>482</v>
+        <v>505</v>
       </c>
       <c r="D11" s="41" t="n">
         <v>4</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>513</v>
+        <v>536</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>514</v>
+        <v>537</v>
       </c>
       <c r="G11" s="15" t="n">
         <f aca="false">機票價格!M12</f>
@@ -16536,15 +17940,15 @@
         <v>17625.1</v>
       </c>
       <c r="L11" s="20" t="s">
-        <v>506</v>
+        <v>529</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>515</v>
+        <v>538</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>516</v>
+        <v>539</v>
       </c>
       <c r="C13" s="3" t="str">
         <f aca="false">INDEX(B5:B11,MATCH(MIN(K5:K11),K5:K11,0))</f>
@@ -16553,343 +17957,6 @@
       <c r="F13" s="18" t="n">
         <f aca="false">MIN(K5:K11)</f>
         <v>11576</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:J14"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="36"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="25" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>519</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>520</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>521</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>522</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>523</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>524</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>525</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>526</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>527</v>
-      </c>
-      <c r="D5" s="31" t="n">
-        <v>1310</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>528</v>
-      </c>
-      <c r="F5" s="31" t="n">
-        <v>9000</v>
-      </c>
-      <c r="G5" s="31" t="n">
-        <v>570</v>
-      </c>
-      <c r="H5" s="42" t="n">
-        <f aca="false">D5+F5+G5</f>
-        <v>10880</v>
-      </c>
-      <c r="I5" s="32" t="n">
-        <f aca="false">H5*總覽!$B$5</f>
-        <v>2284.8</v>
-      </c>
-      <c r="J5" s="43" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>530</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>531</v>
-      </c>
-      <c r="D6" s="31" t="n">
-        <v>2300</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>249</v>
-      </c>
-      <c r="F6" s="31" t="n">
-        <v>20000</v>
-      </c>
-      <c r="G6" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="42" t="n">
-        <f aca="false">D6+F6+G6</f>
-        <v>22300</v>
-      </c>
-      <c r="I6" s="32" t="n">
-        <f aca="false">H6*總覽!$B$5</f>
-        <v>4683</v>
-      </c>
-      <c r="J6" s="43" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>533</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>534</v>
-      </c>
-      <c r="D7" s="31" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>535</v>
-      </c>
-      <c r="F7" s="31" t="n">
-        <v>8000</v>
-      </c>
-      <c r="G7" s="31" t="n">
-        <v>4400</v>
-      </c>
-      <c r="H7" s="42" t="n">
-        <f aca="false">D7+F7+G7</f>
-        <v>13600</v>
-      </c>
-      <c r="I7" s="32" t="n">
-        <f aca="false">H7*總覽!$B$5</f>
-        <v>2856</v>
-      </c>
-      <c r="J7" s="43" t="s">
-        <v>536</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
-        <v>537</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>538</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>539</v>
-      </c>
-      <c r="D8" s="31" t="n">
-        <v>1900</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>540</v>
-      </c>
-      <c r="F8" s="44" t="n">
-        <f aca="false">總覽!B7</f>
-        <v>0</v>
-      </c>
-      <c r="G8" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="42" t="n">
-        <f aca="false">D8+F8+G8</f>
-        <v>1900</v>
-      </c>
-      <c r="I8" s="32" t="n">
-        <f aca="false">H8*總覽!$B$5</f>
-        <v>399</v>
-      </c>
-      <c r="J8" s="45" t="s">
-        <v>541</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>542</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>543</v>
-      </c>
-      <c r="D9" s="31" t="n">
-        <v>2690</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>528</v>
-      </c>
-      <c r="F9" s="31" t="n">
-        <v>9000</v>
-      </c>
-      <c r="G9" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="42" t="n">
-        <f aca="false">D9+F9+G9</f>
-        <v>11690</v>
-      </c>
-      <c r="I9" s="32" t="n">
-        <f aca="false">H9*總覽!$B$5</f>
-        <v>2454.9</v>
-      </c>
-      <c r="J9" s="43"/>
-    </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>544</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>545</v>
-      </c>
-      <c r="D10" s="31" t="n">
-        <v>1540</v>
-      </c>
-      <c r="E10" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="F10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="31" t="n">
-        <v>2200</v>
-      </c>
-      <c r="H10" s="42" t="n">
-        <f aca="false">D10+F10+G10</f>
-        <v>3740</v>
-      </c>
-      <c r="I10" s="32" t="n">
-        <f aca="false">H10*總覽!$B$5</f>
-        <v>785.4</v>
-      </c>
-      <c r="J10" s="43" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="46" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="47" t="n">
-        <f aca="false">SUM(D5:D10)</f>
-        <v>10940</v>
-      </c>
-      <c r="E11" s="16"/>
-      <c r="F11" s="47" t="n">
-        <f aca="false">SUM(F5:F10)</f>
-        <v>46000</v>
-      </c>
-      <c r="G11" s="47" t="n">
-        <f aca="false">SUM(G5:G10)</f>
-        <v>7170</v>
-      </c>
-      <c r="H11" s="47" t="n">
-        <f aca="false">SUM(H5:H10)</f>
-        <v>64110</v>
-      </c>
-      <c r="I11" s="48" t="n">
-        <f aca="false">SUM(I5:I10)</f>
-        <v>13463.1</v>
-      </c>
-      <c r="J11" s="16"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>547</v>
-      </c>
-      <c r="H12" s="49" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>549</v>
-      </c>
-      <c r="H13" s="50" t="n">
-        <f aca="false">H12*6</f>
-        <v>30000</v>
-      </c>
-      <c r="I13" s="51" t="n">
-        <f aca="false">H13*總覽!$B$5</f>
-        <v>6300</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>550</v>
-      </c>
-      <c r="I14" s="18" t="n">
-        <f aca="false">I11+I13</f>
-        <v>19763.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 2-passenger fare comparison (Tokyo vs Sendai, 2026-10-13)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MqDR8ErShU29xSVraYyKeW
</commit_message>
<xml_diff>
--- a/japan-ginzan-plan.xlsx
+++ b/japan-ginzan-plan.xlsx
@@ -14,12 +14,13 @@
     <sheet name="仙台進出 10-10" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="非仙台回程 10-10" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="即時查價 10-13" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="每日行程" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="機票價格" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="方案比較" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="行程預算" sheetId="10" state="visible" r:id="rId12"/>
-    <sheet name="待辦清單" sheetId="11" state="visible" r:id="rId13"/>
-    <sheet name="資料來源" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="兩人票價 10-13" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="每日行程" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="機票價格" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="方案比較" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="行程預算" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="待辦清單" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="資料來源" sheetId="13" state="visible" r:id="rId15"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1241" uniqueCount="631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1325" uniqueCount="676">
   <si>
     <r>
       <rPr>
@@ -6138,6 +6139,886 @@
   </si>
   <si>
     <t xml:space="preserve">15:30 → 19:00</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">兩人同行：目前還買得到 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">張的機票（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Google Flights </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">以「</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">位成人」查詢，</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026/10/13</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">；價格＝兩人合計，新台幣）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">能以 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">人報價代表查詢當下至少還有 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個座位；實際以訂票時為準。陸路＝到山形（藏王）方向的兩人交通費，日圓</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">×</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">匯率（總覽 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">B5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）。廉航行李以每人 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NT$1,000 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">估。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">去程 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/27</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（三）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">機票（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">人）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">行李加購（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">人）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">陸路（日圓，</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">人）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">合計（</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">人）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">每人</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">星宇 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">JX862</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">含行李；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">16:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">到仙台，晚上到藏王溫泉</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">長榮 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">BR</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">含行李；最早到仙台</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">酷航 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">TR</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">桃園→成田</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06:50 → 10:55</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">最便宜；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">04:50 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">前要到機場；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15:30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">左右到山形</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">台灣虎航 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">IT</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">06:10 → 10:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">要搭計程車到機場</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10:40 → 14:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">含行李；時間合理</t>
+  </si>
+  <si>
+    <t xml:space="preserve">星宇</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10:10 → 14:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">含行李；從淡水搭捷運就到</t>
+  </si>
+  <si>
+    <t xml:space="preserve">長榮</t>
+  </si>
+  <si>
+    <t xml:space="preserve">含行李；最早到、離家最近</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">陸路：仙台＝機場線 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">¥680</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">＋仙台→山形巴士 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">¥1,100</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">；成田＝成田特快約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">¥3,100</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">＋新幹線東京→山形 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">¥11,670</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">；羽田＝約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">¥630</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">＋</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">¥11,670</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF5F7285"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（每人）。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">回程 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2/1</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（一）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">長榮 直飛</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">含行李；要把 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1/30–1/31 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">行程改往北走</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">韓亞／大韓 經首爾</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12:45 → 18:10</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">仁川轉機 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">小時；從仙台回、不換機場</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">台灣虎航 直飛</t>
+  </si>
+  <si>
+    <t xml:space="preserve">仙台→高雄</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:50 → 22:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">落地高雄，當晚可能要住高雄</t>
+  </si>
+  <si>
+    <t xml:space="preserve">最便宜，但離銀山溫泉遠、落地晚</t>
+  </si>
+  <si>
+    <t xml:space="preserve">日航轉長榮 經札幌</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12:15 → 18:55</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">新千歲轉機 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">小時 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">星宇 直飛（商務艙）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">泰國獅航（參考：東京回）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">若改成東京進出才適用</t>
+  </si>
+  <si>
+    <t xml:space="preserve">酷航（參考：東京回）</t>
   </si>
   <si>
     <r>
@@ -11323,7 +12204,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="59">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -11477,6 +12358,22 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -12182,6 +13079,420 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:M13"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="44"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="25" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>542</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>543</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>544</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>545</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>546</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>547</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="27" t="s">
+        <v>548</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>549</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>550</v>
+      </c>
+      <c r="D5" s="44" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>551</v>
+      </c>
+      <c r="F5" s="27" t="s">
+        <v>552</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <f aca="false">機票價格!L6+機票價格!L5</f>
+        <v>14588</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <f aca="false">機票價格!O5</f>
+        <v>950</v>
+      </c>
+      <c r="I5" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="30" t="n">
+        <f aca="false">I5*總覽!$B$5</f>
+        <v>0</v>
+      </c>
+      <c r="K5" s="30" t="n">
+        <f aca="false">G5+H5+J5</f>
+        <v>15538</v>
+      </c>
+      <c r="L5" s="27" t="s">
+        <v>553</v>
+      </c>
+      <c r="M5" s="12" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="20" t="s">
+        <v>555</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>556</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>550</v>
+      </c>
+      <c r="D6" s="45" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>557</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>558</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <f aca="false">機票價格!M5</f>
+        <v>9676</v>
+      </c>
+      <c r="H6" s="15" t="n">
+        <f aca="false">2*機票價格!O5</f>
+        <v>1900</v>
+      </c>
+      <c r="I6" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="32" t="n">
+        <f aca="false">I6*總覽!$B$5</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="32" t="n">
+        <f aca="false">G6+H6+J6</f>
+        <v>11576</v>
+      </c>
+      <c r="L6" s="20" t="s">
+        <v>553</v>
+      </c>
+      <c r="M6" s="16" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="20" t="s">
+        <v>560</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>561</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>562</v>
+      </c>
+      <c r="D7" s="45" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>563</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>558</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <f aca="false">機票價格!L6+機票價格!L5</f>
+        <v>14588</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <f aca="false">機票價格!O5</f>
+        <v>950</v>
+      </c>
+      <c r="I7" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="32" t="n">
+        <f aca="false">I7*總覽!$B$5</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="32" t="n">
+        <f aca="false">G7+H7+J7</f>
+        <v>15538</v>
+      </c>
+      <c r="L7" s="20" t="s">
+        <v>553</v>
+      </c>
+      <c r="M7" s="16" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>566</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>562</v>
+      </c>
+      <c r="D8" s="45" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="20" t="s">
+        <v>567</v>
+      </c>
+      <c r="F8" s="20" t="s">
+        <v>568</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <f aca="false">機票價格!M7</f>
+        <v>19586</v>
+      </c>
+      <c r="H8" s="15" t="n">
+        <f aca="false">2*機票價格!O7</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="32" t="n">
+        <f aca="false">I8*總覽!$B$5</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="32" t="n">
+        <f aca="false">G8+H8+J8</f>
+        <v>19586</v>
+      </c>
+      <c r="L8" s="20" t="s">
+        <v>553</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="20" t="s">
+        <v>570</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>571</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>550</v>
+      </c>
+      <c r="D9" s="45" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>572</v>
+      </c>
+      <c r="F9" s="20" t="s">
+        <v>573</v>
+      </c>
+      <c r="G9" s="15" t="n">
+        <f aca="false">機票價格!M8</f>
+        <v>16526</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <f aca="false">2*機票價格!O8</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="31" t="n">
+        <f aca="false">2*(12580+500)-1690-680*2</f>
+        <v>23110</v>
+      </c>
+      <c r="J9" s="32" t="n">
+        <f aca="false">I9*總覽!$B$5</f>
+        <v>4853.1</v>
+      </c>
+      <c r="K9" s="32" t="n">
+        <f aca="false">G9+H9+J9</f>
+        <v>21379.1</v>
+      </c>
+      <c r="L9" s="20" t="s">
+        <v>574</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="20" t="s">
+        <v>576</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>577</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>550</v>
+      </c>
+      <c r="D10" s="45" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="20" t="s">
+        <v>557</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>573</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <f aca="false">機票價格!L5+機票價格!L8</f>
+        <v>15104</v>
+      </c>
+      <c r="H10" s="15" t="n">
+        <f aca="false">機票價格!O5</f>
+        <v>950</v>
+      </c>
+      <c r="I10" s="31" t="n">
+        <f aca="false">12580+500-1690-680</f>
+        <v>10710</v>
+      </c>
+      <c r="J10" s="32" t="n">
+        <f aca="false">I10*總覽!$B$5</f>
+        <v>2249.1</v>
+      </c>
+      <c r="K10" s="32" t="n">
+        <f aca="false">G10+H10+J10</f>
+        <v>18303.1</v>
+      </c>
+      <c r="L10" s="20" t="s">
+        <v>553</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="20" t="s">
+        <v>579</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>580</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>550</v>
+      </c>
+      <c r="D11" s="45" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>581</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>582</v>
+      </c>
+      <c r="G11" s="15" t="n">
+        <f aca="false">機票價格!M12</f>
+        <v>10772</v>
+      </c>
+      <c r="H11" s="15" t="n">
+        <f aca="false">2*機票價格!O12</f>
+        <v>2000</v>
+      </c>
+      <c r="I11" s="31" t="n">
+        <f aca="false">2*(12580+500)-1690-680*2</f>
+        <v>23110</v>
+      </c>
+      <c r="J11" s="32" t="n">
+        <f aca="false">I11*總覽!$B$5</f>
+        <v>4853.1</v>
+      </c>
+      <c r="K11" s="32" t="n">
+        <f aca="false">G11+H11+J11</f>
+        <v>17625.1</v>
+      </c>
+      <c r="L11" s="20" t="s">
+        <v>574</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>584</v>
+      </c>
+      <c r="C13" s="3" t="str">
+        <f aca="false">INDEX(B5:B11,MATCH(MIN(K5:K11),K5:K11,0))</f>
+        <v>虎航來回（最便宜）</v>
+      </c>
+      <c r="F13" s="18" t="n">
+        <f aca="false">MIN(K5:K11)</f>
+        <v>11576</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:J14"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -12198,12 +13509,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>540</v>
+        <v>585</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>541</v>
+        <v>586</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12214,25 +13525,25 @@
         <v>136</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>542</v>
+        <v>587</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>543</v>
+        <v>588</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>544</v>
+        <v>589</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>545</v>
+        <v>590</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>546</v>
+        <v>591</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>547</v>
+        <v>592</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>548</v>
+        <v>593</v>
       </c>
       <c r="J4" s="8" t="s">
         <v>200</v>
@@ -12243,16 +13554,16 @@
         <v>35</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>549</v>
+        <v>594</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>550</v>
+        <v>595</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>1310</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>551</v>
+        <v>596</v>
       </c>
       <c r="F5" s="31" t="n">
         <v>9000</v>
@@ -12260,7 +13571,7 @@
       <c r="G5" s="31" t="n">
         <v>570</v>
       </c>
-      <c r="H5" s="42" t="n">
+      <c r="H5" s="46" t="n">
         <f aca="false">D5+F5+G5</f>
         <v>10880</v>
       </c>
@@ -12268,8 +13579,8 @@
         <f aca="false">H5*總覽!$B$5</f>
         <v>2284.8</v>
       </c>
-      <c r="J5" s="43" t="s">
-        <v>552</v>
+      <c r="J5" s="47" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12277,10 +13588,10 @@
         <v>47</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>553</v>
+        <v>598</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>554</v>
+        <v>599</v>
       </c>
       <c r="D6" s="31" t="n">
         <v>2300</v>
@@ -12294,7 +13605,7 @@
       <c r="G6" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="42" t="n">
+      <c r="H6" s="46" t="n">
         <f aca="false">D6+F6+G6</f>
         <v>22300</v>
       </c>
@@ -12302,8 +13613,8 @@
         <f aca="false">H6*總覽!$B$5</f>
         <v>4683</v>
       </c>
-      <c r="J6" s="43" t="s">
-        <v>555</v>
+      <c r="J6" s="47" t="s">
+        <v>600</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12311,16 +13622,16 @@
         <v>49</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>556</v>
+        <v>601</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>557</v>
+        <v>602</v>
       </c>
       <c r="D7" s="31" t="n">
         <v>1200</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>558</v>
+        <v>603</v>
       </c>
       <c r="F7" s="31" t="n">
         <v>8000</v>
@@ -12328,7 +13639,7 @@
       <c r="G7" s="31" t="n">
         <v>4400</v>
       </c>
-      <c r="H7" s="42" t="n">
+      <c r="H7" s="46" t="n">
         <f aca="false">D7+F7+G7</f>
         <v>13600</v>
       </c>
@@ -12336,34 +13647,34 @@
         <f aca="false">H7*總覽!$B$5</f>
         <v>2856</v>
       </c>
-      <c r="J7" s="43" t="s">
-        <v>559</v>
+      <c r="J7" s="47" t="s">
+        <v>604</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>560</v>
+        <v>605</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>561</v>
+        <v>606</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>562</v>
+        <v>607</v>
       </c>
       <c r="D8" s="31" t="n">
         <v>1900</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>563</v>
-      </c>
-      <c r="F8" s="44" t="n">
+        <v>608</v>
+      </c>
+      <c r="F8" s="48" t="n">
         <f aca="false">總覽!B7</f>
         <v>0</v>
       </c>
       <c r="G8" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="42" t="n">
+      <c r="H8" s="46" t="n">
         <f aca="false">D8+F8+G8</f>
         <v>1900</v>
       </c>
@@ -12371,8 +13682,8 @@
         <f aca="false">H8*總覽!$B$5</f>
         <v>399</v>
       </c>
-      <c r="J8" s="45" t="s">
-        <v>564</v>
+      <c r="J8" s="49" t="s">
+        <v>609</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12380,16 +13691,16 @@
         <v>66</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>565</v>
+        <v>610</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>566</v>
+        <v>611</v>
       </c>
       <c r="D9" s="31" t="n">
         <v>2690</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>551</v>
+        <v>596</v>
       </c>
       <c r="F9" s="31" t="n">
         <v>9000</v>
@@ -12397,7 +13708,7 @@
       <c r="G9" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="42" t="n">
+      <c r="H9" s="46" t="n">
         <f aca="false">D9+F9+G9</f>
         <v>11690</v>
       </c>
@@ -12405,17 +13716,17 @@
         <f aca="false">H9*總覽!$B$5</f>
         <v>2454.9</v>
       </c>
-      <c r="J9" s="43"/>
+      <c r="J9" s="47"/>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>567</v>
+        <v>612</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>568</v>
+        <v>613</v>
       </c>
       <c r="D10" s="31" t="n">
         <v>1540</v>
@@ -12429,7 +13740,7 @@
       <c r="G10" s="31" t="n">
         <v>2200</v>
       </c>
-      <c r="H10" s="42" t="n">
+      <c r="H10" s="46" t="n">
         <f aca="false">D10+F10+G10</f>
         <v>3740</v>
       </c>
@@ -12437,34 +13748,34 @@
         <f aca="false">H10*總覽!$B$5</f>
         <v>785.4</v>
       </c>
-      <c r="J10" s="43" t="s">
-        <v>569</v>
+      <c r="J10" s="47" t="s">
+        <v>614</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="46" t="s">
+      <c r="A11" s="50" t="s">
         <v>25</v>
       </c>
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
-      <c r="D11" s="47" t="n">
+      <c r="D11" s="51" t="n">
         <f aca="false">SUM(D5:D10)</f>
         <v>10940</v>
       </c>
       <c r="E11" s="16"/>
-      <c r="F11" s="47" t="n">
+      <c r="F11" s="51" t="n">
         <f aca="false">SUM(F5:F10)</f>
         <v>46000</v>
       </c>
-      <c r="G11" s="47" t="n">
+      <c r="G11" s="51" t="n">
         <f aca="false">SUM(G5:G10)</f>
         <v>7170</v>
       </c>
-      <c r="H11" s="47" t="n">
+      <c r="H11" s="51" t="n">
         <f aca="false">SUM(H5:H10)</f>
         <v>64110</v>
       </c>
-      <c r="I11" s="48" t="n">
+      <c r="I11" s="52" t="n">
         <f aca="false">SUM(I5:I10)</f>
         <v>13463.1</v>
       </c>
@@ -12472,31 +13783,31 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>570</v>
-      </c>
-      <c r="H12" s="49" t="n">
+        <v>615</v>
+      </c>
+      <c r="H12" s="53" t="n">
         <v>5000</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>571</v>
+        <v>616</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>572</v>
-      </c>
-      <c r="H13" s="50" t="n">
+        <v>617</v>
+      </c>
+      <c r="H13" s="54" t="n">
         <f aca="false">H12*6</f>
         <v>30000</v>
       </c>
-      <c r="I13" s="51" t="n">
+      <c r="I13" s="55" t="n">
         <f aca="false">H13*總覽!$B$5</f>
         <v>6300</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>573</v>
+        <v>618</v>
       </c>
       <c r="I14" s="18" t="n">
         <f aca="false">I11+I13</f>
@@ -12514,7 +13825,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -12530,13 +13841,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>574</v>
+        <v>619</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>575</v>
+        <v>620</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>576</v>
+        <v>621</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>200</v>
@@ -12544,100 +13855,100 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>577</v>
+        <v>622</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>578</v>
-      </c>
-      <c r="C2" s="52" t="s">
-        <v>579</v>
+        <v>623</v>
+      </c>
+      <c r="C2" s="56" t="s">
+        <v>624</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>580</v>
+        <v>625</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>581</v>
+        <v>626</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>578</v>
-      </c>
-      <c r="C3" s="52" t="s">
-        <v>579</v>
+        <v>623</v>
+      </c>
+      <c r="C3" s="56" t="s">
+        <v>624</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>582</v>
+        <v>627</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>583</v>
+        <v>628</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>578</v>
-      </c>
-      <c r="C4" s="52" t="s">
-        <v>579</v>
+        <v>623</v>
+      </c>
+      <c r="C4" s="56" t="s">
+        <v>624</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>584</v>
+        <v>629</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>585</v>
+        <v>630</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>586</v>
-      </c>
-      <c r="C5" s="52" t="s">
-        <v>579</v>
+        <v>631</v>
+      </c>
+      <c r="C5" s="56" t="s">
+        <v>624</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>587</v>
+        <v>632</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>588</v>
+        <v>633</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>589</v>
-      </c>
-      <c r="C6" s="52" t="s">
-        <v>579</v>
+        <v>634</v>
+      </c>
+      <c r="C6" s="56" t="s">
+        <v>624</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>590</v>
+        <v>635</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>591</v>
+        <v>636</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>592</v>
-      </c>
-      <c r="C7" s="52" t="s">
-        <v>579</v>
+        <v>637</v>
+      </c>
+      <c r="C7" s="56" t="s">
+        <v>624</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>593</v>
+        <v>638</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>594</v>
+        <v>639</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>595</v>
-      </c>
-      <c r="C8" s="52" t="s">
-        <v>579</v>
+        <v>640</v>
+      </c>
+      <c r="C8" s="56" t="s">
+        <v>624</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>596</v>
+        <v>641</v>
       </c>
     </row>
   </sheetData>
@@ -12657,7 +13968,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -12671,138 +13982,138 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>597</v>
+        <v>642</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>598</v>
+        <v>643</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>599</v>
-      </c>
-      <c r="B2" s="53" t="s">
-        <v>600</v>
+        <v>644</v>
+      </c>
+      <c r="B2" s="57" t="s">
+        <v>645</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>601</v>
-      </c>
-      <c r="B3" s="53" t="s">
-        <v>602</v>
+        <v>646</v>
+      </c>
+      <c r="B3" s="57" t="s">
+        <v>647</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="54" t="s">
-        <v>603</v>
-      </c>
-      <c r="B4" s="53" t="s">
-        <v>604</v>
+      <c r="A4" s="58" t="s">
+        <v>648</v>
+      </c>
+      <c r="B4" s="57" t="s">
+        <v>649</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="54" t="s">
-        <v>605</v>
-      </c>
-      <c r="B5" s="53" t="s">
-        <v>606</v>
+      <c r="A5" s="58" t="s">
+        <v>650</v>
+      </c>
+      <c r="B5" s="57" t="s">
+        <v>651</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="54" t="s">
-        <v>607</v>
-      </c>
-      <c r="B6" s="53" t="s">
-        <v>608</v>
+      <c r="A6" s="58" t="s">
+        <v>652</v>
+      </c>
+      <c r="B6" s="57" t="s">
+        <v>653</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="54" t="s">
-        <v>609</v>
-      </c>
-      <c r="B7" s="53" t="s">
-        <v>610</v>
+      <c r="A7" s="58" t="s">
+        <v>654</v>
+      </c>
+      <c r="B7" s="57" t="s">
+        <v>655</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="54" t="s">
-        <v>611</v>
-      </c>
-      <c r="B8" s="53" t="s">
-        <v>612</v>
+      <c r="A8" s="58" t="s">
+        <v>656</v>
+      </c>
+      <c r="B8" s="57" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>613</v>
-      </c>
-      <c r="B9" s="53" t="s">
-        <v>614</v>
+        <v>658</v>
+      </c>
+      <c r="B9" s="57" t="s">
+        <v>659</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="54" t="s">
-        <v>615</v>
-      </c>
-      <c r="B10" s="53" t="s">
-        <v>616</v>
+      <c r="A10" s="58" t="s">
+        <v>660</v>
+      </c>
+      <c r="B10" s="57" t="s">
+        <v>661</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="54" t="s">
-        <v>617</v>
-      </c>
-      <c r="B11" s="53" t="s">
-        <v>618</v>
+      <c r="A11" s="58" t="s">
+        <v>662</v>
+      </c>
+      <c r="B11" s="57" t="s">
+        <v>663</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>619</v>
-      </c>
-      <c r="B12" s="53" t="s">
-        <v>620</v>
+        <v>664</v>
+      </c>
+      <c r="B12" s="57" t="s">
+        <v>665</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>621</v>
-      </c>
-      <c r="B13" s="53" t="s">
-        <v>622</v>
+        <v>666</v>
+      </c>
+      <c r="B13" s="57" t="s">
+        <v>667</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>623</v>
-      </c>
-      <c r="B14" s="53" t="s">
-        <v>624</v>
+        <v>668</v>
+      </c>
+      <c r="B14" s="57" t="s">
+        <v>669</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>625</v>
-      </c>
-      <c r="B15" s="53" t="s">
-        <v>626</v>
+        <v>670</v>
+      </c>
+      <c r="B15" s="57" t="s">
+        <v>671</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>627</v>
-      </c>
-      <c r="B16" s="53" t="s">
-        <v>628</v>
+        <v>672</v>
+      </c>
+      <c r="B16" s="57" t="s">
+        <v>673</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>629</v>
-      </c>
-      <c r="B17" s="53" t="s">
-        <v>630</v>
+        <v>674</v>
+      </c>
+      <c r="B17" s="57" t="s">
+        <v>675</v>
       </c>
     </row>
   </sheetData>
@@ -16350,6 +17661,586 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:I23"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="44"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="25" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>319</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>320</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="39" t="s">
+        <v>324</v>
+      </c>
+      <c r="B5" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="40" t="n">
+        <v>34960</v>
+      </c>
+      <c r="E5" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="41" t="n">
+        <v>3560</v>
+      </c>
+      <c r="G5" s="42" t="n">
+        <f aca="false">D5+E5+F5*總覽!$B$5</f>
+        <v>35707.6</v>
+      </c>
+      <c r="H5" s="42" t="n">
+        <f aca="false">G5/2</f>
+        <v>17853.8</v>
+      </c>
+      <c r="I5" s="36" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="36" t="s">
+        <v>326</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="35" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="40" t="n">
+        <v>40532</v>
+      </c>
+      <c r="E6" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="41" t="n">
+        <v>3560</v>
+      </c>
+      <c r="G6" s="42" t="n">
+        <f aca="false">D6+E6+F6*總覽!$B$5</f>
+        <v>41279.6</v>
+      </c>
+      <c r="H6" s="42" t="n">
+        <f aca="false">G6/2</f>
+        <v>20639.8</v>
+      </c>
+      <c r="I6" s="36" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>328</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>329</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>330</v>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>19450</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F7" s="31" t="n">
+        <v>29540</v>
+      </c>
+      <c r="G7" s="32" t="n">
+        <f aca="false">D7+E7+F7*總覽!$B$5</f>
+        <v>27653.4</v>
+      </c>
+      <c r="H7" s="32" t="n">
+        <f aca="false">G7/2</f>
+        <v>13826.7</v>
+      </c>
+      <c r="I7" s="16" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>329</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>333</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>21398</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>1900</v>
+      </c>
+      <c r="F8" s="31" t="n">
+        <v>29540</v>
+      </c>
+      <c r="G8" s="32" t="n">
+        <f aca="false">D8+E8+F8*總覽!$B$5</f>
+        <v>29501.4</v>
+      </c>
+      <c r="H8" s="32" t="n">
+        <f aca="false">G8/2</f>
+        <v>14750.7</v>
+      </c>
+      <c r="I8" s="16" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>329</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>335</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <v>30484</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="31" t="n">
+        <v>29540</v>
+      </c>
+      <c r="G9" s="32" t="n">
+        <f aca="false">D9+E9+F9*總覽!$B$5</f>
+        <v>36687.4</v>
+      </c>
+      <c r="H9" s="32" t="n">
+        <f aca="false">G9/2</f>
+        <v>18343.7</v>
+      </c>
+      <c r="I9" s="16" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="16" t="s">
+        <v>337</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>329</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>338</v>
+      </c>
+      <c r="D10" s="21" t="n">
+        <v>33960</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="31" t="n">
+        <v>29540</v>
+      </c>
+      <c r="G10" s="32" t="n">
+        <f aca="false">D10+E10+F10*總覽!$B$5</f>
+        <v>40163.4</v>
+      </c>
+      <c r="H10" s="32" t="n">
+        <f aca="false">G10/2</f>
+        <v>20081.7</v>
+      </c>
+      <c r="I10" s="16" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="21" t="n">
+        <v>34504</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="31" t="n">
+        <v>24600</v>
+      </c>
+      <c r="G11" s="32" t="n">
+        <f aca="false">D11+E11+F11*總覽!$B$5</f>
+        <v>39670</v>
+      </c>
+      <c r="H11" s="32" t="n">
+        <f aca="false">G11/2</f>
+        <v>19835</v>
+      </c>
+      <c r="I11" s="16" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="16" t="s">
+        <v>340</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" s="21" t="n">
+        <v>34630</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="31" t="n">
+        <v>24600</v>
+      </c>
+      <c r="G12" s="32" t="n">
+        <f aca="false">D12+E12+F12*總覽!$B$5</f>
+        <v>39796</v>
+      </c>
+      <c r="H12" s="32" t="n">
+        <f aca="false">G12/2</f>
+        <v>19898</v>
+      </c>
+      <c r="I12" s="16" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
+        <v>343</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>319</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>320</v>
+      </c>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="I15" s="8" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="s">
+        <v>344</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>314</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>315</v>
+      </c>
+      <c r="D16" s="21" t="n">
+        <v>30174</v>
+      </c>
+      <c r="E16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="16"/>
+      <c r="G16" s="32" t="n">
+        <f aca="false">D16+E16</f>
+        <v>30174</v>
+      </c>
+      <c r="H16" s="32" t="n">
+        <f aca="false">G16/2</f>
+        <v>15087</v>
+      </c>
+      <c r="I16" s="16" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16" t="s">
+        <v>346</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>347</v>
+      </c>
+      <c r="D17" s="21" t="n">
+        <v>35947</v>
+      </c>
+      <c r="E17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="16"/>
+      <c r="G17" s="32" t="n">
+        <f aca="false">D17+E17</f>
+        <v>35947</v>
+      </c>
+      <c r="H17" s="32" t="n">
+        <f aca="false">G17/2</f>
+        <v>17973.5</v>
+      </c>
+      <c r="I17" s="16" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="16" t="s">
+        <v>349</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>350</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>351</v>
+      </c>
+      <c r="D18" s="21" t="n">
+        <v>36317</v>
+      </c>
+      <c r="E18" s="21" t="n">
+        <v>1900</v>
+      </c>
+      <c r="F18" s="16"/>
+      <c r="G18" s="32" t="n">
+        <f aca="false">D18+E18</f>
+        <v>38217</v>
+      </c>
+      <c r="H18" s="32" t="n">
+        <f aca="false">G18/2</f>
+        <v>19108.5</v>
+      </c>
+      <c r="I18" s="16" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="16" t="s">
+        <v>349</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>308</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="D19" s="21" t="n">
+        <v>21923</v>
+      </c>
+      <c r="E19" s="21" t="n">
+        <v>1900</v>
+      </c>
+      <c r="F19" s="16"/>
+      <c r="G19" s="32" t="n">
+        <f aca="false">D19+E19</f>
+        <v>23823</v>
+      </c>
+      <c r="H19" s="32" t="n">
+        <f aca="false">G19/2</f>
+        <v>11911.5</v>
+      </c>
+      <c r="I19" s="16" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="16" t="s">
+        <v>354</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>355</v>
+      </c>
+      <c r="D20" s="21" t="n">
+        <v>53877</v>
+      </c>
+      <c r="E20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="16"/>
+      <c r="G20" s="32" t="n">
+        <f aca="false">D20+E20</f>
+        <v>53877</v>
+      </c>
+      <c r="H20" s="32" t="n">
+        <f aca="false">G20/2</f>
+        <v>26938.5</v>
+      </c>
+      <c r="I20" s="16" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="16" t="s">
+        <v>357</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="D21" s="21" t="n">
+        <v>69051</v>
+      </c>
+      <c r="E21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="16"/>
+      <c r="G21" s="32" t="n">
+        <f aca="false">D21+E21</f>
+        <v>69051</v>
+      </c>
+      <c r="H21" s="32" t="n">
+        <f aca="false">G21/2</f>
+        <v>34525.5</v>
+      </c>
+      <c r="I21" s="16" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="16" t="s">
+        <v>358</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="D22" s="21" t="n">
+        <v>20764</v>
+      </c>
+      <c r="E22" s="21" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F22" s="16"/>
+      <c r="G22" s="32" t="n">
+        <f aca="false">D22+E22</f>
+        <v>22764</v>
+      </c>
+      <c r="H22" s="32" t="n">
+        <f aca="false">G22/2</f>
+        <v>11382</v>
+      </c>
+      <c r="I22" s="16" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="16" t="s">
+        <v>360</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="D23" s="21" t="n">
+        <v>21680</v>
+      </c>
+      <c r="E23" s="21" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F23" s="16"/>
+      <c r="G23" s="32" t="n">
+        <f aca="false">D23+E23</f>
+        <v>23680</v>
+      </c>
+      <c r="H23" s="32" t="n">
+        <f aca="false">G23/2</f>
+        <v>11840</v>
+      </c>
+      <c r="I23" s="16" t="s">
+        <v>359</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:E48"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -16362,12 +18253,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>316</v>
+        <v>361</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16389,34 +18280,34 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="34" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>319</v>
+        <v>364</v>
       </c>
       <c r="C5" s="36" t="s">
-        <v>320</v>
+        <v>365</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>321</v>
+        <v>366</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>322</v>
+        <v>367</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16"/>
       <c r="B6" s="20" t="s">
-        <v>323</v>
+        <v>368</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>324</v>
+        <v>369</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>325</v>
+        <v>370</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>326</v>
+        <v>371</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16425,67 +18316,67 @@
         <v>147</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>327</v>
+        <v>372</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16" t="s">
-        <v>328</v>
+        <v>373</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16"/>
       <c r="B8" s="20" t="s">
-        <v>329</v>
+        <v>374</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>330</v>
+        <v>375</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>331</v>
+        <v>376</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>332</v>
+        <v>377</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16"/>
       <c r="B9" s="20" t="s">
-        <v>333</v>
+        <v>378</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>334</v>
+        <v>379</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16" t="s">
-        <v>335</v>
+        <v>380</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16"/>
       <c r="B10" s="20" t="s">
-        <v>336</v>
+        <v>381</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>337</v>
+        <v>382</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>338</v>
+        <v>383</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>339</v>
+        <v>384</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16"/>
       <c r="B11" s="20" t="s">
-        <v>340</v>
+        <v>385</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>341</v>
+        <v>386</v>
       </c>
       <c r="D11" s="16"/>
       <c r="E11" s="16" t="s">
-        <v>342</v>
+        <v>387</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16496,35 +18387,35 @@
         <v>155</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>343</v>
+        <v>388</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>344</v>
+        <v>389</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>345</v>
+        <v>390</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16"/>
       <c r="B13" s="20" t="s">
-        <v>346</v>
+        <v>391</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>347</v>
+        <v>392</v>
       </c>
       <c r="D13" s="16"/>
       <c r="E13" s="16" t="s">
-        <v>348</v>
+        <v>393</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16"/>
       <c r="B14" s="20" t="s">
-        <v>349</v>
+        <v>394</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>350</v>
+        <v>395</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
@@ -16532,20 +18423,20 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16"/>
       <c r="B15" s="20" t="s">
-        <v>351</v>
+        <v>396</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>352</v>
+        <v>397</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>353</v>
+        <v>398</v>
       </c>
       <c r="E15" s="16"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16"/>
       <c r="B16" s="20" t="s">
-        <v>333</v>
+        <v>378</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>151</v>
@@ -16554,7 +18445,7 @@
         <v>152</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>354</v>
+        <v>399</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16563,26 +18454,26 @@
         <v>180</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>355</v>
+        <v>400</v>
       </c>
       <c r="D17" s="16"/>
       <c r="E17" s="16" t="s">
-        <v>356</v>
+        <v>401</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16"/>
       <c r="B18" s="20" t="s">
-        <v>340</v>
+        <v>385</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>357</v>
+        <v>402</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>358</v>
+        <v>403</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>359</v>
+        <v>404</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16593,22 +18484,22 @@
         <v>155</v>
       </c>
       <c r="C19" s="36" t="s">
-        <v>360</v>
+        <v>405</v>
       </c>
       <c r="D19" s="36" t="s">
-        <v>361</v>
+        <v>406</v>
       </c>
       <c r="E19" s="36" t="s">
-        <v>362</v>
+        <v>407</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16"/>
       <c r="B20" s="20" t="s">
-        <v>349</v>
+        <v>394</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>363</v>
+        <v>408</v>
       </c>
       <c r="D20" s="16"/>
       <c r="E20" s="16"/>
@@ -16616,10 +18507,10 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16"/>
       <c r="B21" s="20" t="s">
-        <v>364</v>
+        <v>409</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>365</v>
+        <v>410</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>152</v>
@@ -16629,25 +18520,25 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16"/>
       <c r="B22" s="20" t="s">
-        <v>336</v>
+        <v>381</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>366</v>
+        <v>411</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>367</v>
+        <v>412</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>368</v>
+        <v>413</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="16"/>
       <c r="B23" s="20" t="s">
-        <v>340</v>
+        <v>385</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>369</v>
+        <v>414</v>
       </c>
       <c r="D23" s="16"/>
       <c r="E23" s="16" t="s">
@@ -16659,77 +18550,77 @@
         <v>165</v>
       </c>
       <c r="B24" s="35" t="s">
-        <v>370</v>
+        <v>415</v>
       </c>
       <c r="C24" s="36" t="s">
-        <v>371</v>
+        <v>416</v>
       </c>
       <c r="D24" s="36"/>
       <c r="E24" s="36" t="s">
-        <v>372</v>
+        <v>417</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16"/>
       <c r="B25" s="20" t="s">
-        <v>373</v>
+        <v>418</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>167</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>374</v>
+        <v>419</v>
       </c>
       <c r="E25" s="16"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16"/>
       <c r="B26" s="20" t="s">
-        <v>364</v>
+        <v>409</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>375</v>
+        <v>420</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>376</v>
+        <v>421</v>
       </c>
       <c r="E26" s="16" t="s">
-        <v>377</v>
+        <v>422</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12"/>
       <c r="B27" s="27" t="s">
-        <v>336</v>
+        <v>381</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>378</v>
+        <v>423</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="12" t="s">
-        <v>379</v>
+        <v>424</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16"/>
       <c r="B28" s="20" t="s">
-        <v>380</v>
+        <v>425</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>381</v>
+        <v>426</v>
       </c>
       <c r="D28" s="16"/>
       <c r="E28" s="16" t="s">
-        <v>382</v>
+        <v>427</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16"/>
       <c r="B29" s="20" t="s">
-        <v>383</v>
+        <v>428</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>384</v>
+        <v>429</v>
       </c>
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
@@ -16737,14 +18628,14 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16"/>
       <c r="B30" s="20" t="s">
-        <v>385</v>
+        <v>430</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>386</v>
+        <v>431</v>
       </c>
       <c r="D30" s="16"/>
       <c r="E30" s="16" t="s">
-        <v>387</v>
+        <v>432</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16759,16 +18650,16 @@
       </c>
       <c r="D31" s="36"/>
       <c r="E31" s="36" t="s">
-        <v>388</v>
+        <v>433</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16"/>
       <c r="B32" s="20" t="s">
-        <v>389</v>
+        <v>434</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>390</v>
+        <v>435</v>
       </c>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
@@ -16776,38 +18667,38 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16"/>
       <c r="B33" s="20" t="s">
-        <v>391</v>
+        <v>436</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>392</v>
+        <v>437</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>393</v>
+        <v>438</v>
       </c>
       <c r="E33" s="16"/>
     </row>
     <row r="34" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="16"/>
       <c r="B34" s="20" t="s">
-        <v>394</v>
+        <v>439</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>395</v>
+        <v>440</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>396</v>
+        <v>441</v>
       </c>
       <c r="E34" s="16" t="s">
-        <v>397</v>
+        <v>442</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16"/>
       <c r="B35" s="20" t="s">
-        <v>333</v>
+        <v>378</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>398</v>
+        <v>443</v>
       </c>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
@@ -16815,27 +18706,27 @@
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16"/>
       <c r="B36" s="20" t="s">
-        <v>336</v>
+        <v>381</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>399</v>
+        <v>444</v>
       </c>
       <c r="D36" s="16"/>
       <c r="E36" s="16" t="s">
-        <v>400</v>
+        <v>445</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16"/>
       <c r="B37" s="20" t="s">
-        <v>383</v>
+        <v>428</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>401</v>
+        <v>446</v>
       </c>
       <c r="D37" s="16"/>
       <c r="E37" s="16" t="s">
-        <v>402</v>
+        <v>447</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16843,10 +18734,10 @@
         <v>183</v>
       </c>
       <c r="B38" s="35" t="s">
-        <v>389</v>
+        <v>434</v>
       </c>
       <c r="C38" s="36" t="s">
-        <v>403</v>
+        <v>448</v>
       </c>
       <c r="D38" s="36"/>
       <c r="E38" s="36"/>
@@ -16857,23 +18748,23 @@
         <v>155</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>404</v>
+        <v>449</v>
       </c>
       <c r="D39" s="20" t="s">
-        <v>405</v>
+        <v>450</v>
       </c>
       <c r="E39" s="16"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16"/>
       <c r="B40" s="20" t="s">
-        <v>406</v>
+        <v>451</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>407</v>
+        <v>452</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>408</v>
+        <v>453</v>
       </c>
       <c r="E40" s="16"/>
     </row>
@@ -16883,85 +18774,85 @@
         <v>166</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>409</v>
+        <v>454</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>410</v>
+        <v>455</v>
       </c>
       <c r="E41" s="16"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="16"/>
       <c r="B42" s="20" t="s">
-        <v>349</v>
+        <v>394</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>411</v>
+        <v>456</v>
       </c>
       <c r="D42" s="16"/>
       <c r="E42" s="16" t="s">
-        <v>412</v>
+        <v>457</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="16"/>
       <c r="B43" s="20" t="s">
-        <v>364</v>
+        <v>409</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>413</v>
+        <v>458</v>
       </c>
       <c r="D43" s="20" t="s">
-        <v>405</v>
+        <v>450</v>
       </c>
       <c r="E43" s="16"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="16"/>
       <c r="B44" s="20" t="s">
-        <v>414</v>
+        <v>459</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>415</v>
+        <v>460</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>331</v>
+        <v>376</v>
       </c>
       <c r="E44" s="16" t="s">
-        <v>416</v>
+        <v>461</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="16"/>
       <c r="B45" s="20" t="s">
-        <v>417</v>
+        <v>462</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>418</v>
+        <v>463</v>
       </c>
       <c r="D45" s="16"/>
       <c r="E45" s="16" t="s">
-        <v>419</v>
+        <v>464</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="16"/>
       <c r="B46" s="20" t="s">
-        <v>420</v>
+        <v>465</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>421</v>
+        <v>466</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>422</v>
+        <v>467</v>
       </c>
       <c r="E46" s="16" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>424</v>
+        <v>469</v>
       </c>
     </row>
   </sheetData>
@@ -16975,7 +18866,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -16999,17 +18890,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>425</v>
+        <v>470</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>426</v>
+        <v>471</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>427</v>
+        <v>472</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>29</v>
@@ -17018,66 +18909,66 @@
         <v>30</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>428</v>
+        <v>473</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>429</v>
+        <v>474</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>430</v>
+        <v>475</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>431</v>
+        <v>476</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>432</v>
+        <v>477</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>433</v>
+        <v>478</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>434</v>
+        <v>479</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>435</v>
+        <v>480</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>436</v>
+        <v>481</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>437</v>
+        <v>482</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>438</v>
+        <v>483</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>439</v>
+        <v>484</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>440</v>
+        <v>485</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>441</v>
+        <v>486</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>442</v>
+        <v>487</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>44</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>443</v>
+        <v>488</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>444</v>
+        <v>489</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>445</v>
+        <v>490</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>446</v>
+        <v>491</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>4743</v>
@@ -17085,8 +18976,8 @@
       <c r="I5" s="21" t="n">
         <v>9676</v>
       </c>
-      <c r="J5" s="39"/>
-      <c r="K5" s="39"/>
+      <c r="J5" s="43"/>
+      <c r="K5" s="43"/>
       <c r="L5" s="32" t="n">
         <f aca="false">IF(J5&gt;0,J5,H5)</f>
         <v>4743</v>
@@ -17096,36 +18987,36 @@
         <v>9676</v>
       </c>
       <c r="N5" s="16" t="s">
-        <v>447</v>
+        <v>492</v>
       </c>
       <c r="O5" s="21" t="n">
         <v>950</v>
       </c>
       <c r="P5" s="16" t="s">
-        <v>448</v>
+        <v>493</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>449</v>
+        <v>494</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>442</v>
+        <v>487</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>37</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>450</v>
+        <v>495</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>451</v>
+        <v>496</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>452</v>
+        <v>497</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>453</v>
+        <v>498</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>9845</v>
@@ -17133,8 +19024,8 @@
       <c r="I6" s="21" t="n">
         <v>17878</v>
       </c>
-      <c r="J6" s="39"/>
-      <c r="K6" s="39"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="43"/>
       <c r="L6" s="32" t="n">
         <f aca="false">IF(J6&gt;0,J6,H6)</f>
         <v>9845</v>
@@ -17144,36 +19035,36 @@
         <v>17878</v>
       </c>
       <c r="N6" s="16" t="s">
-        <v>454</v>
+        <v>499</v>
       </c>
       <c r="O6" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P6" s="16" t="s">
-        <v>455</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>456</v>
+        <v>501</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>442</v>
+        <v>487</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>41</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>457</v>
+        <v>502</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>458</v>
+        <v>503</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>459</v>
+        <v>504</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>460</v>
+        <v>505</v>
       </c>
       <c r="H7" s="21" t="n">
         <v>9720</v>
@@ -17181,8 +19072,8 @@
       <c r="I7" s="21" t="n">
         <v>19586</v>
       </c>
-      <c r="J7" s="39"/>
-      <c r="K7" s="39"/>
+      <c r="J7" s="43"/>
+      <c r="K7" s="43"/>
       <c r="L7" s="32" t="n">
         <f aca="false">IF(J7&gt;0,J7,H7)</f>
         <v>9720</v>
@@ -17192,36 +19083,36 @@
         <v>19586</v>
       </c>
       <c r="N7" s="16" t="s">
-        <v>454</v>
+        <v>499</v>
       </c>
       <c r="O7" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P7" s="16" t="s">
-        <v>461</v>
+        <v>506</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>462</v>
+        <v>507</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>463</v>
+        <v>508</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>37</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>464</v>
+        <v>509</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>465</v>
+        <v>510</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>466</v>
+        <v>511</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>460</v>
+        <v>505</v>
       </c>
       <c r="H8" s="21" t="n">
         <v>10361</v>
@@ -17229,8 +19120,8 @@
       <c r="I8" s="21" t="n">
         <v>16526</v>
       </c>
-      <c r="J8" s="39"/>
-      <c r="K8" s="39"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="43"/>
       <c r="L8" s="32" t="n">
         <f aca="false">IF(J8&gt;0,J8,H8)</f>
         <v>10361</v>
@@ -17240,36 +19131,36 @@
         <v>16526</v>
       </c>
       <c r="N8" s="16" t="s">
-        <v>454</v>
+        <v>499</v>
       </c>
       <c r="O8" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P8" s="16" t="s">
-        <v>467</v>
+        <v>512</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>468</v>
+        <v>513</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>463</v>
+        <v>508</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>469</v>
+        <v>514</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>470</v>
+        <v>515</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>471</v>
+        <v>516</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>466</v>
+        <v>511</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>460</v>
+        <v>505</v>
       </c>
       <c r="H9" s="21" t="n">
         <v>10361</v>
@@ -17277,8 +19168,8 @@
       <c r="I9" s="21" t="n">
         <v>16526</v>
       </c>
-      <c r="J9" s="39"/>
-      <c r="K9" s="39"/>
+      <c r="J9" s="43"/>
+      <c r="K9" s="43"/>
       <c r="L9" s="32" t="n">
         <f aca="false">IF(J9&gt;0,J9,H9)</f>
         <v>10361</v>
@@ -17288,36 +19179,36 @@
         <v>16526</v>
       </c>
       <c r="N9" s="16" t="s">
-        <v>454</v>
+        <v>499</v>
       </c>
       <c r="O9" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P9" s="16" t="s">
-        <v>472</v>
+        <v>517</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>473</v>
+        <v>518</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>463</v>
+        <v>508</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>474</v>
+        <v>519</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>475</v>
+        <v>520</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>476</v>
+        <v>521</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>466</v>
+        <v>511</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>460</v>
+        <v>505</v>
       </c>
       <c r="H10" s="21" t="n">
         <v>10361</v>
@@ -17325,8 +19216,8 @@
       <c r="I10" s="21" t="n">
         <v>16526</v>
       </c>
-      <c r="J10" s="39"/>
-      <c r="K10" s="39"/>
+      <c r="J10" s="43"/>
+      <c r="K10" s="43"/>
       <c r="L10" s="32" t="n">
         <f aca="false">IF(J10&gt;0,J10,H10)</f>
         <v>10361</v>
@@ -17336,36 +19227,36 @@
         <v>16526</v>
       </c>
       <c r="N10" s="16" t="s">
-        <v>454</v>
+        <v>499</v>
       </c>
       <c r="O10" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P10" s="16" t="s">
-        <v>472</v>
+        <v>517</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>477</v>
+        <v>522</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>463</v>
+        <v>508</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>478</v>
+        <v>523</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>479</v>
+        <v>524</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>480</v>
+        <v>525</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>466</v>
+        <v>511</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>460</v>
+        <v>505</v>
       </c>
       <c r="H11" s="21" t="n">
         <v>10361</v>
@@ -17373,8 +19264,8 @@
       <c r="I11" s="21" t="n">
         <v>16526</v>
       </c>
-      <c r="J11" s="39"/>
-      <c r="K11" s="39"/>
+      <c r="J11" s="43"/>
+      <c r="K11" s="43"/>
       <c r="L11" s="32" t="n">
         <f aca="false">IF(J11&gt;0,J11,H11)</f>
         <v>10361</v>
@@ -17384,36 +19275,36 @@
         <v>16526</v>
       </c>
       <c r="N11" s="16" t="s">
-        <v>454</v>
+        <v>499</v>
       </c>
       <c r="O11" s="21" t="n">
         <v>0</v>
       </c>
       <c r="P11" s="16" t="s">
-        <v>472</v>
+        <v>517</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>481</v>
+        <v>526</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>482</v>
+        <v>527</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>93</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>483</v>
+        <v>528</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>484</v>
+        <v>529</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>484</v>
+        <v>529</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>460</v>
+        <v>505</v>
       </c>
       <c r="H12" s="21" t="n">
         <v>5386</v>
@@ -17422,8 +19313,8 @@
         <f aca="false">H12*2</f>
         <v>10772</v>
       </c>
-      <c r="J12" s="39"/>
-      <c r="K12" s="39"/>
+      <c r="J12" s="43"/>
+      <c r="K12" s="43"/>
       <c r="L12" s="32" t="n">
         <f aca="false">IF(J12&gt;0,J12,H12)</f>
         <v>5386</v>
@@ -17433,36 +19324,36 @@
         <v>10772</v>
       </c>
       <c r="N12" s="16" t="s">
-        <v>447</v>
+        <v>492</v>
       </c>
       <c r="O12" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="P12" s="16" t="s">
-        <v>485</v>
+        <v>530</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>486</v>
+        <v>531</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>487</v>
+        <v>532</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>488</v>
+        <v>533</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>489</v>
+        <v>534</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>484</v>
+        <v>529</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>484</v>
+        <v>529</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>460</v>
+        <v>505</v>
       </c>
       <c r="H13" s="21" t="n">
         <v>3748</v>
@@ -17471,8 +19362,8 @@
         <f aca="false">H13*2</f>
         <v>7496</v>
       </c>
-      <c r="J13" s="39"/>
-      <c r="K13" s="39"/>
+      <c r="J13" s="43"/>
+      <c r="K13" s="43"/>
       <c r="L13" s="32" t="n">
         <f aca="false">IF(J13&gt;0,J13,H13)</f>
         <v>3748</v>
@@ -17482,36 +19373,36 @@
         <v>7496</v>
       </c>
       <c r="N13" s="16" t="s">
-        <v>447</v>
+        <v>492</v>
       </c>
       <c r="O13" s="21" t="n">
         <v>1000</v>
       </c>
       <c r="P13" s="16" t="s">
-        <v>490</v>
+        <v>535</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>491</v>
+        <v>536</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>482</v>
+        <v>527</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>44</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>492</v>
+        <v>537</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>484</v>
+        <v>529</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>484</v>
+        <v>529</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>460</v>
+        <v>505</v>
       </c>
       <c r="H14" s="21" t="n">
         <v>6702</v>
@@ -17520,8 +19411,8 @@
         <f aca="false">H14*2</f>
         <v>13404</v>
       </c>
-      <c r="J14" s="39"/>
-      <c r="K14" s="39"/>
+      <c r="J14" s="43"/>
+      <c r="K14" s="43"/>
       <c r="L14" s="32" t="n">
         <f aca="false">IF(J14&gt;0,J14,H14)</f>
         <v>6702</v>
@@ -17531,432 +19422,18 @@
         <v>13404</v>
       </c>
       <c r="N14" s="16" t="s">
-        <v>447</v>
+        <v>492</v>
       </c>
       <c r="O14" s="21" t="n">
         <v>950</v>
       </c>
       <c r="P14" s="16" t="s">
-        <v>493</v>
+        <v>538</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>494</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:M13"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="44"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="25" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
-        <v>497</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>498</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>499</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>500</v>
-      </c>
-      <c r="K4" s="8" t="s">
-        <v>501</v>
-      </c>
-      <c r="L4" s="8" t="s">
-        <v>502</v>
-      </c>
-      <c r="M4" s="8" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="27" t="s">
-        <v>503</v>
-      </c>
-      <c r="B5" s="26" t="s">
-        <v>504</v>
-      </c>
-      <c r="C5" s="27" t="s">
-        <v>505</v>
-      </c>
-      <c r="D5" s="40" t="n">
-        <v>4</v>
-      </c>
-      <c r="E5" s="27" t="s">
-        <v>506</v>
-      </c>
-      <c r="F5" s="27" t="s">
-        <v>507</v>
-      </c>
-      <c r="G5" s="11" t="n">
-        <f aca="false">機票價格!L6+機票價格!L5</f>
-        <v>14588</v>
-      </c>
-      <c r="H5" s="11" t="n">
-        <f aca="false">機票價格!O5</f>
-        <v>950</v>
-      </c>
-      <c r="I5" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="30" t="n">
-        <f aca="false">I5*總覽!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="K5" s="30" t="n">
-        <f aca="false">G5+H5+J5</f>
-        <v>15538</v>
-      </c>
-      <c r="L5" s="27" t="s">
-        <v>508</v>
-      </c>
-      <c r="M5" s="12" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
-        <v>510</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>511</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>505</v>
-      </c>
-      <c r="D6" s="41" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" s="20" t="s">
-        <v>512</v>
-      </c>
-      <c r="F6" s="20" t="s">
-        <v>513</v>
-      </c>
-      <c r="G6" s="15" t="n">
-        <f aca="false">機票價格!M5</f>
-        <v>9676</v>
-      </c>
-      <c r="H6" s="15" t="n">
-        <f aca="false">2*機票價格!O5</f>
-        <v>1900</v>
-      </c>
-      <c r="I6" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="32" t="n">
-        <f aca="false">I6*總覽!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="K6" s="32" t="n">
-        <f aca="false">G6+H6+J6</f>
-        <v>11576</v>
-      </c>
-      <c r="L6" s="20" t="s">
-        <v>508</v>
-      </c>
-      <c r="M6" s="16" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
-        <v>515</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>516</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>517</v>
-      </c>
-      <c r="D7" s="41" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" s="20" t="s">
-        <v>518</v>
-      </c>
-      <c r="F7" s="20" t="s">
-        <v>513</v>
-      </c>
-      <c r="G7" s="15" t="n">
-        <f aca="false">機票價格!L6+機票價格!L5</f>
-        <v>14588</v>
-      </c>
-      <c r="H7" s="15" t="n">
-        <f aca="false">機票價格!O5</f>
-        <v>950</v>
-      </c>
-      <c r="I7" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="32" t="n">
-        <f aca="false">I7*總覽!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="K7" s="32" t="n">
-        <f aca="false">G7+H7+J7</f>
-        <v>15538</v>
-      </c>
-      <c r="L7" s="20" t="s">
-        <v>508</v>
-      </c>
-      <c r="M7" s="16" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
-        <v>520</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>521</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>517</v>
-      </c>
-      <c r="D8" s="41" t="n">
-        <v>3</v>
-      </c>
-      <c r="E8" s="20" t="s">
-        <v>522</v>
-      </c>
-      <c r="F8" s="20" t="s">
-        <v>523</v>
-      </c>
-      <c r="G8" s="15" t="n">
-        <f aca="false">機票價格!M7</f>
-        <v>19586</v>
-      </c>
-      <c r="H8" s="15" t="n">
-        <f aca="false">2*機票價格!O7</f>
-        <v>0</v>
-      </c>
-      <c r="I8" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="32" t="n">
-        <f aca="false">I8*總覽!$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="K8" s="32" t="n">
-        <f aca="false">G8+H8+J8</f>
-        <v>19586</v>
-      </c>
-      <c r="L8" s="20" t="s">
-        <v>508</v>
-      </c>
-      <c r="M8" s="16" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
-        <v>525</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>526</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>505</v>
-      </c>
-      <c r="D9" s="41" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" s="20" t="s">
-        <v>527</v>
-      </c>
-      <c r="F9" s="20" t="s">
-        <v>528</v>
-      </c>
-      <c r="G9" s="15" t="n">
-        <f aca="false">機票價格!M8</f>
-        <v>16526</v>
-      </c>
-      <c r="H9" s="15" t="n">
-        <f aca="false">2*機票價格!O8</f>
-        <v>0</v>
-      </c>
-      <c r="I9" s="31" t="n">
-        <f aca="false">2*(12580+500)-1690-680*2</f>
-        <v>23110</v>
-      </c>
-      <c r="J9" s="32" t="n">
-        <f aca="false">I9*總覽!$B$5</f>
-        <v>4853.1</v>
-      </c>
-      <c r="K9" s="32" t="n">
-        <f aca="false">G9+H9+J9</f>
-        <v>21379.1</v>
-      </c>
-      <c r="L9" s="20" t="s">
-        <v>529</v>
-      </c>
-      <c r="M9" s="16" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
-        <v>531</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>532</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>505</v>
-      </c>
-      <c r="D10" s="41" t="n">
-        <v>4</v>
-      </c>
-      <c r="E10" s="20" t="s">
-        <v>512</v>
-      </c>
-      <c r="F10" s="20" t="s">
-        <v>528</v>
-      </c>
-      <c r="G10" s="15" t="n">
-        <f aca="false">機票價格!L5+機票價格!L8</f>
-        <v>15104</v>
-      </c>
-      <c r="H10" s="15" t="n">
-        <f aca="false">機票價格!O5</f>
-        <v>950</v>
-      </c>
-      <c r="I10" s="31" t="n">
-        <f aca="false">12580+500-1690-680</f>
-        <v>10710</v>
-      </c>
-      <c r="J10" s="32" t="n">
-        <f aca="false">I10*總覽!$B$5</f>
-        <v>2249.1</v>
-      </c>
-      <c r="K10" s="32" t="n">
-        <f aca="false">G10+H10+J10</f>
-        <v>18303.1</v>
-      </c>
-      <c r="L10" s="20" t="s">
-        <v>508</v>
-      </c>
-      <c r="M10" s="16" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
-        <v>534</v>
-      </c>
-      <c r="B11" s="16" t="s">
-        <v>535</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>505</v>
-      </c>
-      <c r="D11" s="41" t="n">
-        <v>4</v>
-      </c>
-      <c r="E11" s="16" t="s">
-        <v>536</v>
-      </c>
-      <c r="F11" s="16" t="s">
-        <v>537</v>
-      </c>
-      <c r="G11" s="15" t="n">
-        <f aca="false">機票價格!M12</f>
-        <v>10772</v>
-      </c>
-      <c r="H11" s="15" t="n">
-        <f aca="false">2*機票價格!O12</f>
-        <v>2000</v>
-      </c>
-      <c r="I11" s="31" t="n">
-        <f aca="false">2*(12580+500)-1690-680*2</f>
-        <v>23110</v>
-      </c>
-      <c r="J11" s="32" t="n">
-        <f aca="false">I11*總覽!$B$5</f>
-        <v>4853.1</v>
-      </c>
-      <c r="K11" s="32" t="n">
-        <f aca="false">G11+H11+J11</f>
-        <v>17625.1</v>
-      </c>
-      <c r="L11" s="20" t="s">
-        <v>529</v>
-      </c>
-      <c r="M11" s="16" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
         <v>539</v>
-      </c>
-      <c r="C13" s="3" t="str">
-        <f aca="false">INDEX(B5:B11,MATCH(MIN(K5:K11),K5:K11,0))</f>
-        <v>虎航來回（最便宜）</v>
-      </c>
-      <c r="F13" s="18" t="n">
-        <f aca="false">MIN(K5:K11)</f>
-        <v>11576</v>
       </c>
     </row>
   </sheetData>

</xml_diff>